<commit_message>
20th Nov 2021 saturday 12 PM
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D8ECDAE-7CB3-4467-BA5B-AC4631D711B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83EC55B9-11A4-41DB-AF1F-FA0DC6B79370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="69">
   <si>
     <t>Statement</t>
   </si>
@@ -156,9 +156,6 @@
     <t>Remove Nth Node From End of List</t>
   </si>
   <si>
-    <t>Add a temp node pointing to head</t>
-  </si>
-  <si>
     <t>resursively iterate till u get null</t>
   </si>
   <si>
@@ -166,13 +163,91 @@
   </si>
   <si>
     <t>remove the node at count = n+1</t>
+  </si>
+  <si>
+    <t>Merge Two Sorted Lists</t>
+  </si>
+  <si>
+    <t>Return any one of given lists, and not the new one</t>
+  </si>
+  <si>
+    <t>Recursive</t>
+  </si>
+  <si>
+    <t>similarly if l2.val &gt; l1.val …</t>
+  </si>
+  <si>
+    <t>end condition:</t>
+  </si>
+  <si>
+    <t>if l1 is null return l2</t>
+  </si>
+  <si>
+    <t>if l2 is null return l1</t>
+  </si>
+  <si>
+    <t>Iterative</t>
+  </si>
+  <si>
+    <t>add a temp node pointing to head</t>
+  </si>
+  <si>
+    <t>create preHead</t>
+  </si>
+  <si>
+    <t>iterate while l1 and l2 are null</t>
+  </si>
+  <si>
+    <t>if l1.val &gt; l2.val, l2.next is recursive result of l1 and l2.next, return l2</t>
+  </si>
+  <si>
+    <t>if l1.val &gt; l2.val, last.next = l2, l2 = l2.next</t>
+  </si>
+  <si>
+    <t>else reverse thing</t>
+  </si>
+  <si>
+    <t>last = last.next</t>
+  </si>
+  <si>
+    <t>create last pointing to preHead</t>
+  </si>
+  <si>
+    <t>After while loop, if l1 is null then last.next = l2, otherwise l1</t>
+  </si>
+  <si>
+    <t>return preHead.next</t>
+  </si>
+  <si>
+    <t>Merge k Sorted Lists</t>
+  </si>
+  <si>
+    <t>Create priorityQueue of type listNode and length n and Comparator.comparing(listNode -&gt; listNode.val)</t>
+  </si>
+  <si>
+    <t>add all heads which are not null</t>
+  </si>
+  <si>
+    <t>while queue is not empty</t>
+  </si>
+  <si>
+    <t>create dummyHead, and lastNode pointing to dummyHead</t>
+  </si>
+  <si>
+    <t>&gt; pop from queue append to lastNode, lastNode = lastNode.next (now lastNode is node that's popped)</t>
+  </si>
+  <si>
+    <t>&gt; if lastNode.next is not null add it to queue</t>
+  </si>
+  <si>
+    <t>reutrn dummyHead.next</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -217,6 +292,14 @@
       <u/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -270,7 +353,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3"/>
@@ -278,6 +361,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Calculation" xfId="2" builtinId="22"/>
@@ -336,6 +420,94 @@
         <a:xfrm>
           <a:off x="2867025" y="609600"/>
           <a:ext cx="4838700" cy="2257143"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4876800</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>190124</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{78B8743F-FCDF-4982-B850-38C307B790CF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2847975" y="3276600"/>
+          <a:ext cx="4848225" cy="3009524"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>771525</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3571525</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>133100</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{02140607-40BA-4DF5-B2F4-B3FC59B830A3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3590925" y="6896100"/>
+          <a:ext cx="2800000" cy="2000000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -925,7 +1097,7 @@
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
     <col min="2" max="2" width="73.85546875" customWidth="1"/>
     <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="4" max="4" width="92.7109375" customWidth="1"/>
     <col min="13" max="13" width="6.7109375" customWidth="1"/>
     <col min="14" max="14" width="8.5703125" customWidth="1"/>
   </cols>
@@ -952,22 +1124,22 @@
         <v>39</v>
       </c>
       <c r="D3" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -978,18 +1150,142 @@
     <row r="16" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C16" s="5"/>
     </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>45</v>
+      </c>
+    </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D18" s="2"/>
+      <c r="D18" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D19" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
+      <c r="D20" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D21" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D22" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D24" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D25" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D26" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D27" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D28" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D29" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D30" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D31" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D32" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D34" s="2"/>
+      <c r="D34" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C35" s="5"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="2"/>
+      <c r="A36" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D36" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D37" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D38" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D39" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D40" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D41" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D42" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D47" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C48" s="5"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D49" s="2"/>
@@ -1004,9 +1300,14 @@
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" xr:uid="{7DFF2091-3C94-4306-9948-C02C8450916F}"/>
     <hyperlink ref="D15" r:id="rId2" xr:uid="{EACB1A9A-0E1F-40EF-A8DA-3D41720EFE9D}"/>
+    <hyperlink ref="A17" r:id="rId3" xr:uid="{29D47218-0B99-4D27-92EB-96B8A53BF540}"/>
+    <hyperlink ref="D34" r:id="rId4" xr:uid="{E6B50439-28D8-4A43-A31B-CA26FE7F6665}"/>
+    <hyperlink ref="A36" r:id="rId5" xr:uid="{B469572D-F03A-49A5-BB95-40D77AF73B8F}"/>
+    <hyperlink ref="D47" r:id="rId6" xr:uid="{B5EB827D-B21A-4924-9D01-9B55F99EE74F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId3"/>
+  <pageSetup orientation="portrait" r:id="rId7"/>
+  <drawing r:id="rId8"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Linked list remove duplicates
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83EC55B9-11A4-41DB-AF1F-FA0DC6B79370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A48CF2F-09B2-4AE2-81CA-4B9CDA110F9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="90">
   <si>
     <t>Statement</t>
   </si>
@@ -241,6 +241,69 @@
   </si>
   <si>
     <t>reutrn dummyHead.next</t>
+  </si>
+  <si>
+    <t>Rotate List</t>
+  </si>
+  <si>
+    <t>If head or head.next is null, return null</t>
+  </si>
+  <si>
+    <t>create dummyHead</t>
+  </si>
+  <si>
+    <t>create slow and fast pointing to dummyHead</t>
+  </si>
+  <si>
+    <t>&gt; count length, so fast pointer at lastNode</t>
+  </si>
+  <si>
+    <t>len - k % len times slow will move forward</t>
+  </si>
+  <si>
+    <t>operate rotation at that point</t>
+  </si>
+  <si>
+    <t>Remove Duplicates from Sorted List</t>
+  </si>
+  <si>
+    <t>Declare and assign ListNode current to head</t>
+  </si>
+  <si>
+    <t>while current is not null</t>
+  </si>
+  <si>
+    <t>&gt; if current.next is null, break</t>
+  </si>
+  <si>
+    <t>&gt; if current.val = current.next.val, current.next = current.next.next</t>
+  </si>
+  <si>
+    <t>&gt; else current = current.next</t>
+  </si>
+  <si>
+    <t>return head</t>
+  </si>
+  <si>
+    <t>Remove Duplicates from Sorted List II</t>
+  </si>
+  <si>
+    <t>Create a ListNode preHead and slow node pointing to preHead</t>
+  </si>
+  <si>
+    <t>create fast node pointing to head</t>
+  </si>
+  <si>
+    <t>while fast is not null</t>
+  </si>
+  <si>
+    <t>&gt; while fast and fast.next are not same, move fast</t>
+  </si>
+  <si>
+    <t>&gt; if slow.next != fast, slow.next = fast.next and fast = fast.next</t>
+  </si>
+  <si>
+    <t>&gt; else move slow and fast</t>
   </si>
 </sst>
 </file>
@@ -508,6 +571,138 @@
         <a:xfrm>
           <a:off x="3590925" y="6896100"/>
           <a:ext cx="2800000" cy="2000000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>180975</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4723832</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>56910</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{69180342-896B-4276-AA66-4AC691C87E15}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3000375" y="9372600"/>
+          <a:ext cx="4542857" cy="1923810"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>790575</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3904861</xdr:colOff>
+      <xdr:row>74</xdr:row>
+      <xdr:rowOff>28271</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7EFC80A3-43EE-4640-94DE-5DFA8D43746B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3609975" y="11696700"/>
+          <a:ext cx="3114286" cy="2428571"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>77</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4914900</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>171267</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{07C4DDB7-29D4-45BF-B6D9-6A1ACCCF81AE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2838450" y="14706600"/>
+          <a:ext cx="4895850" cy="1466667"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1031,7 +1226,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10429FF1-7DBA-415E-968E-9D236B8DC32D}">
-  <dimension ref="A1:D67"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -1049,7 +1244,7 @@
       <c r="B1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D1" s="3" t="s">
@@ -1058,31 +1253,6 @@
     </row>
     <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C2" s="5"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D18" s="2"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D34" s="2"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="2"/>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D49" s="2"/>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="2"/>
-    </row>
-    <row r="67" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D67" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1091,7 +1261,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56E27646-854C-4719-A92C-78F24A8C7C41}">
-  <dimension ref="A1:D67"/>
+  <dimension ref="A1:D86"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -1288,13 +1458,136 @@
       <c r="C48" s="5"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D49" s="2"/>
+      <c r="A49" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D49" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D50" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="2"/>
-    </row>
-    <row r="67" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D67" s="2"/>
+      <c r="D51" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D52" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D53" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D54" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D59" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C60" s="5"/>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D61" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D62" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D63" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D64" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D65" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D66" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D67" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D69" s="7"/>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D75" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C76" s="5"/>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D77" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D78" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D79" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D80" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="81" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D81" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="82" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D82" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="85" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D85" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="86" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C86" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1304,10 +1597,16 @@
     <hyperlink ref="D34" r:id="rId4" xr:uid="{E6B50439-28D8-4A43-A31B-CA26FE7F6665}"/>
     <hyperlink ref="A36" r:id="rId5" xr:uid="{B469572D-F03A-49A5-BB95-40D77AF73B8F}"/>
     <hyperlink ref="D47" r:id="rId6" xr:uid="{B5EB827D-B21A-4924-9D01-9B55F99EE74F}"/>
+    <hyperlink ref="A49" r:id="rId7" xr:uid="{9991CCC5-947C-47FA-94E2-F9C4DC8AEE2F}"/>
+    <hyperlink ref="D59" r:id="rId8" xr:uid="{E43457D5-A59A-4E1A-8DBF-788129276609}"/>
+    <hyperlink ref="A61" r:id="rId9" xr:uid="{87233EE7-0EC1-4307-9FBD-D575CDBE8312}"/>
+    <hyperlink ref="D75" r:id="rId10" xr:uid="{15CFEFB2-0626-4422-8C73-8889EDAD581A}"/>
+    <hyperlink ref="A77" r:id="rId11" xr:uid="{989B3ECE-514E-404A-8626-396B08E7CC8E}"/>
+    <hyperlink ref="D85" r:id="rId12" xr:uid="{0B825229-A326-4F0A-98C7-177795F408C9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId7"/>
-  <drawing r:id="rId8"/>
+  <pageSetup orientation="portrait" r:id="rId13"/>
+  <drawing r:id="rId14"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
partition linked list - tuesday 23 Nov 2021
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A48CF2F-09B2-4AE2-81CA-4B9CDA110F9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16255BBB-D63E-4613-9BC0-64D435ECC08D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="101">
   <si>
     <t>Statement</t>
   </si>
@@ -304,6 +304,39 @@
   </si>
   <si>
     <t>&gt; else move slow and fast</t>
+  </si>
+  <si>
+    <t>Move slow and fast till there are duplicates</t>
+  </si>
+  <si>
+    <t>end of duplicates</t>
+  </si>
+  <si>
+    <t>When u reach duplicates, move fast till u reach -</t>
+  </si>
+  <si>
+    <t>Partition List</t>
+  </si>
+  <si>
+    <t>Create a preHead, and slow node pointing to it</t>
+  </si>
+  <si>
+    <t>move fast node till we find element greater than x, slow as its previous node</t>
+  </si>
+  <si>
+    <t>here we'll append all nodes smaller than x to slow node</t>
+  </si>
+  <si>
+    <t>i.e.</t>
+  </si>
+  <si>
+    <t>while fast != null &amp;&amp; fast.next != null</t>
+  </si>
+  <si>
+    <t>&gt; if(fast.next.val &lt; x) then move fast.next node to slow.next</t>
+  </si>
+  <si>
+    <t>&gt; else fast = fast.next</t>
   </si>
 </sst>
 </file>
@@ -703,6 +736,50 @@
         <a:xfrm>
           <a:off x="2838450" y="14706600"/>
           <a:ext cx="4895850" cy="1466667"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>87</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4914900</xdr:colOff>
+      <xdr:row>98</xdr:row>
+      <xdr:rowOff>161648</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{72C369ED-CB3E-414B-AA88-1A97F9A9B26F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2838450" y="16611600"/>
+          <a:ext cx="4895850" cy="2219048"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1261,7 +1338,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56E27646-854C-4719-A92C-78F24A8C7C41}">
-  <dimension ref="A1:D86"/>
+  <dimension ref="A1:D100"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -1552,16 +1629,25 @@
       <c r="A77" s="2" t="s">
         <v>83</v>
       </c>
+      <c r="C77" s="1" t="s">
+        <v>90</v>
+      </c>
       <c r="D77" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C78" s="1" t="s">
+        <v>92</v>
+      </c>
       <c r="D78" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C79" s="1" t="s">
+        <v>91</v>
+      </c>
       <c r="D79" t="s">
         <v>86</v>
       </c>
@@ -1571,23 +1657,74 @@
         <v>87</v>
       </c>
     </row>
-    <row r="81" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D81" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="82" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D82" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="85" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D85" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="86" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C86" s="5"/>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D87" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D88" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D89" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D90" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D91" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D92" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D93" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D94" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="99" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D99" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="100" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C100" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1603,10 +1740,12 @@
     <hyperlink ref="D75" r:id="rId10" xr:uid="{15CFEFB2-0626-4422-8C73-8889EDAD581A}"/>
     <hyperlink ref="A77" r:id="rId11" xr:uid="{989B3ECE-514E-404A-8626-396B08E7CC8E}"/>
     <hyperlink ref="D85" r:id="rId12" xr:uid="{0B825229-A326-4F0A-98C7-177795F408C9}"/>
+    <hyperlink ref="A87" r:id="rId13" xr:uid="{48BB70FF-A8ED-42E4-8A11-752AF2EB04DC}"/>
+    <hyperlink ref="D99" r:id="rId14" xr:uid="{C55579BE-756D-40BA-A7A4-EA1ABF78C0AC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId13"/>
-  <drawing r:id="rId14"/>
+  <pageSetup orientation="portrait" r:id="rId15"/>
+  <drawing r:id="rId16"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Arrays 28 Nov 2021
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16255BBB-D63E-4613-9BC0-64D435ECC08D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{059CE538-B057-40F9-B1C8-6103C153C8CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="template" sheetId="2" r:id="rId1"/>
-    <sheet name="Linked list" sheetId="3" r:id="rId2"/>
-    <sheet name="Rain water trap" sheetId="1" r:id="rId3"/>
+    <sheet name="Array" sheetId="4" r:id="rId2"/>
+    <sheet name="Linked list" sheetId="3" r:id="rId3"/>
+    <sheet name="Rain water trap" sheetId="1" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="105">
   <si>
     <t>Statement</t>
   </si>
@@ -337,6 +338,18 @@
   </si>
   <si>
     <t>&gt; else fast = fast.next</t>
+  </si>
+  <si>
+    <t>Find First and Last Position of Element in Sorted Array</t>
+  </si>
+  <si>
+    <t>Binary search in such a way that, window finishes to left side - gets first one</t>
+  </si>
+  <si>
+    <t xml:space="preserve">similarly one finishes right </t>
+  </si>
+  <si>
+    <t>&gt; don't return till n.logn</t>
   </si>
 </sst>
 </file>
@@ -483,6 +496,55 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
+      <xdr:colOff>657225</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3704844</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>123764</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{88A1B8D1-BDA7-4105-9268-4996383A9EE8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3905250" y="590550"/>
+          <a:ext cx="3047619" cy="485714"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>47625</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
@@ -791,7 +853,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1337,6 +1399,72 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDA924A8-9114-46BA-B39C-6743F04F80F3}">
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="48.7109375" customWidth="1"/>
+    <col min="2" max="2" width="73.85546875" customWidth="1"/>
+    <col min="3" max="3" width="32.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D7" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C8" s="5"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{1078431E-90B5-490C-89E2-631EC2FC986D}"/>
+    <hyperlink ref="D7" r:id="rId2" xr:uid="{A82BE56D-8664-44EF-9D97-3B9B32089A10}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56E27646-854C-4719-A92C-78F24A8C7C41}">
   <dimension ref="A1:D100"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1749,7 +1877,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CE8EF6C-9017-4EEF-A2CD-F2424B35AA25}">
   <dimension ref="A1:D68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
array - MedianofTwoSortedArrays 6th Dec 2021
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{059CE538-B057-40F9-B1C8-6103C153C8CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64BF1D23-F427-40CF-8C41-77791A811C9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="template" sheetId="2" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="117">
   <si>
     <t>Statement</t>
   </si>
@@ -350,6 +350,42 @@
   </si>
   <si>
     <t>&gt; don't return till n.logn</t>
+  </si>
+  <si>
+    <t>Median of Two Sorted Arrays</t>
+  </si>
+  <si>
+    <t>Initialize 2 pointers i,j for 2 arrays</t>
+  </si>
+  <si>
+    <t>&gt; move until i+j reach sum/2</t>
+  </si>
+  <si>
+    <t>&gt; while moving save if i==n increment j, or if j==m i++ th element to current</t>
+  </si>
+  <si>
+    <t>&gt; store prev element all the time</t>
+  </si>
+  <si>
+    <t>if sum is odd return current, else avg of prev and current</t>
+  </si>
+  <si>
+    <t>2nd</t>
+  </si>
+  <si>
+    <t>If we have k elements in combined array</t>
+  </si>
+  <si>
+    <t>perform binary search(left, right) in first array (smaller one) such that arr1[ele] &lt; arr2[k - ele - 1] (ele = mid)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>result = min of (arr1[left] or arr2[k - left - 1])</t>
+  </si>
+  <si>
+    <t>if k is even =&gt; result1 = max(arr1[left - 1], arr2[k-left-1]) , avg (result, result1)</t>
   </si>
 </sst>
 </file>
@@ -529,6 +565,50 @@
         <a:xfrm>
           <a:off x="3905250" y="590550"/>
           <a:ext cx="3047619" cy="485714"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>390525</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4239162</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>95339</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3CF6FDD2-8501-4CBC-B35D-C5EBC9F6AE77}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3638550" y="1743075"/>
+          <a:ext cx="3848637" cy="638264"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1400,13 +1480,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDA924A8-9114-46BA-B39C-6743F04F80F3}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.7109375" customWidth="1"/>
     <col min="2" max="2" width="73.85546875" customWidth="1"/>
     <col min="3" max="3" width="32.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="4" max="4" width="94.5703125" customWidth="1"/>
     <col min="13" max="13" width="6.7109375" customWidth="1"/>
     <col min="14" max="14" width="8.5703125" customWidth="1"/>
   </cols>
@@ -1454,13 +1534,81 @@
     <row r="8" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C8" s="5"/>
     </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D11" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D12" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D13" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D14" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D16" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="17" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D17" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="18" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D18" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="19" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C19" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D19" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="20" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D20" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="21" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D21" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C22" s="5"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" xr:uid="{1078431E-90B5-490C-89E2-631EC2FC986D}"/>
     <hyperlink ref="D7" r:id="rId2" xr:uid="{A82BE56D-8664-44EF-9D97-3B9B32089A10}"/>
+    <hyperlink ref="A9" r:id="rId3" xr:uid="{E9DDCB05-35C4-411A-9E11-5D6F3CC3AF96}"/>
+    <hyperlink ref="D21" r:id="rId4" xr:uid="{3402BAFA-50FF-4A91-9C05-9F6AEAC01303}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId3"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Spiral matrix - 9th Dec 2021
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64BF1D23-F427-40CF-8C41-77791A811C9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{270F82A2-1FB2-4978-B546-66A92EB219EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="template" sheetId="2" r:id="rId1"/>
     <sheet name="Array" sheetId="4" r:id="rId2"/>
-    <sheet name="Linked list" sheetId="3" r:id="rId3"/>
-    <sheet name="Rain water trap" sheetId="1" r:id="rId4"/>
+    <sheet name="Matrix" sheetId="5" r:id="rId3"/>
+    <sheet name="Linked list" sheetId="3" r:id="rId4"/>
+    <sheet name="Rain water trap" sheetId="1" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="122">
   <si>
     <t>Statement</t>
   </si>
@@ -386,6 +387,21 @@
   </si>
   <si>
     <t>if k is even =&gt; result1 = max(arr1[left - 1], arr2[k-left-1]) , avg (result, result1)</t>
+  </si>
+  <si>
+    <t>Spiral Matrix</t>
+  </si>
+  <si>
+    <t>initialize directions array, and a visited array</t>
+  </si>
+  <si>
+    <t>traverse m*n times</t>
+  </si>
+  <si>
+    <t>if next row is inbounds &amp;&amp; not visited increment row from direction array</t>
+  </si>
+  <si>
+    <t>else change the direction (d+1) % 4</t>
   </si>
 </sst>
 </file>
@@ -625,6 +641,55 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
+      <xdr:colOff>723900</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4096221</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>114707</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7CD7E1E4-7806-4601-9EF5-9310C9337A5A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3543300" y="628650"/>
+          <a:ext cx="3372321" cy="2915057"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>47625</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
@@ -933,7 +998,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1613,6 +1678,77 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83AD0EA2-442A-436B-AA00-D0DF9DB7227A}">
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="2" max="2" width="73.85546875" customWidth="1"/>
+    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D6" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="19" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D19" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C20" s="5"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{EE24117A-8086-489D-A2CA-CE3F018A6E74}"/>
+    <hyperlink ref="D19" r:id="rId2" xr:uid="{40B2AEAE-4A71-4E88-BD4B-30765B996FE5}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56E27646-854C-4719-A92C-78F24A8C7C41}">
   <dimension ref="A1:D100"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2025,7 +2161,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CE8EF6C-9017-4EEF-A2CD-F2424B35AA25}">
   <dimension ref="A1:D68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
dp added - 26 Jan 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -1,23 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24729"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\leetcode-solutions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{270F82A2-1FB2-4978-B546-66A92EB219EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B40ED3-A7C6-453C-A6D0-F5685DEBF5C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="template" sheetId="2" r:id="rId1"/>
-    <sheet name="Array" sheetId="4" r:id="rId2"/>
-    <sheet name="Matrix" sheetId="5" r:id="rId3"/>
-    <sheet name="Linked list" sheetId="3" r:id="rId4"/>
-    <sheet name="Rain water trap" sheetId="1" r:id="rId5"/>
+    <sheet name="dp" sheetId="6" r:id="rId2"/>
+    <sheet name="Array" sheetId="4" r:id="rId3"/>
+    <sheet name="Matrix" sheetId="5" r:id="rId4"/>
+    <sheet name="Linked list" sheetId="3" r:id="rId5"/>
+    <sheet name="Rain water trap" sheetId="1" r:id="rId6"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="126">
   <si>
     <t>Statement</t>
   </si>
@@ -402,6 +403,18 @@
   </si>
   <si>
     <t>else change the direction (d+1) % 4</t>
+  </si>
+  <si>
+    <t>1143. Longest Common Subsequence</t>
+  </si>
+  <si>
+    <t>Using dp or dfs</t>
+  </si>
+  <si>
+    <t>if chars at i and j are same call i-1 and j-1</t>
+  </si>
+  <si>
+    <t>else max between i,j-1 and j,i-1</t>
   </si>
 </sst>
 </file>
@@ -548,6 +561,55 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
+      <xdr:colOff>47626</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4886326</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>133444</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EBF1B06A-14A7-4378-B685-42F84E591CCF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2867026" y="600075"/>
+          <a:ext cx="4838700" cy="676369"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>657225</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
@@ -636,7 +698,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -685,7 +747,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -998,7 +1060,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1544,6 +1606,73 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="2" max="2" width="73.85546875" customWidth="1"/>
+    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D7" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C8" s="5"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{D7F7FCDC-490D-464B-8AC6-FB046B8CD003}"/>
+    <hyperlink ref="D7" r:id="rId2" xr:uid="{9DB89340-9260-4ACB-BC3F-99EE5C02ED06}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
+  <drawing r:id="rId4"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDA924A8-9114-46BA-B39C-6743F04F80F3}">
   <dimension ref="A1:D22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1677,7 +1806,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83AD0EA2-442A-436B-AA00-D0DF9DB7227A}">
   <dimension ref="A1:D20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1748,7 +1877,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56E27646-854C-4719-A92C-78F24A8C7C41}">
   <dimension ref="A1:D100"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2161,7 +2290,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CE8EF6C-9017-4EEF-A2CD-F2424B35AA25}">
   <dimension ref="A1:D68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
dp - 30 Jan 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B40ED3-A7C6-453C-A6D0-F5685DEBF5C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6C186E3-2519-49A6-9768-80607FE4E58D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="137">
   <si>
     <t>Statement</t>
   </si>
@@ -415,6 +415,39 @@
   </si>
   <si>
     <t>else max between i,j-1 and j,i-1</t>
+  </si>
+  <si>
+    <t>72. Edit Distance</t>
+  </si>
+  <si>
+    <t>both strings empty means - requires zero operations (so fill the edges)</t>
+  </si>
+  <si>
+    <t>Bottom up solution - dp[m+1][n+1]</t>
+  </si>
+  <si>
+    <t>while iterating - if both chars are same call next itr ([i][j] = [i-1][j-1])</t>
+  </si>
+  <si>
+    <t>else min of 1 + (addn - [i-1][j], deletn - [i][j-1], replace - [i-1][j-1])</t>
+  </si>
+  <si>
+    <t>97. Interleaving String</t>
+  </si>
+  <si>
+    <t>Using dp or dfs(i, j)</t>
+  </si>
+  <si>
+    <t>if current i+jth element in s3 equals ith element in s1 then dfs for i+1</t>
+  </si>
+  <si>
+    <t>if it equals jth element in s2 then dfs for i+2</t>
+  </si>
+  <si>
+    <t>otherwise return false</t>
+  </si>
+  <si>
+    <t>edge case : if both pointers reach ends</t>
   </si>
 </sst>
 </file>
@@ -594,6 +627,94 @@
         <a:xfrm>
           <a:off x="2867026" y="600075"/>
           <a:ext cx="4838700" cy="676369"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>895350</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3743723</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>183</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A7977868-6FED-4F2A-BB51-24589D1230A5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3714750" y="1733550"/>
+          <a:ext cx="2848373" cy="1314633"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4829175</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>105127</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{85D88232-4D10-43ED-BCE0-A7346AFF16BB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2857500" y="3486150"/>
+          <a:ext cx="4791075" cy="2524477"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1607,7 +1728,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -1661,14 +1782,85 @@
     <row r="8" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C8" s="5"/>
     </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="D9" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D10" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D11" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D12" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D16" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C17" s="5"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D18" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D19" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D20" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D21" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D22" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D31" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C32" s="5"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" xr:uid="{D7F7FCDC-490D-464B-8AC6-FB046B8CD003}"/>
     <hyperlink ref="D7" r:id="rId2" xr:uid="{9DB89340-9260-4ACB-BC3F-99EE5C02ED06}"/>
+    <hyperlink ref="A9" r:id="rId3" xr:uid="{667FAD27-3BED-45E9-9E97-5F74637E28CC}"/>
+    <hyperlink ref="D16" r:id="rId4" xr:uid="{9286C815-A01C-4238-8F25-586F52E5AFCB}"/>
+    <hyperlink ref="A18" r:id="rId5" xr:uid="{E118E9A3-7847-445D-B795-52CF7974AD4F}"/>
+    <hyperlink ref="D31" r:id="rId6" xr:uid="{CB3B5519-6706-4D91-8ED8-B03622537410}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId3"/>
-  <drawing r:id="rId4"/>
+  <pageSetup orientation="portrait" r:id="rId7"/>
+  <drawing r:id="rId8"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Jan 30 - Parenthesis
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6C186E3-2519-49A6-9768-80607FE4E58D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7202448-D1B9-4A83-ADF3-DEAF72F8F66F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="template" sheetId="2" r:id="rId1"/>
-    <sheet name="dp" sheetId="6" r:id="rId2"/>
-    <sheet name="Array" sheetId="4" r:id="rId3"/>
-    <sheet name="Matrix" sheetId="5" r:id="rId4"/>
-    <sheet name="Linked list" sheetId="3" r:id="rId5"/>
-    <sheet name="Rain water trap" sheetId="1" r:id="rId6"/>
+    <sheet name="Parenthesis" sheetId="7" r:id="rId2"/>
+    <sheet name="dp" sheetId="6" r:id="rId3"/>
+    <sheet name="Array" sheetId="4" r:id="rId4"/>
+    <sheet name="Matrix" sheetId="5" r:id="rId5"/>
+    <sheet name="Linked list" sheetId="3" r:id="rId6"/>
+    <sheet name="Rain water trap" sheetId="1" r:id="rId7"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="149">
   <si>
     <t>Statement</t>
   </si>
@@ -448,6 +449,42 @@
   </si>
   <si>
     <t>edge case : if both pointers reach ends</t>
+  </si>
+  <si>
+    <t>20. Valid Parentheses</t>
+  </si>
+  <si>
+    <t>If opening bracket : add to stack</t>
+  </si>
+  <si>
+    <t>elseif stack non-empty and stack peek has opening match of current then stack pop</t>
+  </si>
+  <si>
+    <t>return false</t>
+  </si>
+  <si>
+    <t>finally return stack isEmpty or not</t>
+  </si>
+  <si>
+    <t>678. Valid Parenthesis String</t>
+  </si>
+  <si>
+    <t>Maintain 2 vars leftMax and leftMin</t>
+  </si>
+  <si>
+    <t>for ( incr both, and for ) decr both</t>
+  </si>
+  <si>
+    <t>for wildcard, incr leftMin (consider * as left), and vice-versa</t>
+  </si>
+  <si>
+    <t>if at any point leftMax is -ve, return false</t>
+  </si>
+  <si>
+    <t>if at any point leftMin is -ve set it as zero</t>
+  </si>
+  <si>
+    <t>finally return if leftMin is zero</t>
   </si>
 </sst>
 </file>
@@ -560,7 +597,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3"/>
@@ -569,6 +606,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Calculation" xfId="2" builtinId="22"/>
@@ -590,6 +630,94 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1266825</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1448002" cy="409632"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E98B9060-767F-4501-A00D-7FFEBCE6971B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4086225" y="6296025"/>
+          <a:ext cx="1448002" cy="409632"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1266825</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2648143</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>104843</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{45151AE5-3DF5-4417-ABB8-A19C9813B355}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4086225" y="2095500"/>
+          <a:ext cx="1381318" cy="485843"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -726,7 +854,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -819,7 +947,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -868,7 +996,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1181,7 +1309,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1727,6 +1855,120 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AAA3DB6-B181-432C-9183-F47857237DA8}">
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="2" max="2" width="73.85546875" customWidth="1"/>
+    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D3" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D9" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C10" s="5"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="D11" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D12" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D13" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D15" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D16" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="18" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D18" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C19" s="5"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{A24F529E-D0E4-4D7C-8940-2EF8A048917C}"/>
+    <hyperlink ref="D9" r:id="rId2" xr:uid="{3733EA6B-CA32-4A95-A915-04BBA49179CD}"/>
+    <hyperlink ref="A11" r:id="rId3" xr:uid="{DF0AC1E1-3EA5-40DA-A2FC-0C7AB70D8D78}"/>
+    <hyperlink ref="D18" r:id="rId4" xr:uid="{305DB711-02E8-46A6-A4B2-FBE63ADC1454}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
   <dimension ref="A1:D32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1851,20 +2093,17 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" xr:uid="{D7F7FCDC-490D-464B-8AC6-FB046B8CD003}"/>
-    <hyperlink ref="D7" r:id="rId2" xr:uid="{9DB89340-9260-4ACB-BC3F-99EE5C02ED06}"/>
-    <hyperlink ref="A9" r:id="rId3" xr:uid="{667FAD27-3BED-45E9-9E97-5F74637E28CC}"/>
-    <hyperlink ref="D16" r:id="rId4" xr:uid="{9286C815-A01C-4238-8F25-586F52E5AFCB}"/>
-    <hyperlink ref="A18" r:id="rId5" xr:uid="{E118E9A3-7847-445D-B795-52CF7974AD4F}"/>
-    <hyperlink ref="D31" r:id="rId6" xr:uid="{CB3B5519-6706-4D91-8ED8-B03622537410}"/>
+    <hyperlink ref="D16" r:id="rId1" xr:uid="{9286C815-A01C-4238-8F25-586F52E5AFCB}"/>
+    <hyperlink ref="A18" r:id="rId2" xr:uid="{E118E9A3-7847-445D-B795-52CF7974AD4F}"/>
+    <hyperlink ref="D31" r:id="rId3" xr:uid="{CB3B5519-6706-4D91-8ED8-B03622537410}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId7"/>
-  <drawing r:id="rId8"/>
+  <pageSetup orientation="portrait" r:id="rId4"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDA924A8-9114-46BA-B39C-6743F04F80F3}">
   <dimension ref="A1:D22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1998,7 +2237,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83AD0EA2-442A-436B-AA00-D0DF9DB7227A}">
   <dimension ref="A1:D20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2069,7 +2308,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56E27646-854C-4719-A92C-78F24A8C7C41}">
   <dimension ref="A1:D100"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2482,7 +2721,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CE8EF6C-9017-4EEF-A2CD-F2424B35AA25}">
   <dimension ref="A1:D68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Queue - Feb 2nd 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,18 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7202448-D1B9-4A83-ADF3-DEAF72F8F66F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{759362D2-F8E7-45EB-83DD-D9C5905F59C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="template" sheetId="2" r:id="rId1"/>
     <sheet name="Parenthesis" sheetId="7" r:id="rId2"/>
-    <sheet name="dp" sheetId="6" r:id="rId3"/>
-    <sheet name="Array" sheetId="4" r:id="rId4"/>
-    <sheet name="Matrix" sheetId="5" r:id="rId5"/>
-    <sheet name="Linked list" sheetId="3" r:id="rId6"/>
-    <sheet name="Rain water trap" sheetId="1" r:id="rId7"/>
+    <sheet name="Stack" sheetId="8" r:id="rId3"/>
+    <sheet name="Queue" sheetId="9" r:id="rId4"/>
+    <sheet name="dp" sheetId="6" r:id="rId5"/>
+    <sheet name="Array" sheetId="4" r:id="rId6"/>
+    <sheet name="Matrix" sheetId="5" r:id="rId7"/>
+    <sheet name="Linked list" sheetId="3" r:id="rId8"/>
+    <sheet name="Rain water trap" sheetId="1" r:id="rId9"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -38,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="161">
   <si>
     <t>Statement</t>
   </si>
@@ -485,6 +487,42 @@
   </si>
   <si>
     <t>finally return if leftMin is zero</t>
+  </si>
+  <si>
+    <t>853. Car Fleet</t>
+  </si>
+  <si>
+    <t>sort positions in desc (take care of order of speed by pair), because farthest car cannot be crossed</t>
+  </si>
+  <si>
+    <t>take the times taken by each car</t>
+  </si>
+  <si>
+    <t>add current car to stack if car next to it reaches before</t>
+  </si>
+  <si>
+    <t>note: while dividing distance by speed, make sure speed is in double</t>
+  </si>
+  <si>
+    <t>239. Sliding Window Maximum</t>
+  </si>
+  <si>
+    <t>Use a queue</t>
+  </si>
+  <si>
+    <t>&gt; make sure previous elements in queue are not greater than current</t>
+  </si>
+  <si>
+    <t>&gt; make sure elements out of window doesn't exist</t>
+  </si>
+  <si>
+    <t>while adding current element index:</t>
+  </si>
+  <si>
+    <t>add element</t>
+  </si>
+  <si>
+    <t>thus element at end of queue that remained is always max of current window</t>
   </si>
 </sst>
 </file>
@@ -722,6 +760,104 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4867275</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>105001</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{661829F7-2C76-4BFA-A49C-305648DCF160}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2876550" y="581025"/>
+          <a:ext cx="4810125" cy="1619476"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>647700</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3848547</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>316</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D2F9B49A-F371-4B0F-99A4-5225B872C59A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3467100" y="590550"/>
+          <a:ext cx="3200847" cy="2267266"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>47626</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>28575</xdr:rowOff>
@@ -854,7 +990,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -947,7 +1083,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -996,7 +1132,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1309,7 +1445,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1969,6 +2105,158 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5D8A62A-F83B-49C3-B94F-89CCE841A84E}">
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="2" max="2" width="73.85546875" customWidth="1"/>
+    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D11" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C12" s="5"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{6AAE33F8-490C-4B54-A064-DB29A73C2FC0}"/>
+    <hyperlink ref="D11" r:id="rId2" xr:uid="{9F89C3A2-3C08-4ECF-9472-88C559CBD6E0}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51C4CDD9-9363-46B2-A2D8-BE11DE99714D}">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="2" max="2" width="73.85546875" customWidth="1"/>
+    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="D3" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D6" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D8" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D15" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C16" s="5"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{939F716F-C15C-4A88-A6E5-FB3DE8101485}"/>
+    <hyperlink ref="D15" r:id="rId2" xr:uid="{8A4FF2B5-4B6B-44D6-AA37-2257F9852D45}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
   <dimension ref="A1:D32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2103,7 +2391,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDA924A8-9114-46BA-B39C-6743F04F80F3}">
   <dimension ref="A1:D22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2237,7 +2525,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83AD0EA2-442A-436B-AA00-D0DF9DB7227A}">
   <dimension ref="A1:D20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2308,7 +2596,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56E27646-854C-4719-A92C-78F24A8C7C41}">
   <dimension ref="A1:D100"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2721,7 +3009,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CE8EF6C-9017-4EEF-A2CD-F2424B35AA25}">
   <dimension ref="A1:D68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
LRUCache - Feb 13 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -1,27 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24729"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B3F7231-DC25-4105-B5C9-EC852E08B9B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FA581F8-321D-4A44-9DF4-996EF84A344C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="10" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="template" sheetId="2" r:id="rId1"/>
-    <sheet name="Parenthesis" sheetId="7" r:id="rId2"/>
-    <sheet name="Stack" sheetId="8" r:id="rId3"/>
-    <sheet name="Queue" sheetId="9" r:id="rId4"/>
-    <sheet name="dp" sheetId="6" r:id="rId5"/>
-    <sheet name="Array" sheetId="4" r:id="rId6"/>
-    <sheet name="Matrix" sheetId="5" r:id="rId7"/>
-    <sheet name="Linked list" sheetId="3" r:id="rId8"/>
-    <sheet name="Rain water trap" sheetId="1" r:id="rId9"/>
+    <sheet name="greedy" sheetId="10" r:id="rId2"/>
+    <sheet name="Parenthesis" sheetId="7" r:id="rId3"/>
+    <sheet name="Stack" sheetId="8" r:id="rId4"/>
+    <sheet name="Queue" sheetId="9" r:id="rId5"/>
+    <sheet name="dp" sheetId="6" r:id="rId6"/>
+    <sheet name="Array" sheetId="4" r:id="rId7"/>
+    <sheet name="Matrix" sheetId="5" r:id="rId8"/>
+    <sheet name="Linked list" sheetId="3" r:id="rId9"/>
+    <sheet name="Rain water trap" sheetId="1" r:id="rId10"/>
+    <sheet name="Low level design" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -40,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="172">
   <si>
     <t>Statement</t>
   </si>
@@ -538,13 +540,31 @@
   </si>
   <si>
     <t>&gt; if closecount &lt; opencount, do the same for ")"</t>
+  </si>
+  <si>
+    <t>create monotonous increasing stack</t>
+  </si>
+  <si>
+    <t>&gt; if current element is greater than previous - just add it to stack with its index</t>
+  </si>
+  <si>
+    <t>else remove, calculate area - and add current element with last removed elements index</t>
+  </si>
+  <si>
+    <t>&gt; at end stack will have only elements that are increasing - so width will be till end always..</t>
+  </si>
+  <si>
+    <t>146. LRU Cache</t>
+  </si>
+  <si>
+    <t>Use map with Integer key and doubly linked list Node as value</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -601,8 +621,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -617,6 +644,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -644,13 +676,14 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3"/>
@@ -662,11 +695,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="4"/>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="5">
     <cellStyle name="Calculation" xfId="2" builtinId="22"/>
     <cellStyle name="Good" xfId="1" builtinId="26"/>
     <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
+    <cellStyle name="Neutral" xfId="4" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1674,6 +1709,55 @@
         <a:xfrm>
           <a:off x="3276600" y="9725025"/>
           <a:ext cx="3914286" cy="3161905"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>133350</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4848225</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>133500</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{52E4C730-3BE1-44CF-9014-48300B6746B7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2952750" y="581025"/>
+          <a:ext cx="4714875" cy="1076475"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2049,7 +2133,357 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CE8EF6C-9017-4EEF-A2CD-F2424B35AA25}">
+  <dimension ref="A1:D68"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="2" max="2" width="73.85546875" customWidth="1"/>
+    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D18" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C19" s="5"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B20" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D21" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D22" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D23" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D24" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D25" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D26" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D28" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D30" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D31" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D32" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D34" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C35" s="5"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D36" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D37" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D38" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D39" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D40" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D41" s="9"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D42" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D43" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D44" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D45" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D46" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D47" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D49" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C50" s="5"/>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B51" t="s">
+        <v>34</v>
+      </c>
+      <c r="D51" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D52" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D53" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D54" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="67" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D67" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="68" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C68" s="5"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{F4D67A5D-744F-4C81-957E-33D3253297A2}"/>
+    <hyperlink ref="A20" r:id="rId2" xr:uid="{CDAA1F07-861A-43F8-806E-CBF196F42093}"/>
+    <hyperlink ref="D18" r:id="rId3" xr:uid="{30328AA2-76F9-472A-BAB3-B3B0C7802963}"/>
+    <hyperlink ref="D34" r:id="rId4" xr:uid="{FBB1B328-6337-43BB-960F-5B6CAE89E813}"/>
+    <hyperlink ref="A36" r:id="rId5" xr:uid="{33CB1418-814A-466E-8725-5800B98469F7}"/>
+    <hyperlink ref="D49" r:id="rId6" xr:uid="{6329D858-D8F3-4698-AF57-250A8ABB78A2}"/>
+    <hyperlink ref="A51" r:id="rId7" xr:uid="{C5538507-5156-4F6A-800E-694A86C1DE83}"/>
+    <hyperlink ref="D67" r:id="rId8" xr:uid="{A272D98F-93C2-491D-BEBC-54FFA0BBC858}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId9"/>
+  <drawing r:id="rId10"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7BE8B5F-B3C3-43A1-BD9C-D35CE748D483}">
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="2" max="2" width="73.85546875" customWidth="1"/>
+    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="D3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D9" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C10" s="5"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{976A6329-CE7B-45FA-9EC8-39B157036788}"/>
+    <hyperlink ref="D9" r:id="rId2" xr:uid="{60C7CCA8-6DFD-471B-BE7B-FBA6AA3D39EF}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55C26914-8137-4079-AF30-EE7EDC55D866}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="2" max="2" width="73.85546875" customWidth="1"/>
+    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AAA3DB6-B181-432C-9183-F47857237DA8}">
   <dimension ref="A1:D26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2196,7 +2630,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5D8A62A-F83B-49C3-B94F-89CCE841A84E}">
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2267,7 +2701,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51C4CDD9-9363-46B2-A2D8-BE11DE99714D}">
   <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2348,7 +2782,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
   <dimension ref="A1:D32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2483,7 +2917,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDA924A8-9114-46BA-B39C-6743F04F80F3}">
   <dimension ref="A1:D22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2617,7 +3051,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83AD0EA2-442A-436B-AA00-D0DF9DB7227A}">
   <dimension ref="A1:D20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2688,7 +3122,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56E27646-854C-4719-A92C-78F24A8C7C41}">
   <dimension ref="A1:D100"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3099,240 +3533,4 @@
   <pageSetup orientation="portrait" r:id="rId15"/>
   <drawing r:id="rId16"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CE8EF6C-9017-4EEF-A2CD-F2424B35AA25}">
-  <dimension ref="A1:D68"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="42.28515625" customWidth="1"/>
-    <col min="2" max="2" width="73.85546875" customWidth="1"/>
-    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="91.7109375" customWidth="1"/>
-    <col min="13" max="13" width="6.7109375" customWidth="1"/>
-    <col min="14" max="14" width="8.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C2" s="5"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C4" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D18" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C19" s="5"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B20" t="s">
-        <v>10</v>
-      </c>
-      <c r="D20" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D21" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D22" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D23" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D24" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D25" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D26" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D28" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D30" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D31" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D32" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D34" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C35" s="5"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D36" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D37" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D38" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D39" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D40" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D41" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D42" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D49" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C50" s="5"/>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B51" t="s">
-        <v>34</v>
-      </c>
-      <c r="D51" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D52" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D53" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D54" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="67" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="D67" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="68" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C68" s="5"/>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" xr:uid="{F4D67A5D-744F-4C81-957E-33D3253297A2}"/>
-    <hyperlink ref="A20" r:id="rId2" xr:uid="{CDAA1F07-861A-43F8-806E-CBF196F42093}"/>
-    <hyperlink ref="D18" r:id="rId3" xr:uid="{30328AA2-76F9-472A-BAB3-B3B0C7802963}"/>
-    <hyperlink ref="D34" r:id="rId4" xr:uid="{FBB1B328-6337-43BB-960F-5B6CAE89E813}"/>
-    <hyperlink ref="A36" r:id="rId5" xr:uid="{33CB1418-814A-466E-8725-5800B98469F7}"/>
-    <hyperlink ref="D49" r:id="rId6" xr:uid="{6329D858-D8F3-4698-AF57-250A8ABB78A2}"/>
-    <hyperlink ref="A51" r:id="rId7" xr:uid="{C5538507-5156-4F6A-800E-694A86C1DE83}"/>
-    <hyperlink ref="D67" r:id="rId8" xr:uid="{A272D98F-93C2-491D-BEBC-54FFA0BBC858}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId9"/>
-  <drawing r:id="rId10"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Trie Implementation - Feb 14 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FA581F8-321D-4A44-9DF4-996EF84A344C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B75ED3E9-82B3-4E1F-AA03-D0F57283EBA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="10" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="174">
   <si>
     <t>Statement</t>
   </si>
@@ -558,6 +558,12 @@
   </si>
   <si>
     <t>Use map with Integer key and doubly linked list Node as value</t>
+  </si>
+  <si>
+    <t>208. Implement Trie (Prefix Tree)</t>
+  </si>
+  <si>
+    <t>Create triNode with children - hashmap and isEnd boolean to check end of string</t>
   </si>
 </sst>
 </file>
@@ -1758,6 +1764,50 @@
         <a:xfrm>
           <a:off x="2952750" y="581025"/>
           <a:ext cx="4714875" cy="1076475"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4876800</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>152552</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6A0B79F1-825F-454F-9878-AE73349857FE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2876550" y="2114550"/>
+          <a:ext cx="4819650" cy="1086002"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2394,7 +2444,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7BE8B5F-B3C3-43A1-BD9C-D35CE748D483}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -2438,13 +2488,31 @@
     <row r="10" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C10" s="5"/>
     </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="D11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="17" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D17" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C18" s="5"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" xr:uid="{976A6329-CE7B-45FA-9EC8-39B157036788}"/>
     <hyperlink ref="D9" r:id="rId2" xr:uid="{60C7CCA8-6DFD-471B-BE7B-FBA6AA3D39EF}"/>
+    <hyperlink ref="A11" r:id="rId3" xr:uid="{B613807D-978E-4CA0-928A-B9CD9644C8F6}"/>
+    <hyperlink ref="D17" r:id="rId4" xr:uid="{6226ADC2-6F8E-4914-A1E9-DA822FBF2A00}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId3"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
dijkstra's - networkDelayTime - Feb 16 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1625C487-B80D-4511-91AE-678DE9424725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81ABCCE8-27F9-4BEB-AE2B-E28345B0C767}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="11" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="182">
   <si>
     <t>Statement</t>
   </si>
@@ -571,13 +571,53 @@
   </si>
   <si>
     <t>85. Maximal Rectangle</t>
+  </si>
+  <si>
+    <t>743. Network Delay Time</t>
+  </si>
+  <si>
+    <t>create adjacent list using as map v1 -&gt; [(v2, w)]</t>
+  </si>
+  <si>
+    <t>use minHeap (wrt weight) and add src vertex</t>
+  </si>
+  <si>
+    <t>while heap is empty remove top element and add its adj nodes</t>
+  </si>
+  <si>
+    <t>but here keep noting the max weight and visit all vertexes</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">for normal </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>dijkstra's</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> we compare dest if removed node is destination</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -644,6 +684,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -866,6 +913,55 @@
         <a:xfrm>
           <a:off x="3181350" y="3867150"/>
           <a:ext cx="3829584" cy="485843"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>533400</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4458248</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>171840</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C8BF61F0-8C11-4999-AFCC-E8237884BC76}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3352800" y="1381125"/>
+          <a:ext cx="3924848" cy="2791215"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2540,7 +2636,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E87A3A0-D815-41F9-954B-826D58641E2B}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -2579,11 +2675,51 @@
     <row r="6" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C6" s="5"/>
     </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="D7" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D8" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D10" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D11" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="22" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D22" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C23" s="5"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" xr:uid="{414C119C-B593-46C0-B062-D367285561EC}"/>
+    <hyperlink ref="A7" r:id="rId2" xr:uid="{B9CA0EA5-4F0F-4EFF-AFEE-A344B19A5F86}"/>
+    <hyperlink ref="D22" r:id="rId3" xr:uid="{6B6353B9-F816-42F2-BA1E-3D7BDF1A1DCD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId4"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
cost to connect all points in 2d axis
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81ABCCE8-27F9-4BEB-AE2B-E28345B0C767}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8168D8E-4E9A-495B-B823-69C16CC6AC93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="11" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="186">
   <si>
     <t>Statement</t>
   </si>
@@ -611,6 +611,18 @@
       </rPr>
       <t xml:space="preserve"> we compare dest if removed node is destination</t>
     </r>
+  </si>
+  <si>
+    <t>1584. Min Cost to Connect All Points</t>
+  </si>
+  <si>
+    <t>Prims algorithm</t>
+  </si>
+  <si>
+    <t>consider each point as vertex</t>
+  </si>
+  <si>
+    <t>add cost every time a new vertex comes out of minHeap</t>
   </si>
 </sst>
 </file>
@@ -962,6 +974,50 @@
         <a:xfrm>
           <a:off x="3352800" y="1381125"/>
           <a:ext cx="3924848" cy="2791215"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>695325</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4210541</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>105234</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6E3CCC62-444B-4F0A-AA4F-63EE120A8F8F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3514725" y="4629150"/>
+          <a:ext cx="3515216" cy="3286584"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2636,7 +2692,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E87A3A0-D815-41F9-954B-826D58641E2B}">
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -2703,23 +2759,51 @@
         <v>180</v>
       </c>
     </row>
-    <row r="22" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D22" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C23" s="5"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="D24" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D25" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D26" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="42" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D42" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C43" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" xr:uid="{414C119C-B593-46C0-B062-D367285561EC}"/>
     <hyperlink ref="A7" r:id="rId2" xr:uid="{B9CA0EA5-4F0F-4EFF-AFEE-A344B19A5F86}"/>
     <hyperlink ref="D22" r:id="rId3" xr:uid="{6B6353B9-F816-42F2-BA1E-3D7BDF1A1DCD}"/>
+    <hyperlink ref="A24" r:id="rId4" xr:uid="{D61A6DAF-DB73-42F2-9403-929004DBE0ED}"/>
+    <hyperlink ref="D42" r:id="rId5" xr:uid="{F3A8C9B4-E9D7-40BD-998D-9D8B5A0C2897}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
-  <drawing r:id="rId5"/>
+  <pageSetup orientation="portrait" r:id="rId6"/>
+  <drawing r:id="rId7"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
cloneGraph - Feb 18 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8168D8E-4E9A-495B-B823-69C16CC6AC93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F199E3D-8DD0-4FE4-9069-D353D6939AAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="11" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="196">
   <si>
     <t>Statement</t>
   </si>
@@ -623,6 +623,60 @@
   </si>
   <si>
     <t>add cost every time a new vertex comes out of minHeap</t>
+  </si>
+  <si>
+    <t>178 · Graph Valid Tree</t>
+  </si>
+  <si>
+    <t>dfs from starting vertex</t>
+  </si>
+  <si>
+    <t>leetcode</t>
+  </si>
+  <si>
+    <t>for each neighbour call dfs</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">if visited size is not == n then return false - as it will </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>not be connected graph</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">if ever a vertex is visited again return false - (handle prev vertex) - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>cycle detection</t>
+    </r>
+  </si>
+  <si>
+    <t>133. Clone Graph</t>
+  </si>
+  <si>
+    <t>dfs</t>
+  </si>
+  <si>
+    <t>copy node and store it in hashmap as value with key as original node</t>
+  </si>
+  <si>
+    <t>and do this recursively for all neighbors</t>
   </si>
 </sst>
 </file>
@@ -1018,6 +1072,94 @@
         <a:xfrm>
           <a:off x="3514725" y="4629150"/>
           <a:ext cx="3515216" cy="3286584"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>180975</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4801245</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>19131</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5C7BFA47-99A5-4DD4-A65C-538204B1AA00}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3000375" y="8391525"/>
+          <a:ext cx="4620270" cy="581106"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>142875</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4819650</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>115191</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5C8B32F2-4113-49E3-BBD5-96C105B8A12A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2962275" y="9734550"/>
+          <a:ext cx="4676775" cy="6382641"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2692,7 +2834,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E87A3A0-D815-41F9-954B-826D58641E2B}">
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D86"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -2785,13 +2927,73 @@
         <v>185</v>
       </c>
     </row>
-    <row r="42" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D42" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="43" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C43" s="5"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="D44" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D45" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="D46" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D47" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D49" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C50" s="5"/>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="D51" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D52" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D53" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="70" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D70" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="3:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C86" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2800,10 +3002,15 @@
     <hyperlink ref="D22" r:id="rId3" xr:uid="{6B6353B9-F816-42F2-BA1E-3D7BDF1A1DCD}"/>
     <hyperlink ref="A24" r:id="rId4" xr:uid="{D61A6DAF-DB73-42F2-9403-929004DBE0ED}"/>
     <hyperlink ref="D42" r:id="rId5" xr:uid="{F3A8C9B4-E9D7-40BD-998D-9D8B5A0C2897}"/>
+    <hyperlink ref="A44" r:id="rId6" xr:uid="{ED8C921A-4967-4122-958D-181A85084C3B}"/>
+    <hyperlink ref="A46" r:id="rId7" xr:uid="{89A4A849-7B5D-40EE-8695-C17AF750CDCA}"/>
+    <hyperlink ref="D49" r:id="rId8" xr:uid="{2F45B791-FFC4-4EED-BAE1-F6993629E708}"/>
+    <hyperlink ref="A51" r:id="rId9" xr:uid="{672C6366-C89C-4627-9004-8E5507FB8AA0}"/>
+    <hyperlink ref="D70" r:id="rId10" xr:uid="{A9AC05DA-6BC8-43F2-AFAD-89C00D3D4512}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId6"/>
-  <drawing r:id="rId7"/>
+  <pageSetup orientation="portrait" r:id="rId11"/>
+  <drawing r:id="rId12"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
SurroundedRegions - 19 Feb 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F199E3D-8DD0-4FE4-9069-D353D6939AAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3A6894B-8CBB-495A-ADD8-0843A39FE551}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="11" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="205">
   <si>
     <t>Statement</t>
   </si>
@@ -677,6 +677,33 @@
   </si>
   <si>
     <t>and do this recursively for all neighbors</t>
+  </si>
+  <si>
+    <t>207. Course Schedule</t>
+  </si>
+  <si>
+    <t>keep a visited set</t>
+  </si>
+  <si>
+    <t>for each book as start, do dfs</t>
+  </si>
+  <si>
+    <t>if any node is visited twice return false - loop means not possible to read all books</t>
+  </si>
+  <si>
+    <t>create adj list - graph is directed</t>
+  </si>
+  <si>
+    <t>finally if visited set equals total vertexes - then return true</t>
+  </si>
+  <si>
+    <t>130. Surrounded Regions</t>
+  </si>
+  <si>
+    <t>do dfs on border cells - change all O linked cells to Temp T</t>
+  </si>
+  <si>
+    <t>then change remaining O to X and T to O</t>
   </si>
 </sst>
 </file>
@@ -1160,6 +1187,94 @@
         <a:xfrm>
           <a:off x="2962275" y="9734550"/>
           <a:ext cx="4676775" cy="6382641"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>87</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4896528</xdr:colOff>
+      <xdr:row>91</xdr:row>
+      <xdr:rowOff>95364</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{419BD70B-D29F-47D2-98A4-795635A21345}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2857500" y="16611600"/>
+          <a:ext cx="4858428" cy="819264"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>19051</xdr:colOff>
+      <xdr:row>97</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4895851</xdr:colOff>
+      <xdr:row>111</xdr:row>
+      <xdr:rowOff>181371</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DCA87E4E-91D5-41F2-AA12-C5D1F1A1C95A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2838451" y="18488025"/>
+          <a:ext cx="4876800" cy="2838846"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2834,7 +2949,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E87A3A0-D815-41F9-954B-826D58641E2B}">
-  <dimension ref="A1:D86"/>
+  <dimension ref="A1:D113"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -2992,8 +3107,70 @@
         <v>9</v>
       </c>
     </row>
-    <row r="86" spans="3:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C86" s="5"/>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="D87" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D88" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D89" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D90" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D91" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D92" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D95" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C96" s="5"/>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="D97" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D98" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D111" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="3:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C113" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3007,10 +3184,14 @@
     <hyperlink ref="D49" r:id="rId8" xr:uid="{2F45B791-FFC4-4EED-BAE1-F6993629E708}"/>
     <hyperlink ref="A51" r:id="rId9" xr:uid="{672C6366-C89C-4627-9004-8E5507FB8AA0}"/>
     <hyperlink ref="D70" r:id="rId10" xr:uid="{A9AC05DA-6BC8-43F2-AFAD-89C00D3D4512}"/>
+    <hyperlink ref="A87" r:id="rId11" xr:uid="{DC0604AA-792A-43AF-911E-C9540B23F78C}"/>
+    <hyperlink ref="D95" r:id="rId12" xr:uid="{8872328D-61D7-4547-8FF7-479ED08BFBCC}"/>
+    <hyperlink ref="A97" r:id="rId13" xr:uid="{FFC83952-6DF4-4D2B-9794-7BE41DB5095E}"/>
+    <hyperlink ref="D111" r:id="rId14" xr:uid="{3EE638A9-17A4-457C-9C53-D2E84457850F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId11"/>
-  <drawing r:id="rId12"/>
+  <pageSetup orientation="portrait" r:id="rId15"/>
+  <drawing r:id="rId16"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
NumberofIslands - Feb 19 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3A6894B-8CBB-495A-ADD8-0843A39FE551}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5C60FCE-265F-448B-BB08-CAC39D28449A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="11" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="template" sheetId="2" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="212">
   <si>
     <t>Statement</t>
   </si>
@@ -704,6 +704,27 @@
   </si>
   <si>
     <t>then change remaining O to X and T to O</t>
+  </si>
+  <si>
+    <t>200. Number of Islands</t>
+  </si>
+  <si>
+    <t>if any index has 1 - do dfs starting from that and count++</t>
+  </si>
+  <si>
+    <t>463. Island Perimeter</t>
+  </si>
+  <si>
+    <t>if for any land start dfs</t>
+  </si>
+  <si>
+    <t>keep a visited set to keep track of visited land</t>
+  </si>
+  <si>
+    <t>if we find any water or out of bounds index return 1</t>
+  </si>
+  <si>
+    <t>else keep dfs'ing in 4 directions</t>
   </si>
 </sst>
 </file>
@@ -1652,6 +1673,94 @@
         <a:xfrm>
           <a:off x="3543300" y="628650"/>
           <a:ext cx="3372321" cy="2915057"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1352550</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3191132</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>162128</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{917E0654-9350-4167-BF0F-2B3E2917DBA5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4171950" y="4038600"/>
+          <a:ext cx="1838582" cy="1457528"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>447675</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4534470</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>105129</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F06FCB54-AFC9-4DD0-9544-A3A0C9A19CA6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3267075" y="5953125"/>
+          <a:ext cx="4086795" cy="2534004"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3802,7 +3911,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83AD0EA2-442A-436B-AA00-D0DF9DB7227A}">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -3853,21 +3962,77 @@
         <v>107</v>
       </c>
     </row>
-    <row r="19" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D19" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C20" s="5"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="D21" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D22" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D29" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C30" s="5"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="D31" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D32" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="33" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D33" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="34" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D34" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="43" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D43" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C46" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" display="Spiral Matrix" xr:uid="{EE24117A-8086-489D-A2CA-CE3F018A6E74}"/>
     <hyperlink ref="D19" r:id="rId2" xr:uid="{40B2AEAE-4A71-4E88-BD4B-30765B996FE5}"/>
+    <hyperlink ref="A21" r:id="rId3" xr:uid="{ABA8CF29-614D-4606-B196-05F9C79E2AB1}"/>
+    <hyperlink ref="D29" r:id="rId4" xr:uid="{AE068BF9-E00D-4A52-912C-FAF893DCE140}"/>
+    <hyperlink ref="A31" r:id="rId5" xr:uid="{E38CCC9C-9408-4335-8A45-68FC60A3701A}"/>
+    <hyperlink ref="D43" r:id="rId6" xr:uid="{60E813ED-AC35-4B86-9781-5B80FA133723}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId3"/>
+  <drawing r:id="rId7"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
removeKdigits stack - Feb 19 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5C60FCE-265F-448B-BB08-CAC39D28449A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCAE968E-47A6-4A56-A09F-768867AD10C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="template" sheetId="2" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="219">
   <si>
     <t>Statement</t>
   </si>
@@ -726,12 +726,33 @@
   <si>
     <t>else keep dfs'ing in 4 directions</t>
   </si>
+  <si>
+    <t>402. Remove K Digits</t>
+  </si>
+  <si>
+    <t>Use monotonic increasing stack</t>
+  </si>
+  <si>
+    <t>ie. If number is increasing than previous in stack just add to stack</t>
+  </si>
+  <si>
+    <t>else keep removing till k &gt; 0 and previous is greater</t>
+  </si>
+  <si>
+    <t>finally remove last ones if k still &gt; 0</t>
+  </si>
+  <si>
+    <t>12345 means remove from last</t>
+  </si>
+  <si>
+    <t>54321 means remove from first</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -809,6 +830,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -862,15 +891,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="6">
+  <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3"/>
@@ -884,10 +914,12 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="4" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="6"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="7">
     <cellStyle name="Bad" xfId="5" builtinId="27"/>
     <cellStyle name="Calculation" xfId="2" builtinId="22"/>
+    <cellStyle name="Explanatory Text" xfId="6" builtinId="53"/>
     <cellStyle name="Good" xfId="1" builtinId="26"/>
     <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
     <cellStyle name="Neutral" xfId="4" builtinId="28"/>
@@ -1345,6 +1377,50 @@
         <a:xfrm>
           <a:off x="2876550" y="581025"/>
           <a:ext cx="4810125" cy="1619476"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1171575</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3295946</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>95312</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D9304C8E-6D04-4480-AC28-668B02851827}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3990975" y="2505075"/>
+          <a:ext cx="2124371" cy="447737"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2894,32 +2970,32 @@
       <c r="D41" s="8"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D42" t="s">
+      <c r="D42" s="11" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D43" t="s">
+      <c r="D43" s="11" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D44" t="s">
+      <c r="D44" s="11" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D45" t="s">
+      <c r="D45" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D46" t="s">
+      <c r="D46" s="11" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D47" t="s">
+      <c r="D47" s="11" t="s">
         <v>29</v>
       </c>
     </row>
@@ -3488,7 +3564,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5D8A62A-F83B-49C3-B94F-89CCE841A84E}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -3547,13 +3623,52 @@
     <row r="12" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C12" s="5"/>
     </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="D13" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C14" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D14" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D15" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D16" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="18" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D18" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C19" s="5"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" xr:uid="{6AAE33F8-490C-4B54-A064-DB29A73C2FC0}"/>
     <hyperlink ref="D11" r:id="rId2" xr:uid="{9F89C3A2-3C08-4ECF-9472-88C559CBD6E0}"/>
+    <hyperlink ref="A13" r:id="rId3" xr:uid="{9B0E0792-F2BF-4326-AE22-484FC8152DDE}"/>
+    <hyperlink ref="D18" r:id="rId4" xr:uid="{E62DF899-E1F2-4263-802D-E6519B60DC6C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId3"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
alien dictionary - Feb 21 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCAE968E-47A6-4A56-A09F-768867AD10C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F36DAFD7-99E4-40B0-84D6-F9DEABCCEF4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="12" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="template" sheetId="2" r:id="rId1"/>
@@ -25,6 +25,7 @@
     <sheet name="Rain water trap" sheetId="1" r:id="rId10"/>
     <sheet name="Low level design" sheetId="11" r:id="rId11"/>
     <sheet name="Graph" sheetId="12" r:id="rId12"/>
+    <sheet name="Dictionary" sheetId="13" r:id="rId13"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="222">
   <si>
     <t>Statement</t>
   </si>
@@ -746,6 +747,15 @@
   </si>
   <si>
     <t>54321 means remove from first</t>
+  </si>
+  <si>
+    <t>953. Verifying an Alien Dictionary</t>
+  </si>
+  <si>
+    <t>Create an array[26] and add new topological order</t>
+  </si>
+  <si>
+    <t xml:space="preserve">for all consecutive pairs - compare </t>
   </si>
 </sst>
 </file>
@@ -1328,6 +1338,55 @@
         <a:xfrm>
           <a:off x="2838451" y="18488025"/>
           <a:ext cx="4876800" cy="2838846"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4895850</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>38156</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BD7495A4-0DA6-48C1-A492-701084AE0AAB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2867025" y="590550"/>
+          <a:ext cx="4848225" cy="400106"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3380,6 +3439,67 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{170CF2C0-E5DC-4FCA-8D73-E7E5C7297110}">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="2" max="2" width="73.85546875" customWidth="1"/>
+    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="D3" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D6" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C7" s="5"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{F701FCD9-E8B1-4408-A945-690189F730C8}"/>
+    <hyperlink ref="D6" r:id="rId2" xr:uid="{E3A37132-9B1F-4936-A0FA-8D44020D3DD2}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55C26914-8137-4079-AF30-EE7EDC55D866}">
   <dimension ref="A1:D2"/>

</xml_diff>

<commit_message>
quickSort && quickSelect - 22 Feb 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,24 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F36DAFD7-99E4-40B0-84D6-F9DEABCCEF4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72C5F417-EF5E-41BC-9259-0378C505FA68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="12" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="13" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
-    <sheet name="template" sheetId="2" r:id="rId1"/>
-    <sheet name="greedy" sheetId="10" r:id="rId2"/>
-    <sheet name="Parenthesis" sheetId="7" r:id="rId3"/>
-    <sheet name="Stack" sheetId="8" r:id="rId4"/>
-    <sheet name="Queue" sheetId="9" r:id="rId5"/>
-    <sheet name="dp" sheetId="6" r:id="rId6"/>
-    <sheet name="Array" sheetId="4" r:id="rId7"/>
-    <sheet name="Matrix" sheetId="5" r:id="rId8"/>
-    <sheet name="Linked list" sheetId="3" r:id="rId9"/>
-    <sheet name="Rain water trap" sheetId="1" r:id="rId10"/>
-    <sheet name="Low level design" sheetId="11" r:id="rId11"/>
-    <sheet name="Graph" sheetId="12" r:id="rId12"/>
-    <sheet name="Dictionary" sheetId="13" r:id="rId13"/>
+    <sheet name="greedy" sheetId="10" r:id="rId1"/>
+    <sheet name="Parenthesis" sheetId="7" r:id="rId2"/>
+    <sheet name="Stack" sheetId="8" r:id="rId3"/>
+    <sheet name="Queue" sheetId="9" r:id="rId4"/>
+    <sheet name="dp" sheetId="6" r:id="rId5"/>
+    <sheet name="Array" sheetId="4" r:id="rId6"/>
+    <sheet name="Matrix" sheetId="5" r:id="rId7"/>
+    <sheet name="Linked list" sheetId="3" r:id="rId8"/>
+    <sheet name="Rain water trap" sheetId="1" r:id="rId9"/>
+    <sheet name="Low level design" sheetId="11" r:id="rId10"/>
+    <sheet name="Graph" sheetId="12" r:id="rId11"/>
+    <sheet name="Dictionary" sheetId="13" r:id="rId12"/>
+    <sheet name="template" sheetId="2" r:id="rId13"/>
+    <sheet name="Sorting Algorithms" sheetId="15" r:id="rId14"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="231">
   <si>
     <t>Statement</t>
   </si>
@@ -756,6 +757,33 @@
   </si>
   <si>
     <t xml:space="preserve">for all consecutive pairs - compare </t>
+  </si>
+  <si>
+    <t>Quick sort</t>
+  </si>
+  <si>
+    <t>215. Kth Largest Element in an Array</t>
+  </si>
+  <si>
+    <t>use priority queue - minHeap</t>
+  </si>
+  <si>
+    <t>add elements and remove 1 while adding if size is k+1 - so we maintain only k at a given time</t>
+  </si>
+  <si>
+    <t>finally remove one to get kth largest</t>
+  </si>
+  <si>
+    <t>Using quick-select like quick-sort</t>
+  </si>
+  <si>
+    <t>select pivot (last index) and find its position</t>
+  </si>
+  <si>
+    <t>finding kth largest means means newK = n-kth smallest</t>
+  </si>
+  <si>
+    <t>do quick select until newK is pivot</t>
   </si>
 </sst>
 </file>
@@ -1387,6 +1415,55 @@
         <a:xfrm>
           <a:off x="2867025" y="590550"/>
           <a:ext cx="4848225" cy="400106"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>923925</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3410297</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>114384</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{381FF2E1-DE0E-4FD0-84D9-1D3679F1C0E3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3743325" y="466725"/>
+          <a:ext cx="2486372" cy="600159"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2824,7 +2901,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10429FF1-7DBA-415E-968E-9D236B8DC32D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55C26914-8137-4079-AF30-EE7EDC55D866}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2859,265 +2936,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CE8EF6C-9017-4EEF-A2CD-F2424B35AA25}">
-  <dimension ref="A1:D68"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="42.28515625" customWidth="1"/>
-    <col min="2" max="2" width="73.85546875" customWidth="1"/>
-    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="91.7109375" customWidth="1"/>
-    <col min="13" max="13" width="6.7109375" customWidth="1"/>
-    <col min="14" max="14" width="8.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C2" s="5"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
-        <v>172</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D18" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C19" s="5"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="9" t="s">
-        <v>173</v>
-      </c>
-      <c r="B20" t="s">
-        <v>8</v>
-      </c>
-      <c r="D20" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D21" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D22" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D23" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D24" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D25" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D26" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D28" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D30" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D31" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D32" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D34" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C35" s="5"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="9" t="s">
-        <v>174</v>
-      </c>
-      <c r="D36" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D37" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D38" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D39" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D40" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D41" s="8"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D42" s="11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D43" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D44" s="11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D45" s="11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D46" s="11" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D47" s="11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D49" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C50" s="5"/>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="9" t="s">
-        <v>175</v>
-      </c>
-      <c r="B51" t="s">
-        <v>30</v>
-      </c>
-      <c r="D51" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D52" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D53" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D54" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="67" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="D67" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="68" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C68" s="5"/>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" display="Container with most water" xr:uid="{F4D67A5D-744F-4C81-957E-33D3253297A2}"/>
-    <hyperlink ref="A20" r:id="rId2" display="Trapping Rain Water" xr:uid="{CDAA1F07-861A-43F8-806E-CBF196F42093}"/>
-    <hyperlink ref="D18" r:id="rId3" xr:uid="{30328AA2-76F9-472A-BAB3-B3B0C7802963}"/>
-    <hyperlink ref="D34" r:id="rId4" xr:uid="{FBB1B328-6337-43BB-960F-5B6CAE89E813}"/>
-    <hyperlink ref="A36" r:id="rId5" display="Largest Rectangle in Histogram" xr:uid="{33CB1418-814A-466E-8725-5800B98469F7}"/>
-    <hyperlink ref="D49" r:id="rId6" xr:uid="{6329D858-D8F3-4698-AF57-250A8ABB78A2}"/>
-    <hyperlink ref="A51" r:id="rId7" display="Maximal Rectangle" xr:uid="{C5538507-5156-4F6A-800E-694A86C1DE83}"/>
-    <hyperlink ref="D67" r:id="rId8" xr:uid="{A272D98F-93C2-491D-BEBC-54FFA0BBC858}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId9"/>
-  <drawing r:id="rId10"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7BE8B5F-B3C3-43A1-BD9C-D35CE748D483}">
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3191,7 +3009,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E87A3A0-D815-41F9-954B-826D58641E2B}">
   <dimension ref="A1:D113"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3439,7 +3257,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{170CF2C0-E5DC-4FCA-8D73-E7E5C7297110}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3500,8 +3318,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55C26914-8137-4079-AF30-EE7EDC55D866}">
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10429FF1-7DBA-415E-968E-9D236B8DC32D}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3535,7 +3353,100 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0397D5EA-9127-4F39-A242-D8D4A93871ED}">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="2" max="2" width="73.85546875" customWidth="1"/>
+    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="D3" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D4" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D6" s="8"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D8" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D10" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D12" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C13" s="5"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A4" r:id="rId1" xr:uid="{CBB80B45-9FC6-4C3A-BE11-6373B320529E}"/>
+    <hyperlink ref="A3" r:id="rId2" xr:uid="{1B705FA7-8F6C-4A90-88DF-06E322C116EF}"/>
+    <hyperlink ref="D12" r:id="rId3" xr:uid="{87407450-9806-4982-AA5D-2AE0CB10FC73}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId4"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AAA3DB6-B181-432C-9183-F47857237DA8}">
   <dimension ref="A1:D26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3682,7 +3593,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5D8A62A-F83B-49C3-B94F-89CCE841A84E}">
   <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3792,7 +3703,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51C4CDD9-9363-46B2-A2D8-BE11DE99714D}">
   <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3873,7 +3784,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
   <dimension ref="A1:D32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4010,7 +3921,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDA924A8-9114-46BA-B39C-6743F04F80F3}">
   <dimension ref="A1:D22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4144,7 +4055,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83AD0EA2-442A-436B-AA00-D0DF9DB7227A}">
   <dimension ref="A1:D46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4271,7 +4182,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56E27646-854C-4719-A92C-78F24A8C7C41}">
   <dimension ref="A1:D100"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4682,4 +4593,263 @@
   <pageSetup orientation="portrait" r:id="rId15"/>
   <drawing r:id="rId16"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CE8EF6C-9017-4EEF-A2CD-F2424B35AA25}">
+  <dimension ref="A1:D68"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="2" max="2" width="73.85546875" customWidth="1"/>
+    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D18" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C19" s="5"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="B20" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D21" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D22" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D23" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D24" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D25" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D28" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D30" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D31" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D32" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D34" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C35" s="5"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="D36" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D37" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D38" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D39" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D40" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D41" s="8"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D42" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D43" s="11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D44" s="11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D45" s="11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D46" s="11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D47" s="11" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D49" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C50" s="5"/>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="B51" t="s">
+        <v>30</v>
+      </c>
+      <c r="D51" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D52" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D53" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D54" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="67" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D67" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C68" s="5"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" display="Container with most water" xr:uid="{F4D67A5D-744F-4C81-957E-33D3253297A2}"/>
+    <hyperlink ref="A20" r:id="rId2" display="Trapping Rain Water" xr:uid="{CDAA1F07-861A-43F8-806E-CBF196F42093}"/>
+    <hyperlink ref="D18" r:id="rId3" xr:uid="{30328AA2-76F9-472A-BAB3-B3B0C7802963}"/>
+    <hyperlink ref="D34" r:id="rId4" xr:uid="{FBB1B328-6337-43BB-960F-5B6CAE89E813}"/>
+    <hyperlink ref="A36" r:id="rId5" display="Largest Rectangle in Histogram" xr:uid="{33CB1418-814A-466E-8725-5800B98469F7}"/>
+    <hyperlink ref="D49" r:id="rId6" xr:uid="{6329D858-D8F3-4698-AF57-250A8ABB78A2}"/>
+    <hyperlink ref="A51" r:id="rId7" display="Maximal Rectangle" xr:uid="{C5538507-5156-4F6A-800E-694A86C1DE83}"/>
+    <hyperlink ref="D67" r:id="rId8" xr:uid="{A272D98F-93C2-491D-BEBC-54FFA0BBC858}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId9"/>
+  <drawing r:id="rId10"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
FindKClosestElements - Feb 23 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72C5F417-EF5E-41BC-9259-0378C505FA68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDD15B88-6F2F-47B7-B6D6-02CEED7C86A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="13" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="14" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -25,8 +25,9 @@
     <sheet name="Low level design" sheetId="11" r:id="rId10"/>
     <sheet name="Graph" sheetId="12" r:id="rId11"/>
     <sheet name="Dictionary" sheetId="13" r:id="rId12"/>
-    <sheet name="template" sheetId="2" r:id="rId13"/>
-    <sheet name="Sorting Algorithms" sheetId="15" r:id="rId14"/>
+    <sheet name="Sorting Algorithms" sheetId="15" r:id="rId13"/>
+    <sheet name="template" sheetId="2" r:id="rId14"/>
+    <sheet name="Binary search" sheetId="16" r:id="rId15"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="237">
   <si>
     <t>Statement</t>
   </si>
@@ -784,6 +785,24 @@
   </si>
   <si>
     <t>do quick select until newK is pivot</t>
+  </si>
+  <si>
+    <t>658. Find K Closest Elements</t>
+  </si>
+  <si>
+    <t>binary search and find index that has min difference with given value</t>
+  </si>
+  <si>
+    <t>then find left and right range from array to copy</t>
+  </si>
+  <si>
+    <t>copy array from found range</t>
+  </si>
+  <si>
+    <t>Try finding left index for best window possible</t>
+  </si>
+  <si>
+    <t>don’t use Math.abs while comparing</t>
   </si>
 </sst>
 </file>
@@ -1464,6 +1483,55 @@
         <a:xfrm>
           <a:off x="3743325" y="466725"/>
           <a:ext cx="2486372" cy="600159"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>847725</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3600834</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>142945</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{96852D08-DDF7-4290-8E9F-2D7EB6390BEE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3667125" y="590550"/>
+          <a:ext cx="2753109" cy="504895"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3319,6 +3387,99 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0397D5EA-9127-4F39-A242-D8D4A93871ED}">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="2" max="2" width="73.85546875" customWidth="1"/>
+    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="D3" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D4" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D6" s="8"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D8" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D10" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D12" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C13" s="5"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A4" r:id="rId1" xr:uid="{CBB80B45-9FC6-4C3A-BE11-6373B320529E}"/>
+    <hyperlink ref="A3" r:id="rId2" xr:uid="{1B705FA7-8F6C-4A90-88DF-06E322C116EF}"/>
+    <hyperlink ref="D12" r:id="rId3" xr:uid="{87407450-9806-4982-AA5D-2AE0CB10FC73}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId4"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10429FF1-7DBA-415E-968E-9D236B8DC32D}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3353,9 +3514,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0397D5EA-9127-4F39-A242-D8D4A93871ED}">
-  <dimension ref="A1:D13"/>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC70315-55E0-46CA-8156-25A8AD92E211}">
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -3385,23 +3546,20 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="D3" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>222</v>
-      </c>
       <c r="D4" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -3409,40 +3567,29 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D9" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D10" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D12" s="2" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D11" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C13" s="5"/>
+    <row r="12" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C12" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A4" r:id="rId1" xr:uid="{CBB80B45-9FC6-4C3A-BE11-6373B320529E}"/>
-    <hyperlink ref="A3" r:id="rId2" xr:uid="{1B705FA7-8F6C-4A90-88DF-06E322C116EF}"/>
-    <hyperlink ref="D12" r:id="rId3" xr:uid="{87407450-9806-4982-AA5D-2AE0CB10FC73}"/>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{D15C5DE0-706A-4DBB-8F74-06E5036954E1}"/>
+    <hyperlink ref="D11" r:id="rId2" xr:uid="{78DAAF07-C11E-4A2F-B6D7-95F5F0D44DB8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId4"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
AlienDictionary - Feb 26 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDD15B88-6F2F-47B7-B6D6-02CEED7C86A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79ED6BC8-B355-425E-897A-6096529B1AF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="14" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="11" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="245">
   <si>
     <t>Statement</t>
   </si>
@@ -804,12 +804,36 @@
   <si>
     <t>don’t use Math.abs while comparing</t>
   </si>
+  <si>
+    <t>265. Alien Dictionary</t>
+  </si>
+  <si>
+    <t>incomplete</t>
+  </si>
+  <si>
+    <t>premium</t>
+  </si>
+  <si>
+    <t>892 · Alien Dictionary - Lintcode</t>
+  </si>
+  <si>
+    <t>create adj set</t>
+  </si>
+  <si>
+    <t>do dfs on keySet of adj</t>
+  </si>
+  <si>
+    <t>make sure to back track visited chars</t>
+  </si>
+  <si>
+    <t>add char to StringBuilder and finally reverse it</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -895,8 +919,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -923,8 +955,13 @@
         <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -947,8 +984,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="7">
+  <cellStyleXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
@@ -956,8 +1008,9 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3"/>
@@ -972,10 +1025,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="6"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="2" xfId="7"/>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="8">
     <cellStyle name="Bad" xfId="5" builtinId="27"/>
     <cellStyle name="Calculation" xfId="2" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="7" builtinId="23"/>
     <cellStyle name="Explanatory Text" xfId="6" builtinId="53"/>
     <cellStyle name="Good" xfId="1" builtinId="26"/>
     <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
@@ -1434,6 +1489,50 @@
         <a:xfrm>
           <a:off x="2867025" y="590550"/>
           <a:ext cx="4848225" cy="400106"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>723900</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4134326</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>76449</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4E7C6E2B-D536-47D3-88B6-8028AC6B6A3A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3543300" y="1571625"/>
+          <a:ext cx="3410426" cy="1781424"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3327,7 +3426,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{170CF2C0-E5DC-4FCA-8D73-E7E5C7297110}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -3373,16 +3472,60 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" s="4" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C7" s="5"/>
+    </row>
+    <row r="8" spans="1:4" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="12" t="s">
+        <v>237</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="D8" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="D9" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D10" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D11" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="17" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D17" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C19" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" xr:uid="{F701FCD9-E8B1-4408-A945-690189F730C8}"/>
     <hyperlink ref="D6" r:id="rId2" xr:uid="{E3A37132-9B1F-4936-A0FA-8D44020D3DD2}"/>
+    <hyperlink ref="A8" r:id="rId3" xr:uid="{B129EF4E-1CD6-4BAF-A906-93595E1759FD}"/>
+    <hyperlink ref="A9" r:id="rId4" display="892 · Alien Dictionary" xr:uid="{5F66370E-D1B4-4C8A-9548-539C76AC4C9E}"/>
+    <hyperlink ref="D17" r:id="rId5" xr:uid="{D5E2F6F0-5D26-4A69-B165-B451444EDDC1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId3"/>
+  <pageSetup orientation="portrait" r:id="rId6"/>
+  <drawing r:id="rId7"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
circular queue design - Feb 28 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79ED6BC8-B355-425E-897A-6096529B1AF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{493EC270-8479-4DE0-A613-66FDB6BDFD17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="11" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="9" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="251">
   <si>
     <t>Statement</t>
   </si>
@@ -827,6 +827,24 @@
   </si>
   <si>
     <t>add char to StringBuilder and finally reverse it</t>
+  </si>
+  <si>
+    <t>622. Design Circular Queue</t>
+  </si>
+  <si>
+    <t>use an array</t>
+  </si>
+  <si>
+    <t>init front = 0, rear = -1</t>
+  </si>
+  <si>
+    <t>change front/rear to ++rear % maxSize/--front % maxSize before enqueue or deQueue</t>
+  </si>
+  <si>
+    <t>check if size is full or empty befor doing above operations</t>
+  </si>
+  <si>
+    <t>soution</t>
   </si>
 </sst>
 </file>
@@ -2727,6 +2745,50 @@
         <a:xfrm>
           <a:off x="2876550" y="2114550"/>
           <a:ext cx="4819650" cy="1086002"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>47626</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4905376</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>123999</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0DC5E8BC-C6E7-442E-88B2-47BABB480DDA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2867026" y="3638550"/>
+          <a:ext cx="4857750" cy="1247949"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3104,7 +3166,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7BE8B5F-B3C3-43A1-BD9C-D35CE748D483}">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -3156,13 +3218,44 @@
         <v>159</v>
       </c>
     </row>
-    <row r="17" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D17" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C18" s="5"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="D19" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D20" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D21" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D22" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D26" s="2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C27" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3170,9 +3263,11 @@
     <hyperlink ref="D9" r:id="rId2" xr:uid="{60C7CCA8-6DFD-471B-BE7B-FBA6AA3D39EF}"/>
     <hyperlink ref="A11" r:id="rId3" xr:uid="{B613807D-978E-4CA0-928A-B9CD9644C8F6}"/>
     <hyperlink ref="D17" r:id="rId4" xr:uid="{6226ADC2-6F8E-4914-A1E9-DA822FBF2A00}"/>
+    <hyperlink ref="A19" r:id="rId5" xr:uid="{1C07BF01-9F0C-4351-A36A-823B3D1421E1}"/>
+    <hyperlink ref="D26" r:id="rId6" xr:uid="{DD2E06CD-E5AB-4B10-B597-A62BC91B4CE4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId5"/>
+  <drawing r:id="rId7"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
openLock - Mar 01 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{493EC270-8479-4DE0-A613-66FDB6BDFD17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F34270FA-6AB2-447B-9C03-7DFEBB150E68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="9" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="3" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="255">
   <si>
     <t>Statement</t>
   </si>
@@ -845,6 +845,18 @@
   </si>
   <si>
     <t>soution</t>
+  </si>
+  <si>
+    <t>752. Open the Lock</t>
+  </si>
+  <si>
+    <t>BFS</t>
+  </si>
+  <si>
+    <t>put each up and down combinations for current batch into queue</t>
+  </si>
+  <si>
+    <t>and cnt++</t>
   </si>
 </sst>
 </file>
@@ -1791,6 +1803,50 @@
         <a:xfrm>
           <a:off x="3467100" y="590550"/>
           <a:ext cx="3200847" cy="2267266"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4905375</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>104943</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{10070385-CBBB-4997-A789-94A71BE50875}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2847975" y="3286125"/>
+          <a:ext cx="4876800" cy="1200318"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4090,7 +4146,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51C4CDD9-9363-46B2-A2D8-BE11DE99714D}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -4159,13 +4215,41 @@
     <row r="16" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C16" s="5"/>
     </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="D17" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D18" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D19" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D24" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C25" s="5"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" xr:uid="{939F716F-C15C-4A88-A6E5-FB3DE8101485}"/>
     <hyperlink ref="D15" r:id="rId2" xr:uid="{8A4FF2B5-4B6B-44D6-AA37-2257F9852D45}"/>
+    <hyperlink ref="A17" r:id="rId3" xr:uid="{528F5FE6-1479-40BB-A002-8A1E7211AB8C}"/>
+    <hyperlink ref="D24" r:id="rId4" xr:uid="{DE2913A7-D3DA-46B3-83F9-C18D6E3ED24C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId3"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
SplittingaStringIntoDescendingConsecutiveValues - 2nd Mar 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F34270FA-6AB2-447B-9C03-7DFEBB150E68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87C26168-BA2D-4519-AFBA-A193BF0B2981}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="3" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="14" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -25,9 +25,10 @@
     <sheet name="Low level design" sheetId="11" r:id="rId10"/>
     <sheet name="Graph" sheetId="12" r:id="rId11"/>
     <sheet name="Dictionary" sheetId="13" r:id="rId12"/>
-    <sheet name="Sorting Algorithms" sheetId="15" r:id="rId13"/>
-    <sheet name="template" sheetId="2" r:id="rId14"/>
-    <sheet name="Binary search" sheetId="16" r:id="rId15"/>
+    <sheet name="template" sheetId="2" r:id="rId13"/>
+    <sheet name="dfs" sheetId="17" r:id="rId14"/>
+    <sheet name="Sorting Algorithms" sheetId="15" r:id="rId15"/>
+    <sheet name="Binary search" sheetId="16" r:id="rId16"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="260">
   <si>
     <t>Statement</t>
   </si>
@@ -324,25 +325,13 @@
     <t xml:space="preserve">similarly one finishes right </t>
   </si>
   <si>
-    <t>&gt; don't return till n.logn</t>
-  </si>
-  <si>
     <t>Initialize 2 pointers i,j for 2 arrays</t>
   </si>
   <si>
     <t>&gt; move until i+j reach sum/2</t>
   </si>
   <si>
-    <t>&gt; while moving save if i==n increment j, or if j==m i++ th element to current</t>
-  </si>
-  <si>
     <t>&gt; store prev element all the time</t>
-  </si>
-  <si>
-    <t>if sum is odd return current, else avg of prev and current</t>
-  </si>
-  <si>
-    <t>2nd</t>
   </si>
   <si>
     <t>If we have k elements in combined array</t>
@@ -857,6 +846,33 @@
   </si>
   <si>
     <t>and cnt++</t>
+  </si>
+  <si>
+    <t>&gt; don't return till n.logn - i.e. iterate even if u get first element</t>
+  </si>
+  <si>
+    <t>if sum is odd return current, else avg of prev and current typecasted to float</t>
+  </si>
+  <si>
+    <t>&gt; while moving save if i==n j++, or if j==m i++ th element to current, else compare &amp; ++ the smaller one</t>
+  </si>
+  <si>
+    <t>&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;</t>
+  </si>
+  <si>
+    <t>1849. Splitting a String Into Descending Consecutive Values</t>
+  </si>
+  <si>
+    <t>call dfs after each first value</t>
+  </si>
+  <si>
+    <t>In dfs function : iterate over each combination and call dfs if value of current long is less by 1</t>
+  </si>
+  <si>
+    <t>&gt; current = Long.parseLong(s.subString(l, r)) will give exception</t>
+  </si>
+  <si>
+    <t>&gt; so use current = current * 10 + (s.charAt(r) - '0')</t>
   </si>
 </sst>
 </file>
@@ -1579,6 +1595,55 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
+      <xdr:colOff>85725</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4629150</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>28922</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A8D9FA0A-94B1-4965-855B-B142A80B4A8B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3600450" y="590550"/>
+          <a:ext cx="4543425" cy="2486372"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>923925</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>85725</xdr:rowOff>
@@ -1623,7 +1688,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing14.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -3252,10 +3317,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="D3" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -3268,10 +3333,10 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="D11" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -3284,30 +3349,30 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="D19" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D20" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D21" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D26" s="2" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
     </row>
     <row r="27" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3359,10 +3424,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="6" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3370,30 +3435,30 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="D7" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D9" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -3406,20 +3471,20 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D24" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D25" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D26" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -3432,28 +3497,28 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="8" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="D44" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D45" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="D46" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D47" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -3466,20 +3531,20 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="D51" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D52" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D53" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
     </row>
     <row r="70" spans="4:4" x14ac:dyDescent="0.25">
@@ -3492,35 +3557,35 @@
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="8" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="D87" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D88" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D89" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D90" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D91" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D92" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
@@ -3533,15 +3598,15 @@
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="8" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="D97" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D98" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
@@ -3607,15 +3672,15 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="D3" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -3628,34 +3693,34 @@
     </row>
     <row r="8" spans="1:4" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
+        <v>233</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="D8" t="s">
         <v>237</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="D8" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="D9" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
     </row>
     <row r="17" spans="3:4" x14ac:dyDescent="0.25">
@@ -3681,6 +3746,112 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10429FF1-7DBA-415E-968E-9D236B8DC32D}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="2" max="2" width="73.85546875" customWidth="1"/>
+    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E9C6576-B939-40FE-9164-B9EF7525065D}">
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="52.7109375" customWidth="1"/>
+    <col min="2" max="2" width="70.28515625" customWidth="1"/>
+    <col min="3" max="3" width="33.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="D3" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D6" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D16" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="3:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C17" s="5"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{FA9D13DB-E1B4-4F9E-8A08-75017F0A9267}"/>
+    <hyperlink ref="D16" r:id="rId2" xr:uid="{7DB504AE-B17D-4007-9242-6FFA0122E7AC}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0397D5EA-9127-4F39-A242-D8D4A93871ED}">
   <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3712,23 +3883,23 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="D3" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="D4" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -3736,22 +3907,22 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D9" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -3773,42 +3944,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10429FF1-7DBA-415E-968E-9D236B8DC32D}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="42.28515625" customWidth="1"/>
-    <col min="2" max="2" width="73.85546875" customWidth="1"/>
-    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="91.7109375" customWidth="1"/>
-    <col min="13" max="13" width="6.7109375" customWidth="1"/>
-    <col min="14" max="14" width="8.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C2" s="5"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC70315-55E0-46CA-8156-25A8AD92E211}">
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3840,20 +3976,20 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="D3" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -3861,12 +3997,12 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -3919,25 +4055,25 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="D3" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -3950,35 +4086,35 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="D11" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D12" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D13" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D14" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D15" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D16" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -3991,25 +4127,25 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="D20" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D21" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D23" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -4066,25 +4202,25 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -4097,31 +4233,31 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="D13" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C14" s="1" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="D14" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D15" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D16" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
     </row>
     <row r="18" spans="3:4" x14ac:dyDescent="0.25">
@@ -4176,35 +4312,35 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="D3" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -4217,20 +4353,20 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D17" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D18" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D19" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -4285,20 +4421,20 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D3" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -4311,25 +4447,25 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D9" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D12" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -4342,30 +4478,30 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D18" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D19" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D20" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D21" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -4422,7 +4558,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="D3" t="s">
         <v>90</v>
@@ -4435,7 +4571,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>92</v>
+        <v>251</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -4448,60 +4584,60 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D12" t="s">
-        <v>95</v>
+        <v>253</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D13" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D14" t="s">
-        <v>97</v>
+        <v>252</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D16" t="s">
-        <v>98</v>
+        <v>254</v>
       </c>
     </row>
     <row r="17" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D17" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
     </row>
     <row r="18" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D18" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="19" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C19" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="D19" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
     </row>
     <row r="20" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D20" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="21" spans="3:4" x14ac:dyDescent="0.25">
@@ -4556,25 +4692,25 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="D3" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -4587,15 +4723,15 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="D21" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -4608,25 +4744,25 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="D31" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D32" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
     </row>
     <row r="33" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D33" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
     </row>
     <row r="34" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D34" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="43" spans="3:4" x14ac:dyDescent="0.25">
@@ -4683,7 +4819,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="D3" t="s">
         <v>45</v>
@@ -4714,7 +4850,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B17" t="s">
         <v>38</v>
@@ -4805,7 +4941,7 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D36" t="s">
         <v>55</v>
@@ -4851,7 +4987,7 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D49" t="s">
         <v>62</v>
@@ -4893,7 +5029,7 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="D61" s="7" t="s">
         <v>44</v>
@@ -4942,7 +5078,7 @@
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="8" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C77" s="1" t="s">
         <v>80</v>
@@ -4992,7 +5128,7 @@
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="8" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="D87" t="s">
         <v>83</v>
@@ -5096,7 +5232,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
@@ -5136,7 +5272,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B20" t="s">
         <v>8</v>
@@ -5205,7 +5341,7 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D36" t="s">
         <v>23</v>
@@ -5213,22 +5349,22 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D37" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D38" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D39" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D40" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -5274,7 +5410,7 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="9" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="B51" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
sorting algorithms - Mar 6th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87C26168-BA2D-4519-AFBA-A193BF0B2981}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEEA7A9A-11CA-42AF-87F6-74A041205046}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="14" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="4" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="273">
   <si>
     <t>Statement</t>
   </si>
@@ -873,6 +873,45 @@
   </si>
   <si>
     <t>&gt; so use current = current * 10 + (s.charAt(r) - '0')</t>
+  </si>
+  <si>
+    <t>289. Game of Life</t>
+  </si>
+  <si>
+    <t>count live neighbors</t>
+  </si>
+  <si>
+    <t>just temporarily map 00-&gt;0, 10-&gt;1, 01-&gt;2, 11-&gt;3</t>
+  </si>
+  <si>
+    <t>198. House Robber</t>
+  </si>
+  <si>
+    <t>i = i + max(i-2, i-3)</t>
+  </si>
+  <si>
+    <t>currMax = max(i+rob1, rob2)</t>
+  </si>
+  <si>
+    <t>494. Target Sum</t>
+  </si>
+  <si>
+    <t>use index and currentSum as key</t>
+  </si>
+  <si>
+    <t>endcase = if index reach end of nums , if sum == target return 1 else 0</t>
+  </si>
+  <si>
+    <t>call dfs for index+1 by 1) adding current num 2) subtracting current num</t>
+  </si>
+  <si>
+    <t>70. Climbing Stairs</t>
+  </si>
+  <si>
+    <t>if n==1 or n==2 return n</t>
+  </si>
+  <si>
+    <t>else return dfs(n-1)+dfs(n-2)</t>
   </si>
 </sst>
 </file>
@@ -2057,6 +2096,138 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4867946</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>133470</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{237B0BA2-D7DB-4329-BDC1-58D9AF75069F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2876550" y="6324600"/>
+          <a:ext cx="4810796" cy="857370"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4886325</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>152629</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{21779FD1-0DD5-44AB-AC5A-B7BF6AF15F26}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2867025" y="7658100"/>
+          <a:ext cx="4838700" cy="1638529"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>590550</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4267713</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>66813</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F6F69E29-9686-4BAA-937D-9A341EB14077}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3409950" y="9744075"/>
+          <a:ext cx="3677163" cy="990738"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2279,6 +2450,50 @@
         <a:xfrm>
           <a:off x="3267075" y="5953125"/>
           <a:ext cx="4086795" cy="2534004"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>85725</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4914900</xdr:colOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>162716</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DACB0E49-FE94-4E2D-BC99-C5ACB0B17F3A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2905125" y="8972550"/>
+          <a:ext cx="4829175" cy="5668166"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4391,7 +4606,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -4512,6 +4727,87 @@
     <row r="32" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C32" s="5"/>
     </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="D33" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D34" s="4"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D35" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D38" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C39" s="5"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="D40" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D41" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D42" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D43" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D49" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C50" s="5"/>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="D51" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D52" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D53" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D56" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C58" s="5"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D16" r:id="rId1" xr:uid="{9286C815-A01C-4238-8F25-586F52E5AFCB}"/>
@@ -4519,10 +4815,16 @@
     <hyperlink ref="D31" r:id="rId3" xr:uid="{CB3B5519-6706-4D91-8ED8-B03622537410}"/>
     <hyperlink ref="A3" r:id="rId4" xr:uid="{BBBEC409-91C1-4247-A04A-0D6745237535}"/>
     <hyperlink ref="A9" r:id="rId5" xr:uid="{8657ECCA-D251-4695-9C7A-63DC0476CAED}"/>
+    <hyperlink ref="A33" r:id="rId6" xr:uid="{F736A361-9C09-42E1-AF14-5F43CBB90345}"/>
+    <hyperlink ref="D38" r:id="rId7" xr:uid="{9403F647-BC63-4576-B6D3-DB4EA4516551}"/>
+    <hyperlink ref="A40" r:id="rId8" xr:uid="{27D42C47-BEEA-4D5B-8976-5CE03CE33F58}"/>
+    <hyperlink ref="D49" r:id="rId9" xr:uid="{21155A71-595E-45BE-AB49-00633373E3B6}"/>
+    <hyperlink ref="A51" r:id="rId10" xr:uid="{96ACD755-849B-4666-A201-DBBCD536D0D8}"/>
+    <hyperlink ref="D56" r:id="rId11" xr:uid="{721907C8-B3FE-4468-BB59-DC7D65817E15}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId6"/>
-  <drawing r:id="rId7"/>
+  <pageSetup orientation="portrait" r:id="rId12"/>
+  <drawing r:id="rId13"/>
 </worksheet>
 </file>
 
@@ -4662,7 +4964,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83AD0EA2-442A-436B-AA00-D0DF9DB7227A}">
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D78"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -4755,23 +5057,44 @@
         <v>205</v>
       </c>
     </row>
-    <row r="33" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D33" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="34" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D34" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="43" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D43" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="46" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C46" s="5"/>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="D47" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D48" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="77" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D77" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C78" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -4781,9 +5104,12 @@
     <hyperlink ref="D29" r:id="rId4" xr:uid="{AE068BF9-E00D-4A52-912C-FAF893DCE140}"/>
     <hyperlink ref="A31" r:id="rId5" xr:uid="{E38CCC9C-9408-4335-8A45-68FC60A3701A}"/>
     <hyperlink ref="D43" r:id="rId6" xr:uid="{60E813ED-AC35-4B86-9781-5B80FA133723}"/>
+    <hyperlink ref="A47" r:id="rId7" xr:uid="{B9C0BE08-1E7F-4552-9904-54253A2CA85D}"/>
+    <hyperlink ref="D77" r:id="rId8" xr:uid="{32267523-470D-47CA-8715-C3AB3030E922}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId7"/>
+  <pageSetup orientation="portrait" r:id="rId9"/>
+  <drawing r:id="rId10"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
dp - Mar 6th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,27 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEEA7A9A-11CA-42AF-87F6-74A041205046}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B76D2933-2DAA-45CF-A563-8F32758AA0E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="4" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" activeTab="15" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
     <sheet name="Parenthesis" sheetId="7" r:id="rId2"/>
     <sheet name="Stack" sheetId="8" r:id="rId3"/>
     <sheet name="Queue" sheetId="9" r:id="rId4"/>
-    <sheet name="dp" sheetId="6" r:id="rId5"/>
-    <sheet name="Array" sheetId="4" r:id="rId6"/>
-    <sheet name="Matrix" sheetId="5" r:id="rId7"/>
-    <sheet name="Linked list" sheetId="3" r:id="rId8"/>
-    <sheet name="Rain water trap" sheetId="1" r:id="rId9"/>
-    <sheet name="Low level design" sheetId="11" r:id="rId10"/>
-    <sheet name="Graph" sheetId="12" r:id="rId11"/>
-    <sheet name="Dictionary" sheetId="13" r:id="rId12"/>
-    <sheet name="template" sheetId="2" r:id="rId13"/>
-    <sheet name="dfs" sheetId="17" r:id="rId14"/>
-    <sheet name="Sorting Algorithms" sheetId="15" r:id="rId15"/>
-    <sheet name="Binary search" sheetId="16" r:id="rId16"/>
+    <sheet name="Array" sheetId="4" r:id="rId5"/>
+    <sheet name="Matrix" sheetId="5" r:id="rId6"/>
+    <sheet name="Linked list" sheetId="3" r:id="rId7"/>
+    <sheet name="Rain water trap" sheetId="1" r:id="rId8"/>
+    <sheet name="Low level design" sheetId="11" r:id="rId9"/>
+    <sheet name="Graph" sheetId="12" r:id="rId10"/>
+    <sheet name="Dictionary" sheetId="13" r:id="rId11"/>
+    <sheet name="template" sheetId="2" r:id="rId12"/>
+    <sheet name="dfs" sheetId="17" r:id="rId13"/>
+    <sheet name="Sorting Algorithms" sheetId="15" r:id="rId14"/>
+    <sheet name="Binary search" sheetId="16" r:id="rId15"/>
+    <sheet name="dp" sheetId="6" r:id="rId16"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="277">
   <si>
     <t>Statement</t>
   </si>
@@ -912,6 +912,18 @@
   </si>
   <si>
     <t>else return dfs(n-1)+dfs(n-2)</t>
+  </si>
+  <si>
+    <t>983. Minimum Cost For Tickets</t>
+  </si>
+  <si>
+    <t>For 1, 7, 30 days</t>
+  </si>
+  <si>
+    <t>for a given pass - travel through max days possible and call dfs for newIndex</t>
+  </si>
+  <si>
+    <t>for each day try all 3 passes &amp; return min money required using any pass to reach final index</t>
   </si>
 </sst>
 </file>
@@ -1272,275 +1284,6 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>533400</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>4458248</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>171840</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C8BF61F0-8C11-4999-AFCC-E8237884BC76}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3352800" y="1381125"/>
-          <a:ext cx="3924848" cy="2791215"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>695325</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>4210541</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>105234</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6E3CCC62-444B-4F0A-AA4F-63EE120A8F8F}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3514725" y="4629150"/>
-          <a:ext cx="3515216" cy="3286584"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>180975</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>4801245</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>19131</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5C7BFA47-99A5-4DD4-A65C-538204B1AA00}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3000375" y="8391525"/>
-          <a:ext cx="4620270" cy="581106"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>142875</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>4819650</xdr:colOff>
-      <xdr:row>84</xdr:row>
-      <xdr:rowOff>115191</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5C8B32F2-4113-49E3-BBD5-96C105B8A12A}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2962275" y="9734550"/>
-          <a:ext cx="4676775" cy="6382641"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>87</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>4896528</xdr:colOff>
-      <xdr:row>91</xdr:row>
-      <xdr:rowOff>95364</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Picture 5">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{419BD70B-D29F-47D2-98A4-795635A21345}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2857500" y="16611600"/>
-          <a:ext cx="4858428" cy="819264"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>19051</xdr:colOff>
-      <xdr:row>97</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>4895851</xdr:colOff>
-      <xdr:row>111</xdr:row>
-      <xdr:rowOff>181371</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Picture 6">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DCA87E4E-91D5-41F2-AA12-C5D1F1A1C95A}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2838451" y="18488025"/>
-          <a:ext cx="4876800" cy="2838846"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
       <xdr:colOff>47625</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
@@ -1629,7 +1372,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1678,7 +1421,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1727,7 +1470,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1765,6 +1508,319 @@
         <a:xfrm>
           <a:off x="3667125" y="590550"/>
           <a:ext cx="2753109" cy="504895"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing14.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>47626</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4886326</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>133444</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EBF1B06A-14A7-4378-B685-42F84E591CCF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2867026" y="600075"/>
+          <a:ext cx="4838700" cy="676369"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>895350</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3743723</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>183</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A7977868-6FED-4F2A-BB51-24589D1230A5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3714750" y="1733550"/>
+          <a:ext cx="2848373" cy="1314633"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4829175</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>105127</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{85D88232-4D10-43ED-BCE0-A7346AFF16BB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2857500" y="3486150"/>
+          <a:ext cx="4791075" cy="2524477"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4867946</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>133470</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{237B0BA2-D7DB-4329-BDC1-58D9AF75069F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2876550" y="6324600"/>
+          <a:ext cx="4810796" cy="857370"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4886325</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>152629</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{21779FD1-0DD5-44AB-AC5A-B7BF6AF15F26}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2867025" y="7658100"/>
+          <a:ext cx="4838700" cy="1638529"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>590550</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4267713</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>66813</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F6F69E29-9686-4BAA-937D-9A341EB14077}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3409950" y="9744075"/>
+          <a:ext cx="3677163" cy="990738"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4895850</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>95445</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5256F350-38B3-4EAD-A551-BFD88D1E9502}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2838450" y="11268075"/>
+          <a:ext cx="4876800" cy="1400370"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1967,275 +2023,6 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>47626</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>4886326</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>133444</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EBF1B06A-14A7-4378-B685-42F84E591CCF}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2867026" y="600075"/>
-          <a:ext cx="4838700" cy="676369"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>895350</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>3743723</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>183</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A7977868-6FED-4F2A-BB51-24589D1230A5}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3714750" y="1733550"/>
-          <a:ext cx="2848373" cy="1314633"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>4829175</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>105127</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{85D88232-4D10-43ED-BCE0-A7346AFF16BB}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2857500" y="3486150"/>
-          <a:ext cx="4791075" cy="2524477"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>57150</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>4867946</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>133470</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{237B0BA2-D7DB-4329-BDC1-58D9AF75069F}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2876550" y="6324600"/>
-          <a:ext cx="4810796" cy="857370"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>47625</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>4886325</xdr:colOff>
-      <xdr:row>48</xdr:row>
-      <xdr:rowOff>152629</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Picture 5">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{21779FD1-0DD5-44AB-AC5A-B7BF6AF15F26}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2867025" y="7658100"/>
-          <a:ext cx="4838700" cy="1638529"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>590550</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>4267713</xdr:colOff>
-      <xdr:row>56</xdr:row>
-      <xdr:rowOff>66813</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Picture 6">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F6F69E29-9686-4BAA-937D-9A341EB14077}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3409950" y="9744075"/>
-          <a:ext cx="3677163" cy="990738"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
       <xdr:colOff>657225</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
@@ -2324,7 +2111,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -2505,7 +2292,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -2818,7 +2605,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -2999,7 +2786,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -3125,6 +2912,275 @@
         <a:xfrm>
           <a:off x="2867026" y="3638550"/>
           <a:ext cx="4857750" cy="1247949"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>533400</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4458248</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>171840</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C8BF61F0-8C11-4999-AFCC-E8237884BC76}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3352800" y="1381125"/>
+          <a:ext cx="3924848" cy="2791215"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>695325</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4210541</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>105234</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6E3CCC62-444B-4F0A-AA4F-63EE120A8F8F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3514725" y="4629150"/>
+          <a:ext cx="3515216" cy="3286584"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>180975</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4801245</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>19131</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5C7BFA47-99A5-4DD4-A65C-538204B1AA00}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3000375" y="8391525"/>
+          <a:ext cx="4620270" cy="581106"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>142875</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4819650</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>115191</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5C8B32F2-4113-49E3-BBD5-96C105B8A12A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2962275" y="9734550"/>
+          <a:ext cx="4676775" cy="6382641"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>87</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4896528</xdr:colOff>
+      <xdr:row>91</xdr:row>
+      <xdr:rowOff>95364</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{419BD70B-D29F-47D2-98A4-795635A21345}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2857500" y="16611600"/>
+          <a:ext cx="4858428" cy="819264"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>19051</xdr:colOff>
+      <xdr:row>97</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4895851</xdr:colOff>
+      <xdr:row>111</xdr:row>
+      <xdr:rowOff>181371</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DCA87E4E-91D5-41F2-AA12-C5D1F1A1C95A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2838451" y="18488025"/>
+          <a:ext cx="4876800" cy="2838846"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3501,113 +3557,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7BE8B5F-B3C3-43A1-BD9C-D35CE748D483}">
-  <dimension ref="A1:D27"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="42.28515625" customWidth="1"/>
-    <col min="2" max="2" width="73.85546875" customWidth="1"/>
-    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="91.7109375" customWidth="1"/>
-    <col min="13" max="13" width="6.7109375" customWidth="1"/>
-    <col min="14" max="14" width="8.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C2" s="5"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="D3" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D9" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C10" s="5"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="D11" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D17" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C18" s="5"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
-        <v>241</v>
-      </c>
-      <c r="D19" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D20" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D21" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D22" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D26" s="2" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C27" s="5"/>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" xr:uid="{976A6329-CE7B-45FA-9EC8-39B157036788}"/>
-    <hyperlink ref="D9" r:id="rId2" xr:uid="{60C7CCA8-6DFD-471B-BE7B-FBA6AA3D39EF}"/>
-    <hyperlink ref="A11" r:id="rId3" xr:uid="{B613807D-978E-4CA0-928A-B9CD9644C8F6}"/>
-    <hyperlink ref="D17" r:id="rId4" xr:uid="{6226ADC2-6F8E-4914-A1E9-DA822FBF2A00}"/>
-    <hyperlink ref="A19" r:id="rId5" xr:uid="{1C07BF01-9F0C-4351-A36A-823B3D1421E1}"/>
-    <hyperlink ref="D26" r:id="rId6" xr:uid="{DD2E06CD-E5AB-4B10-B597-A62BC91B4CE4}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId7"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E87A3A0-D815-41F9-954B-826D58641E2B}">
   <dimension ref="A1:D113"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3855,7 +3804,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{170CF2C0-E5DC-4FCA-8D73-E7E5C7297110}">
   <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3960,7 +3909,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10429FF1-7DBA-415E-968E-9D236B8DC32D}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3995,7 +3944,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E9C6576-B939-40FE-9164-B9EF7525065D}">
   <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4066,7 +4015,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0397D5EA-9127-4F39-A242-D8D4A93871ED}">
   <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4159,7 +4108,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC70315-55E0-46CA-8156-25A8AD92E211}">
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4235,6 +4184,261 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
+  <dimension ref="A1:D68"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="2" max="2" width="73.85546875" customWidth="1"/>
+    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="D3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D7" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C8" s="5"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="D9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D10" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D11" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D12" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D16" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C17" s="5"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="D18" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D19" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D20" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D21" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D22" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D31" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C32" s="5"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="D33" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D34" s="4"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D35" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D38" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C39" s="5"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="D40" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D41" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D42" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D43" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D49" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C50" s="5"/>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="D51" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D52" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D53" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D56" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C58" s="5"/>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="D59" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C60" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="D60" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D61" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="67" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D67" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C68" s="5"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D16" r:id="rId1" xr:uid="{9286C815-A01C-4238-8F25-586F52E5AFCB}"/>
+    <hyperlink ref="A18" r:id="rId2" xr:uid="{E118E9A3-7847-445D-B795-52CF7974AD4F}"/>
+    <hyperlink ref="D31" r:id="rId3" xr:uid="{CB3B5519-6706-4D91-8ED8-B03622537410}"/>
+    <hyperlink ref="A3" r:id="rId4" xr:uid="{BBBEC409-91C1-4247-A04A-0D6745237535}"/>
+    <hyperlink ref="A9" r:id="rId5" xr:uid="{8657ECCA-D251-4695-9C7A-63DC0476CAED}"/>
+    <hyperlink ref="A33" r:id="rId6" xr:uid="{F736A361-9C09-42E1-AF14-5F43CBB90345}"/>
+    <hyperlink ref="D38" r:id="rId7" xr:uid="{9403F647-BC63-4576-B6D3-DB4EA4516551}"/>
+    <hyperlink ref="A40" r:id="rId8" xr:uid="{27D42C47-BEEA-4D5B-8976-5CE03CE33F58}"/>
+    <hyperlink ref="D49" r:id="rId9" xr:uid="{21155A71-595E-45BE-AB49-00633373E3B6}"/>
+    <hyperlink ref="A51" r:id="rId10" xr:uid="{96ACD755-849B-4666-A201-DBBCD536D0D8}"/>
+    <hyperlink ref="D56" r:id="rId11" xr:uid="{721907C8-B3FE-4468-BB59-DC7D65817E15}"/>
+    <hyperlink ref="A59" r:id="rId12" xr:uid="{BA4760B5-DD05-4193-AC5F-E1DD01C33202}"/>
+    <hyperlink ref="D67" r:id="rId13" xr:uid="{EEF239C6-6D8D-4374-977C-9A3AC3457FD5}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId14"/>
+  <drawing r:id="rId15"/>
 </worksheet>
 </file>
 
@@ -4605,230 +4809,6 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
-  <dimension ref="A1:D58"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="42.28515625" customWidth="1"/>
-    <col min="2" max="2" width="73.85546875" customWidth="1"/>
-    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="91.7109375" customWidth="1"/>
-    <col min="13" max="13" width="6.7109375" customWidth="1"/>
-    <col min="14" max="14" width="8.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C2" s="5"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="D3" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D4" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D5" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C8" s="5"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="D9" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D10" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D11" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D12" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D16" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C17" s="5"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="D18" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D19" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D20" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D21" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D22" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D31" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C32" s="5"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
-        <v>263</v>
-      </c>
-      <c r="D33" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D34" s="4"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D35" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D38" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C39" s="5"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="8" t="s">
-        <v>266</v>
-      </c>
-      <c r="D40" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D41" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D42" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D43" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D49" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C50" s="5"/>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="4" t="s">
-        <v>270</v>
-      </c>
-      <c r="D51" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D52" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D53" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D56" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C58" s="5"/>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D16" r:id="rId1" xr:uid="{9286C815-A01C-4238-8F25-586F52E5AFCB}"/>
-    <hyperlink ref="A18" r:id="rId2" xr:uid="{E118E9A3-7847-445D-B795-52CF7974AD4F}"/>
-    <hyperlink ref="D31" r:id="rId3" xr:uid="{CB3B5519-6706-4D91-8ED8-B03622537410}"/>
-    <hyperlink ref="A3" r:id="rId4" xr:uid="{BBBEC409-91C1-4247-A04A-0D6745237535}"/>
-    <hyperlink ref="A9" r:id="rId5" xr:uid="{8657ECCA-D251-4695-9C7A-63DC0476CAED}"/>
-    <hyperlink ref="A33" r:id="rId6" xr:uid="{F736A361-9C09-42E1-AF14-5F43CBB90345}"/>
-    <hyperlink ref="D38" r:id="rId7" xr:uid="{9403F647-BC63-4576-B6D3-DB4EA4516551}"/>
-    <hyperlink ref="A40" r:id="rId8" xr:uid="{27D42C47-BEEA-4D5B-8976-5CE03CE33F58}"/>
-    <hyperlink ref="D49" r:id="rId9" xr:uid="{21155A71-595E-45BE-AB49-00633373E3B6}"/>
-    <hyperlink ref="A51" r:id="rId10" xr:uid="{96ACD755-849B-4666-A201-DBBCD536D0D8}"/>
-    <hyperlink ref="D56" r:id="rId11" xr:uid="{721907C8-B3FE-4468-BB59-DC7D65817E15}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId12"/>
-  <drawing r:id="rId13"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDA924A8-9114-46BA-B39C-6743F04F80F3}">
   <dimension ref="A1:D22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4962,7 +4942,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83AD0EA2-442A-436B-AA00-D0DF9DB7227A}">
   <dimension ref="A1:D78"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5113,7 +5093,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56E27646-854C-4719-A92C-78F24A8C7C41}">
   <dimension ref="A1:D100"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5526,7 +5506,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CE8EF6C-9017-4EEF-A2CD-F2424B35AA25}">
   <dimension ref="A1:D68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5783,4 +5763,111 @@
   <pageSetup orientation="portrait" r:id="rId9"/>
   <drawing r:id="rId10"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7BE8B5F-B3C3-43A1-BD9C-D35CE748D483}">
+  <dimension ref="A1:D27"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="2" max="2" width="73.85546875" customWidth="1"/>
+    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="D3" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D9" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C10" s="5"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="D11" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D17" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C18" s="5"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="D19" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D20" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D21" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D22" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D26" s="2" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C27" s="5"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{976A6329-CE7B-45FA-9EC8-39B157036788}"/>
+    <hyperlink ref="D9" r:id="rId2" xr:uid="{60C7CCA8-6DFD-471B-BE7B-FBA6AA3D39EF}"/>
+    <hyperlink ref="A11" r:id="rId3" xr:uid="{B613807D-978E-4CA0-928A-B9CD9644C8F6}"/>
+    <hyperlink ref="D17" r:id="rId4" xr:uid="{6226ADC2-6F8E-4914-A1E9-DA822FBF2A00}"/>
+    <hyperlink ref="A19" r:id="rId5" xr:uid="{1C07BF01-9F0C-4351-A36A-823B3D1421E1}"/>
+    <hyperlink ref="D26" r:id="rId6" xr:uid="{DD2E06CD-E5AB-4B10-B597-A62BC91B4CE4}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId7"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
coinChange dp - Mar 12 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B76D2933-2DAA-45CF-A563-8F32758AA0E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F571A8-B218-4DAF-A477-10954C230B2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" activeTab="15" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="282">
   <si>
     <t>Statement</t>
   </si>
@@ -924,6 +924,21 @@
   </si>
   <si>
     <t>for each day try all 3 passes &amp; return min money required using any pass to reach final index</t>
+  </si>
+  <si>
+    <t>322. Coin Change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dfs </t>
+  </si>
+  <si>
+    <t>call dfs using current coin i.e. for the remaining amount</t>
+  </si>
+  <si>
+    <t>518. Coin Change 2</t>
+  </si>
+  <si>
+    <t>dfs as above but keep track of current index to avoid duplicates</t>
   </si>
 </sst>
 </file>
@@ -1821,6 +1836,94 @@
         <a:xfrm>
           <a:off x="2838450" y="11268075"/>
           <a:ext cx="4876800" cy="1400370"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1076325</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3543644</xdr:colOff>
+      <xdr:row>72</xdr:row>
+      <xdr:rowOff>123917</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{11D1165B-1EEC-4415-A416-FE256B0D0835}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3895725" y="13182600"/>
+          <a:ext cx="2467319" cy="657317"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>438150</xdr:colOff>
+      <xdr:row>75</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4267734</xdr:colOff>
+      <xdr:row>82</xdr:row>
+      <xdr:rowOff>95445</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{25E0F410-A54A-4236-82A7-FAD7AA631F32}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3257550" y="14316075"/>
+          <a:ext cx="3829584" cy="1400370"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4189,7 +4292,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
-  <dimension ref="A1:D68"/>
+  <dimension ref="A1:D84"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -4412,13 +4515,50 @@
         <v>275</v>
       </c>
     </row>
-    <row r="67" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D67" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="68" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C68" s="5"/>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="D69" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D70" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D73" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C74" s="5"/>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="D75" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="83" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D83" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C84" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -4435,10 +4575,14 @@
     <hyperlink ref="D56" r:id="rId11" xr:uid="{721907C8-B3FE-4468-BB59-DC7D65817E15}"/>
     <hyperlink ref="A59" r:id="rId12" xr:uid="{BA4760B5-DD05-4193-AC5F-E1DD01C33202}"/>
     <hyperlink ref="D67" r:id="rId13" xr:uid="{EEF239C6-6D8D-4374-977C-9A3AC3457FD5}"/>
+    <hyperlink ref="A69" r:id="rId14" xr:uid="{AB7FBEEE-1168-436F-BA4D-AB14A31716CD}"/>
+    <hyperlink ref="D73" r:id="rId15" xr:uid="{5222E615-2E8F-47B0-8227-1D722BB1CAC0}"/>
+    <hyperlink ref="A75" r:id="rId16" xr:uid="{CF30A95F-E849-47BE-81B9-FBC5959A2D28}"/>
+    <hyperlink ref="D83" r:id="rId17" xr:uid="{377BFE9B-D854-4666-AE5C-BFE02A69AF01}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId14"/>
-  <drawing r:id="rId15"/>
+  <pageSetup orientation="portrait" r:id="rId18"/>
+  <drawing r:id="rId19"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
wordBreak - Mar 13 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F571A8-B218-4DAF-A477-10954C230B2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{599FB9C8-5013-45C4-9B42-097D71C9E809}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" activeTab="15" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="290">
   <si>
     <t>Statement</t>
   </si>
@@ -939,6 +939,30 @@
   </si>
   <si>
     <t>dfs as above but keep track of current index to avoid duplicates</t>
+  </si>
+  <si>
+    <t>use 1d dp array of size amount+1</t>
+  </si>
+  <si>
+    <t>init dp[0] to 1</t>
+  </si>
+  <si>
+    <t>for each coin check if possible to make up the amount</t>
+  </si>
+  <si>
+    <t>139. Word Break</t>
+  </si>
+  <si>
+    <t>keep dp boolean arr of size s</t>
+  </si>
+  <si>
+    <t>iterate s from last for each word</t>
+  </si>
+  <si>
+    <t>if word matches with s at current index, then dp[i] = dp[i+word.length]</t>
+  </si>
+  <si>
+    <t>do the same but through dfs, from top to bottom</t>
   </si>
 </sst>
 </file>
@@ -1924,6 +1948,50 @@
         <a:xfrm>
           <a:off x="3257550" y="14316075"/>
           <a:ext cx="3829584" cy="1400370"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>85</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4886325</xdr:colOff>
+      <xdr:row>88</xdr:row>
+      <xdr:rowOff>152496</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Picture 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C3C864FF-832A-4FDE-BC4A-609937A6A2AF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2895600" y="16230600"/>
+          <a:ext cx="4810125" cy="685896"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4292,7 +4360,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
-  <dimension ref="A1:D84"/>
+  <dimension ref="A1:D92"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -4552,13 +4620,65 @@
         <v>281</v>
       </c>
     </row>
-    <row r="83" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D76" s="4"/>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D77" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D78" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D79" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D83" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="84" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C84" s="5"/>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" s="8" t="s">
+        <v>285</v>
+      </c>
+      <c r="D85" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D86" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D87" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D88" s="4"/>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D89" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D91" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C92" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -4579,10 +4699,12 @@
     <hyperlink ref="D73" r:id="rId15" xr:uid="{5222E615-2E8F-47B0-8227-1D722BB1CAC0}"/>
     <hyperlink ref="A75" r:id="rId16" xr:uid="{CF30A95F-E849-47BE-81B9-FBC5959A2D28}"/>
     <hyperlink ref="D83" r:id="rId17" xr:uid="{377BFE9B-D854-4666-AE5C-BFE02A69AF01}"/>
+    <hyperlink ref="A85" r:id="rId18" xr:uid="{87D4722A-CBC5-4636-B3BA-A13BD3CAC44E}"/>
+    <hyperlink ref="D91" r:id="rId19" xr:uid="{E5CDA3AC-AFF1-4DA7-96D8-C017EE7EB73F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId18"/>
-  <drawing r:id="rId19"/>
+  <pageSetup orientation="portrait" r:id="rId20"/>
+  <drawing r:id="rId21"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
palindrome - Mar 15th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{599FB9C8-5013-45C4-9B42-097D71C9E809}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE466F1E-340A-4BF8-80FA-EA47B467B56A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" activeTab="15" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="16" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -29,6 +29,7 @@
     <sheet name="Sorting Algorithms" sheetId="15" r:id="rId14"/>
     <sheet name="Binary search" sheetId="16" r:id="rId15"/>
     <sheet name="dp" sheetId="6" r:id="rId16"/>
+    <sheet name="String" sheetId="18" r:id="rId17"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="294">
   <si>
     <t>Statement</t>
   </si>
@@ -963,6 +964,18 @@
   </si>
   <si>
     <t>do the same but through dfs, from top to bottom</t>
+  </si>
+  <si>
+    <t>5. Longest Palindromic Substring</t>
+  </si>
+  <si>
+    <t>iterate all chars with for loop</t>
+  </si>
+  <si>
+    <t>with current middle as odd palindrome - find max possibe</t>
+  </si>
+  <si>
+    <t>same with even</t>
   </si>
 </sst>
 </file>
@@ -1992,6 +2005,55 @@
         <a:xfrm>
           <a:off x="2895600" y="16230600"/>
           <a:ext cx="4810125" cy="685896"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing15.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>857250</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3829465</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>47706</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E8622481-DC5C-46FF-BD17-12F0D8C10BBF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3676650" y="609600"/>
+          <a:ext cx="2972215" cy="581106"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4708,6 +4770,72 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BDF4E8D-D4E1-4180-9015-2E66B34CBB41}">
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="2" max="2" width="73.85546875" customWidth="1"/>
+    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="D3" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D7" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C8" s="5"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{21D017E7-6C7E-4EA6-AE55-30155D149EEC}"/>
+    <hyperlink ref="D7" r:id="rId2" xr:uid="{B5902076-F258-44B7-A10E-28D7D53892DD}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AAA3DB6-B181-432C-9183-F47857237DA8}">
   <dimension ref="A1:D26"/>

</xml_diff>

<commit_message>
DecodeWays - Mar 15th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE466F1E-340A-4BF8-80FA-EA47B467B56A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D59643DD-28A7-4884-B293-5B8AC32AE8B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="16" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="12" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="303">
   <si>
     <t>Statement</t>
   </si>
@@ -976,6 +976,33 @@
   </si>
   <si>
     <t>same with even</t>
+  </si>
+  <si>
+    <t>91. Decode Ways</t>
+  </si>
+  <si>
+    <t>dfs from first char</t>
+  </si>
+  <si>
+    <t>if char[i] == 0 return 0</t>
+  </si>
+  <si>
+    <t>if i == n return 1</t>
+  </si>
+  <si>
+    <t>call dfs for i+1</t>
+  </si>
+  <si>
+    <t>if current + next char &gt;0 &lt;26 call dfs for i+2</t>
+  </si>
+  <si>
+    <t>use dp of size n+1</t>
+  </si>
+  <si>
+    <t>dp[0]=1 &amp; dp[1] = 1 if s[0] != '0'</t>
+  </si>
+  <si>
+    <t>iterate from 2nd char and fill dp considering i-1 &amp; i-2 values as dfs</t>
   </si>
 </sst>
 </file>
@@ -1462,6 +1489,50 @@
         <a:xfrm>
           <a:off x="3600450" y="590550"/>
           <a:ext cx="4543425" cy="2486372"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4477348</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>38184</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C7AE088B-8408-4A1E-9B1E-FE0FA8A5C0DA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3705225" y="3438525"/>
+          <a:ext cx="4286848" cy="600159"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4179,7 +4250,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E9C6576-B939-40FE-9164-B9EF7525065D}">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52.7109375" customWidth="1"/>
@@ -4235,16 +4306,72 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="3:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C17" s="5"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="8" t="s">
+        <v>294</v>
+      </c>
+      <c r="D18" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D19" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D20" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D21" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D22" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D23" s="4"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D24" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D25" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D26" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D27" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C28" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" xr:uid="{FA9D13DB-E1B4-4F9E-8A08-75017F0A9267}"/>
     <hyperlink ref="D16" r:id="rId2" xr:uid="{7DB504AE-B17D-4007-9242-6FFA0122E7AC}"/>
+    <hyperlink ref="A18" r:id="rId3" xr:uid="{88CD3D46-E074-402C-B2B3-12F18B9A8948}"/>
+    <hyperlink ref="D27" r:id="rId4" xr:uid="{D59A0C57-BC2B-4F4C-BFDD-37EBC7D8A67A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId3"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
 
@@ -4760,9 +4887,9 @@
     <hyperlink ref="A69" r:id="rId14" xr:uid="{AB7FBEEE-1168-436F-BA4D-AB14A31716CD}"/>
     <hyperlink ref="D73" r:id="rId15" xr:uid="{5222E615-2E8F-47B0-8227-1D722BB1CAC0}"/>
     <hyperlink ref="A75" r:id="rId16" xr:uid="{CF30A95F-E849-47BE-81B9-FBC5959A2D28}"/>
-    <hyperlink ref="D83" r:id="rId17" xr:uid="{377BFE9B-D854-4666-AE5C-BFE02A69AF01}"/>
-    <hyperlink ref="A85" r:id="rId18" xr:uid="{87D4722A-CBC5-4636-B3BA-A13BD3CAC44E}"/>
-    <hyperlink ref="D91" r:id="rId19" xr:uid="{E5CDA3AC-AFF1-4DA7-96D8-C017EE7EB73F}"/>
+    <hyperlink ref="A85" r:id="rId17" xr:uid="{87D4722A-CBC5-4636-B3BA-A13BD3CAC44E}"/>
+    <hyperlink ref="D91" r:id="rId18" xr:uid="{E5CDA3AC-AFF1-4DA7-96D8-C017EE7EB73F}"/>
+    <hyperlink ref="D83" r:id="rId19" xr:uid="{377BFE9B-D854-4666-AE5C-BFE02A69AF01}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId20"/>

</xml_diff>

<commit_message>
dp - Mar 16th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D59643DD-28A7-4884-B293-5B8AC32AE8B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90B01839-0A2C-4024-9B30-F9D3DAC78480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="12" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="15" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -25,9 +25,9 @@
     <sheet name="Graph" sheetId="12" r:id="rId10"/>
     <sheet name="Dictionary" sheetId="13" r:id="rId11"/>
     <sheet name="template" sheetId="2" r:id="rId12"/>
-    <sheet name="dfs" sheetId="17" r:id="rId13"/>
-    <sheet name="Sorting Algorithms" sheetId="15" r:id="rId14"/>
-    <sheet name="Binary search" sheetId="16" r:id="rId15"/>
+    <sheet name="Sorting Algorithms" sheetId="15" r:id="rId13"/>
+    <sheet name="Binary search" sheetId="16" r:id="rId14"/>
+    <sheet name="dfs" sheetId="17" r:id="rId15"/>
     <sheet name="dp" sheetId="6" r:id="rId16"/>
     <sheet name="String" sheetId="18" r:id="rId17"/>
   </sheets>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="322">
   <si>
     <t>Statement</t>
   </si>
@@ -1003,6 +1003,63 @@
   </si>
   <si>
     <t>iterate from 2nd char and fill dp considering i-1 &amp; i-2 values as dfs</t>
+  </si>
+  <si>
+    <t>dfs - Max(include current + dfs(i+2), dfs(i+1))</t>
+  </si>
+  <si>
+    <t>213. House Robber II</t>
+  </si>
+  <si>
+    <t>1. ignore 1st element</t>
+  </si>
+  <si>
+    <t>2. last element</t>
+  </si>
+  <si>
+    <t>In house robber 2</t>
+  </si>
+  <si>
+    <t>find max among -</t>
+  </si>
+  <si>
+    <t>515 · Paint House</t>
+  </si>
+  <si>
+    <t>start with index = 0, prev = -1</t>
+  </si>
+  <si>
+    <t>end condition is to reach length of matrix</t>
+  </si>
+  <si>
+    <t>iterate from 0-2 and call dfs with index + 1 and prev = current among 0-2 (iff prev != current among 0-2)</t>
+  </si>
+  <si>
+    <t>return min</t>
+  </si>
+  <si>
+    <t>300. Longest Increasing Subsequence</t>
+  </si>
+  <si>
+    <t>use dp of size 3</t>
+  </si>
+  <si>
+    <t>for each house take 1 color and add max among prev colors in dp</t>
+  </si>
+  <si>
+    <t>change dp array</t>
+  </si>
+  <si>
+    <t>dp of size n filled with 1</t>
+  </si>
+  <si>
+    <t>iterate from last i</t>
+  </si>
+  <si>
+    <t>iterate from i to end - if j &gt; i dp at i = max at i or 1+j =&gt; return max among dp</t>
+  </si>
+  <si>
+    <t>diffficult</t>
   </si>
 </sst>
 </file>
@@ -1456,6 +1513,104 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
+      <xdr:colOff>923925</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3410297</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>114384</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{381FF2E1-DE0E-4FD0-84D9-1D3679F1C0E3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3743325" y="466725"/>
+          <a:ext cx="2486372" cy="600159"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>847725</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3600834</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>142945</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{96852D08-DDF7-4290-8E9F-2D7EB6390BEE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3667125" y="590550"/>
+          <a:ext cx="2753109" cy="504895"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>85725</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
@@ -1544,104 +1699,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>923925</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>85725</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>3410297</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>114384</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{381FF2E1-DE0E-4FD0-84D9-1D3679F1C0E3}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3743325" y="466725"/>
-          <a:ext cx="2486372" cy="600159"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>847725</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>3600834</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>142945</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{96852D08-DDF7-4290-8E9F-2D7EB6390BEE}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3667125" y="590550"/>
-          <a:ext cx="2753109" cy="504895"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/drawings/drawing14.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
@@ -2076,6 +2133,94 @@
         <a:xfrm>
           <a:off x="2895600" y="16230600"/>
           <a:ext cx="4810125" cy="685896"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>762000</xdr:colOff>
+      <xdr:row>92</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4067636</xdr:colOff>
+      <xdr:row>95</xdr:row>
+      <xdr:rowOff>19120</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Picture 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4A38EE57-D6F4-4302-8AA8-C82DDF573F53}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3581400" y="17611725"/>
+          <a:ext cx="3305636" cy="504895"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>104</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4914900</xdr:colOff>
+      <xdr:row>107</xdr:row>
+      <xdr:rowOff>114392</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Picture 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6254A785-74D7-498D-AC04-7F04D1FD4C94}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2847975" y="19840575"/>
+          <a:ext cx="4886325" cy="657317"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4249,6 +4394,178 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0397D5EA-9127-4F39-A242-D8D4A93871ED}">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="2" max="2" width="73.85546875" customWidth="1"/>
+    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="D3" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="D4" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D6" s="8"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D10" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D12" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C13" s="5"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A4" r:id="rId1" xr:uid="{CBB80B45-9FC6-4C3A-BE11-6373B320529E}"/>
+    <hyperlink ref="A3" r:id="rId2" xr:uid="{1B705FA7-8F6C-4A90-88DF-06E322C116EF}"/>
+    <hyperlink ref="D12" r:id="rId3" xr:uid="{87407450-9806-4982-AA5D-2AE0CB10FC73}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId4"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC70315-55E0-46CA-8156-25A8AD92E211}">
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="2" max="2" width="73.85546875" customWidth="1"/>
+    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="D3" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D6" s="8"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D8" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D11" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C12" s="5"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{D15C5DE0-706A-4DBB-8F74-06E5036954E1}"/>
+    <hyperlink ref="D11" r:id="rId2" xr:uid="{78DAAF07-C11E-4A2F-B6D7-95F5F0D44DB8}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E9C6576-B939-40FE-9164-B9EF7525065D}">
   <dimension ref="A1:D28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4375,9 +4692,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0397D5EA-9127-4F39-A242-D8D4A93871ED}">
-  <dimension ref="A1:D13"/>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
+  <dimension ref="A1:D111"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -4407,178 +4724,6 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>219</v>
-      </c>
-      <c r="D3" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="D4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D5" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="8"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D8" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D9" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D10" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D12" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C13" s="5"/>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A4" r:id="rId1" xr:uid="{CBB80B45-9FC6-4C3A-BE11-6373B320529E}"/>
-    <hyperlink ref="A3" r:id="rId2" xr:uid="{1B705FA7-8F6C-4A90-88DF-06E322C116EF}"/>
-    <hyperlink ref="D12" r:id="rId3" xr:uid="{87407450-9806-4982-AA5D-2AE0CB10FC73}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId4"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC70315-55E0-46CA-8156-25A8AD92E211}">
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="42.28515625" customWidth="1"/>
-    <col min="2" max="2" width="73.85546875" customWidth="1"/>
-    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="91.7109375" customWidth="1"/>
-    <col min="13" max="13" width="6.7109375" customWidth="1"/>
-    <col min="14" max="14" width="8.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C2" s="5"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
-        <v>227</v>
-      </c>
-      <c r="D3" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D4" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D5" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="8"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D8" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D11" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C12" s="5"/>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" xr:uid="{D15C5DE0-706A-4DBB-8F74-06E5036954E1}"/>
-    <hyperlink ref="D11" r:id="rId2" xr:uid="{78DAAF07-C11E-4A2F-B6D7-95F5F0D44DB8}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
-  <dimension ref="A1:D92"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="42.28515625" customWidth="1"/>
-    <col min="2" max="2" width="73.85546875" customWidth="1"/>
-    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="91.7109375" customWidth="1"/>
-    <col min="13" max="13" width="6.7109375" customWidth="1"/>
-    <col min="14" max="14" width="8.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C2" s="5"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
         <v>104</v>
       </c>
       <c r="D3" t="s">
@@ -4674,15 +4819,38 @@
       <c r="A33" s="4" t="s">
         <v>263</v>
       </c>
+      <c r="C33" s="1" t="s">
+        <v>307</v>
+      </c>
       <c r="D33" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="D34" s="4"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C35" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="D35" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D34" s="4"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D35" t="s">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C36" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="D36" s="4"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D37" t="s">
         <v>265</v>
       </c>
     </row>
@@ -4868,6 +5036,94 @@
     </row>
     <row r="92" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C92" s="5"/>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A93" s="8" t="s">
+        <v>309</v>
+      </c>
+      <c r="D93" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D94" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D95" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D96" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D97" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D98" s="4"/>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D99" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D100" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D101" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D102" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C103" s="5"/>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A104" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="D104" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D105" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D106" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D107" s="4"/>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D108" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D110" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C111" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -4890,10 +5146,15 @@
     <hyperlink ref="A85" r:id="rId17" xr:uid="{87D4722A-CBC5-4636-B3BA-A13BD3CAC44E}"/>
     <hyperlink ref="D91" r:id="rId18" xr:uid="{E5CDA3AC-AFF1-4DA7-96D8-C017EE7EB73F}"/>
     <hyperlink ref="D83" r:id="rId19" xr:uid="{377BFE9B-D854-4666-AE5C-BFE02A69AF01}"/>
+    <hyperlink ref="A34" r:id="rId20" xr:uid="{937F3935-0316-4115-8802-7A6C8E04B698}"/>
+    <hyperlink ref="A93" r:id="rId21" xr:uid="{979771A5-E362-48DE-9923-7D8436A11AD2}"/>
+    <hyperlink ref="D102" r:id="rId22" xr:uid="{28D9FF8F-A25F-449D-BEAB-973FACA4FD3A}"/>
+    <hyperlink ref="A104" r:id="rId23" xr:uid="{F9969AE5-D9FE-4FC5-967E-01985A0E78AA}"/>
+    <hyperlink ref="D110" r:id="rId24" xr:uid="{EEBC8969-80BD-4AA0-8CF2-85A96BF48EC0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId20"/>
-  <drawing r:id="rId21"/>
+  <pageSetup orientation="portrait" r:id="rId25"/>
+  <drawing r:id="rId26"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
subarray sum and product - Mar 17th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90B01839-0A2C-4024-9B30-F9D3DAC78480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92D34205-1E04-4384-BCAA-73BF20CA6879}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="15" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="4" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="333">
   <si>
     <t>Statement</t>
   </si>
@@ -1023,9 +1023,6 @@
     <t>find max among -</t>
   </si>
   <si>
-    <t>515 · Paint House</t>
-  </si>
-  <si>
     <t>start with index = 0, prev = -1</t>
   </si>
   <si>
@@ -1059,7 +1056,43 @@
     <t>iterate from i to end - if j &gt; i dp at i = max at i or 1+j =&gt; return max among dp</t>
   </si>
   <si>
-    <t>diffficult</t>
+    <t>256· Paint House</t>
+  </si>
+  <si>
+    <t>Lintcode - 515 · Paint House</t>
+  </si>
+  <si>
+    <t>difficult</t>
+  </si>
+  <si>
+    <t>152. Maximum Product Subarray</t>
+  </si>
+  <si>
+    <t>keep variables maxProduct &amp; minProduct till now = 1, 1</t>
+  </si>
+  <si>
+    <t>iterate through all elements - maxProduct = max among maxProduct * current, minProduct * current and current</t>
+  </si>
+  <si>
+    <t>similarly keep track of minProduct</t>
+  </si>
+  <si>
+    <t>note max in all iterations</t>
+  </si>
+  <si>
+    <t>53. Maximum Subarray</t>
+  </si>
+  <si>
+    <t>init max = first and sum = 0</t>
+  </si>
+  <si>
+    <t>iterate and add nums to sum</t>
+  </si>
+  <si>
+    <t>update max</t>
+  </si>
+  <si>
+    <t>if sum &lt; 0 , reset to 0</t>
   </si>
 </sst>
 </file>
@@ -1243,7 +1276,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3"/>
@@ -1259,6 +1292,7 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="6"/>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="2" xfId="7"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="3" applyFill="1"/>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="Bad" xfId="5" builtinId="27"/>
@@ -2549,6 +2583,94 @@
         <a:xfrm>
           <a:off x="3638550" y="1743075"/>
           <a:ext cx="3848637" cy="638264"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>866775</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4048569</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>142969</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AA24E61E-FC5F-4318-BE0F-D6811A2D561A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4257675" y="4419600"/>
+          <a:ext cx="3181794" cy="676369"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>847725</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4172414</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>85810</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AAA63E16-7B74-4F3F-8D95-7E5AA6C7B7E4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4238625" y="5762625"/>
+          <a:ext cx="3324689" cy="609685"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5038,31 +5160,34 @@
       <c r="C92" s="5"/>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A93" s="8" t="s">
-        <v>309</v>
+      <c r="A93" s="13" t="s">
+        <v>320</v>
       </c>
       <c r="D93" t="s">
         <v>278</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A94" s="2" t="s">
+        <v>321</v>
+      </c>
       <c r="D94" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D95" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D96" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D97" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
@@ -5070,17 +5195,17 @@
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D99" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D100" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D101" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
@@ -5093,20 +5218,20 @@
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="8" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D104" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D105" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D106" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
@@ -5114,7 +5239,7 @@
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D108" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
@@ -5151,10 +5276,11 @@
     <hyperlink ref="D102" r:id="rId22" xr:uid="{28D9FF8F-A25F-449D-BEAB-973FACA4FD3A}"/>
     <hyperlink ref="A104" r:id="rId23" xr:uid="{F9969AE5-D9FE-4FC5-967E-01985A0E78AA}"/>
     <hyperlink ref="D110" r:id="rId24" xr:uid="{EEBC8969-80BD-4AA0-8CF2-85A96BF48EC0}"/>
+    <hyperlink ref="A94" r:id="rId25" xr:uid="{CE5BE0DF-21EC-4745-89A4-E000FF1A053F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId25"/>
-  <drawing r:id="rId26"/>
+  <pageSetup orientation="portrait" r:id="rId26"/>
+  <drawing r:id="rId27"/>
 </worksheet>
 </file>
 
@@ -5592,13 +5718,13 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDA924A8-9114-46BA-B39C-6743F04F80F3}">
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50.85546875" customWidth="1"/>
     <col min="2" max="2" width="73.85546875" customWidth="1"/>
     <col min="3" max="3" width="32.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="94.5703125" customWidth="1"/>
+    <col min="4" max="4" width="100.28515625" customWidth="1"/>
     <col min="13" max="13" width="6.7109375" customWidth="1"/>
     <col min="14" max="14" width="8.5703125" customWidth="1"/>
   </cols>
@@ -5681,17 +5807,17 @@
         <v>254</v>
       </c>
     </row>
-    <row r="17" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D17" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="18" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D18" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="19" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C19" s="1" t="s">
         <v>97</v>
       </c>
@@ -5699,18 +5825,80 @@
         <v>98</v>
       </c>
     </row>
-    <row r="20" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D20" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="21" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D21" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C22" s="5"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="8" t="s">
+        <v>323</v>
+      </c>
+      <c r="D23" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D24" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D25" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D26" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D28" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C29" s="5"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="D30" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D31" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D32" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="33" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D33" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="34" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D34" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C35" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -5718,9 +5906,13 @@
     <hyperlink ref="D7" r:id="rId2" xr:uid="{A82BE56D-8664-44EF-9D97-3B9B32089A10}"/>
     <hyperlink ref="A9" r:id="rId3" display="Median of Two Sorted Arrays" xr:uid="{E9DDCB05-35C4-411A-9E11-5D6F3CC3AF96}"/>
     <hyperlink ref="D21" r:id="rId4" xr:uid="{3402BAFA-50FF-4A91-9C05-9F6AEAC01303}"/>
+    <hyperlink ref="A23" r:id="rId5" xr:uid="{3ACA7BEF-5C8E-4D55-93F2-5B76A49DE403}"/>
+    <hyperlink ref="A30" r:id="rId6" xr:uid="{F636B6F6-9869-4224-B82D-26113E394418}"/>
+    <hyperlink ref="D28" r:id="rId7" xr:uid="{F7E2B43E-CE74-4C6C-BC40-1AF4C8945908}"/>
+    <hyperlink ref="D34" r:id="rId8" xr:uid="{677AF4C7-26E2-44C0-9632-F27FA8D63E1F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId5"/>
+  <drawing r:id="rId9"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
maximalSquare - Mar 17th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92D34205-1E04-4384-BCAA-73BF20CA6879}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66FA96F8-C36C-45AB-BA89-40CC95CCD520}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="4" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="5" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="344">
   <si>
     <t>Statement</t>
   </si>
@@ -1093,6 +1093,39 @@
   </si>
   <si>
     <t>if sum &lt; 0 , reset to 0</t>
+  </si>
+  <si>
+    <t>221. Maximal Square</t>
+  </si>
+  <si>
+    <t>Bruteforce - (mn)^2</t>
+  </si>
+  <si>
+    <t>if a cell is 1 start finding current max for it</t>
+  </si>
+  <si>
+    <t>start with curr = 1</t>
+  </si>
+  <si>
+    <t>for row check last columns, and for column check last rows</t>
+  </si>
+  <si>
+    <t>if last rows &amp; columns are 1's then curr++, till they are 1's</t>
+  </si>
+  <si>
+    <t>note the max</t>
+  </si>
+  <si>
+    <t>use dp[m+1][n+1]</t>
+  </si>
+  <si>
+    <t>start from 1 - mn</t>
+  </si>
+  <si>
+    <t>max = min(m-1,n-1 &amp;&amp; m-1,n &amp;&amp; m,n-1) + 1 if current == 1</t>
+  </si>
+  <si>
+    <t>note the max as well</t>
   </si>
 </sst>
 </file>
@@ -2852,6 +2885,50 @@
         <a:xfrm>
           <a:off x="2905125" y="8972550"/>
           <a:ext cx="4829175" cy="5668166"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>95251</xdr:colOff>
+      <xdr:row>79</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4857751</xdr:colOff>
+      <xdr:row>97</xdr:row>
+      <xdr:rowOff>162422</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{58CCB3D4-4B21-433A-8E71-C329700759ED}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2914651" y="15078075"/>
+          <a:ext cx="4762500" cy="3562847"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5918,7 +5995,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83AD0EA2-442A-436B-AA00-D0DF9DB7227A}">
-  <dimension ref="A1:D78"/>
+  <dimension ref="A1:D99"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -6042,13 +6119,77 @@
         <v>262</v>
       </c>
     </row>
-    <row r="77" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D77" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="78" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C78" s="5"/>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="D79" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D80" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="81" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D81" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="82" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D82" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="83" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D83" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="84" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D84" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="85" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D85" s="4"/>
+    </row>
+    <row r="86" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D86" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="87" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D87" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="88" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D88" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="89" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D89" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="98" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D98" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C99" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -6060,10 +6201,12 @@
     <hyperlink ref="D43" r:id="rId6" xr:uid="{60E813ED-AC35-4B86-9781-5B80FA133723}"/>
     <hyperlink ref="A47" r:id="rId7" xr:uid="{B9C0BE08-1E7F-4552-9904-54253A2CA85D}"/>
     <hyperlink ref="D77" r:id="rId8" xr:uid="{32267523-470D-47CA-8715-C3AB3030E922}"/>
+    <hyperlink ref="A79" r:id="rId9" xr:uid="{DC3476C5-9FFE-4318-B6B8-5984BE1EAFD5}"/>
+    <hyperlink ref="D98" r:id="rId10" xr:uid="{01BE9452-404A-4580-8C56-B003AE57914E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId9"/>
-  <drawing r:id="rId10"/>
+  <pageSetup orientation="portrait" r:id="rId11"/>
+  <drawing r:id="rId12"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
tree - Mar 18th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66FA96F8-C36C-45AB-BA89-40CC95CCD520}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62E18BB1-1B00-41B6-BE67-45BC281ECD5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="5" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="16" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -29,7 +29,8 @@
     <sheet name="Binary search" sheetId="16" r:id="rId14"/>
     <sheet name="dfs" sheetId="17" r:id="rId15"/>
     <sheet name="dp" sheetId="6" r:id="rId16"/>
-    <sheet name="String" sheetId="18" r:id="rId17"/>
+    <sheet name="Tree" sheetId="19" r:id="rId17"/>
+    <sheet name="String" sheetId="18" r:id="rId18"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -48,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="355">
   <si>
     <t>Statement</t>
   </si>
@@ -1126,6 +1127,39 @@
   </si>
   <si>
     <t>note the max as well</t>
+  </si>
+  <si>
+    <t>120. Triangle</t>
+  </si>
+  <si>
+    <t>iterate from last but 1 row</t>
+  </si>
+  <si>
+    <t>add min of current and next value from next row</t>
+  </si>
+  <si>
+    <t>return first element</t>
+  </si>
+  <si>
+    <t>else similarly do dp of 1d or 2d array</t>
+  </si>
+  <si>
+    <t>96. Unique Binary Search Trees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">consider each node as root </t>
+  </si>
+  <si>
+    <t>so use dp = array list</t>
+  </si>
+  <si>
+    <t>0=&gt;1 &amp; 1=&gt;1</t>
+  </si>
+  <si>
+    <t>iterate to fill dp from 2 - n</t>
+  </si>
+  <si>
+    <t>for any n - find combinations by putting some on left and n - some -1 on right</t>
   </si>
 </sst>
 </file>
@@ -2296,10 +2330,103 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>112</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4905375</xdr:colOff>
+      <xdr:row>120</xdr:row>
+      <xdr:rowOff>114525</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Picture 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{23AD56BA-928B-4D4B-8BF2-91442C14975B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2867025" y="21364575"/>
+          <a:ext cx="4857750" cy="1609950"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing15.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>66676</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4867276</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>181262</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{82B46A45-5469-48BE-9BC5-9A0B45F0D98E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2886076" y="600075"/>
+          <a:ext cx="4800600" cy="2057687"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing16.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -4893,7 +5020,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
-  <dimension ref="A1:D111"/>
+  <dimension ref="A1:D122"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -5326,6 +5453,40 @@
     </row>
     <row r="111" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C111" s="5"/>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A112" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="D112" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="113" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D113" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="114" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D114" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="115" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D115" s="4"/>
+    </row>
+    <row r="116" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D116" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="121" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D121" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C122" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -5354,14 +5515,92 @@
     <hyperlink ref="A104" r:id="rId23" xr:uid="{F9969AE5-D9FE-4FC5-967E-01985A0E78AA}"/>
     <hyperlink ref="D110" r:id="rId24" xr:uid="{EEBC8969-80BD-4AA0-8CF2-85A96BF48EC0}"/>
     <hyperlink ref="A94" r:id="rId25" xr:uid="{CE5BE0DF-21EC-4745-89A4-E000FF1A053F}"/>
+    <hyperlink ref="A112" r:id="rId26" xr:uid="{3B73D3B5-CE16-4ED9-A68E-2CFE5F8AE2D8}"/>
+    <hyperlink ref="D121" r:id="rId27" xr:uid="{C6CC741C-F1EF-403B-933A-047E364E457D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId26"/>
-  <drawing r:id="rId27"/>
+  <pageSetup orientation="portrait" r:id="rId28"/>
+  <drawing r:id="rId29"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36268CC4-0AC5-4653-846F-9B607EC203E4}">
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="2" max="2" width="73.85546875" customWidth="1"/>
+    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>349</v>
+      </c>
+      <c r="D3" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D6" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D14" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C15" s="5"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{54117466-2782-468C-AD18-FC894EF7B088}"/>
+    <hyperlink ref="D14" r:id="rId2" xr:uid="{16097345-4A31-47BC-92C1-D1A6FA33CDED}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BDF4E8D-D4E1-4180-9015-2E66B34CBB41}">
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
dp - Mar 19th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62E18BB1-1B00-41B6-BE67-45BC281ECD5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BBD2303-1735-4F14-98C8-F796E8B2C0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="16" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="5" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="373">
   <si>
     <t>Statement</t>
   </si>
@@ -1160,6 +1160,60 @@
   </si>
   <si>
     <t>for any n - find combinations by putting some on left and n - some -1 on right</t>
+  </si>
+  <si>
+    <t>10. Regular Expression Matching</t>
+  </si>
+  <si>
+    <t>start from i and j</t>
+  </si>
+  <si>
+    <t>end cases - if j reach end i should be at end</t>
+  </si>
+  <si>
+    <t>check first match for char and .</t>
+  </si>
+  <si>
+    <t>if wildcard matches i.e j+1 is *, then either use first match or else don't use wildcard</t>
+  </si>
+  <si>
+    <t>else check first match and use both chars</t>
+  </si>
+  <si>
+    <t>55. Jump Game</t>
+  </si>
+  <si>
+    <t xml:space="preserve">make last as goal </t>
+  </si>
+  <si>
+    <t>iterate from last but one to 0</t>
+  </si>
+  <si>
+    <t>if from i we can jump to goal -  make i as goal</t>
+  </si>
+  <si>
+    <t>45. Jump Game II</t>
+  </si>
+  <si>
+    <t>for jump game 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">use farthest from current group </t>
+  </si>
+  <si>
+    <t>and from prev group</t>
+  </si>
+  <si>
+    <t>62. Unique Paths</t>
+  </si>
+  <si>
+    <t>end case to reach m-1, n-1</t>
+  </si>
+  <si>
+    <t>start from 0, 0</t>
+  </si>
+  <si>
+    <t>return dfs for (i+1,j) + (i, j+1)</t>
   </si>
 </sst>
 </file>
@@ -2472,6 +2526,50 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4429665</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>85813</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{80716C16-881E-4527-8CEF-4A43228211C1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3381375" y="1743075"/>
+          <a:ext cx="3867690" cy="628738"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2839,6 +2937,50 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4914900</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>76288</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FD5AA444-F6C5-4C63-9117-58A08610081E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3419475" y="6877050"/>
+          <a:ext cx="4886325" cy="628738"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -3056,6 +3198,50 @@
         <a:xfrm>
           <a:off x="2914651" y="15078075"/>
           <a:ext cx="4762500" cy="3562847"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>590550</xdr:colOff>
+      <xdr:row>100</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4477292</xdr:colOff>
+      <xdr:row>111</xdr:row>
+      <xdr:rowOff>152707</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7CFB0031-873D-4D67-8934-3757CD372C6F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3409950" y="19097625"/>
+          <a:ext cx="3886742" cy="2200582"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5602,7 +5788,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BDF4E8D-D4E1-4180-9015-2E66B34CBB41}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -5656,13 +5842,56 @@
     <row r="8" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C8" s="5"/>
     </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
+        <v>355</v>
+      </c>
+      <c r="D9" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D10" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D11" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D12" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D13" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D14" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D16" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="3:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C17" s="5"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" xr:uid="{21D017E7-6C7E-4EA6-AE55-30155D149EEC}"/>
     <hyperlink ref="D7" r:id="rId2" xr:uid="{B5902076-F258-44B7-A10E-28D7D53892DD}"/>
+    <hyperlink ref="A9" r:id="rId3" xr:uid="{41CA7DEA-C842-4838-AA5B-416057A8B26C}"/>
+    <hyperlink ref="D16" r:id="rId4" xr:uid="{7D78E185-BD0C-42CC-955B-A30BB33C24AE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId3"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
 
@@ -6034,7 +6263,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDA924A8-9114-46BA-B39C-6743F04F80F3}">
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50.85546875" customWidth="1"/>
@@ -6155,7 +6384,7 @@
       <c r="C22" s="5"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="8" t="s">
+      <c r="A23" s="13" t="s">
         <v>323</v>
       </c>
       <c r="D23" t="s">
@@ -6203,18 +6432,56 @@
         <v>331</v>
       </c>
     </row>
-    <row r="33" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D33" t="s">
         <v>332</v>
       </c>
     </row>
-    <row r="34" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D34" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C35" s="5"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="13" t="s">
+        <v>361</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="D36" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="D37" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C38" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="D38" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D40" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C41" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -6222,19 +6489,22 @@
     <hyperlink ref="D7" r:id="rId2" xr:uid="{A82BE56D-8664-44EF-9D97-3B9B32089A10}"/>
     <hyperlink ref="A9" r:id="rId3" display="Median of Two Sorted Arrays" xr:uid="{E9DDCB05-35C4-411A-9E11-5D6F3CC3AF96}"/>
     <hyperlink ref="D21" r:id="rId4" xr:uid="{3402BAFA-50FF-4A91-9C05-9F6AEAC01303}"/>
-    <hyperlink ref="A23" r:id="rId5" xr:uid="{3ACA7BEF-5C8E-4D55-93F2-5B76A49DE403}"/>
-    <hyperlink ref="A30" r:id="rId6" xr:uid="{F636B6F6-9869-4224-B82D-26113E394418}"/>
-    <hyperlink ref="D28" r:id="rId7" xr:uid="{F7E2B43E-CE74-4C6C-BC40-1AF4C8945908}"/>
-    <hyperlink ref="D34" r:id="rId8" xr:uid="{677AF4C7-26E2-44C0-9632-F27FA8D63E1F}"/>
+    <hyperlink ref="A30" r:id="rId5" xr:uid="{F636B6F6-9869-4224-B82D-26113E394418}"/>
+    <hyperlink ref="D28" r:id="rId6" xr:uid="{F7E2B43E-CE74-4C6C-BC40-1AF4C8945908}"/>
+    <hyperlink ref="D34" r:id="rId7" xr:uid="{677AF4C7-26E2-44C0-9632-F27FA8D63E1F}"/>
+    <hyperlink ref="A36" r:id="rId8" xr:uid="{20862B18-8968-4B87-9A93-3C252D794975}"/>
+    <hyperlink ref="A23" r:id="rId9" xr:uid="{F16EB101-F0CB-48DB-8CC1-4B777907F79A}"/>
+    <hyperlink ref="D40" r:id="rId10" xr:uid="{1392FFB3-5685-43A8-8CC5-71556F981E6A}"/>
+    <hyperlink ref="A37" r:id="rId11" xr:uid="{E12E6C6B-5CBE-4336-9DD7-AB14B0F9585C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId9"/>
+  <drawing r:id="rId12"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83AD0EA2-442A-436B-AA00-D0DF9DB7227A}">
-  <dimension ref="A1:D99"/>
+  <dimension ref="A1:D113"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -6422,13 +6692,44 @@
         <v>343</v>
       </c>
     </row>
-    <row r="98" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D98" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="99" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C99" s="5"/>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A100" s="13" t="s">
+        <v>369</v>
+      </c>
+      <c r="D100" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D101" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D102" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D103" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D112" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="3:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C113" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -6442,10 +6743,12 @@
     <hyperlink ref="D77" r:id="rId8" xr:uid="{32267523-470D-47CA-8715-C3AB3030E922}"/>
     <hyperlink ref="A79" r:id="rId9" xr:uid="{DC3476C5-9FFE-4318-B6B8-5984BE1EAFD5}"/>
     <hyperlink ref="D98" r:id="rId10" xr:uid="{01BE9452-404A-4580-8C56-B003AE57914E}"/>
+    <hyperlink ref="A100" r:id="rId11" xr:uid="{CECF130D-CC26-4D13-BA9A-5504D8EA8278}"/>
+    <hyperlink ref="D112" r:id="rId12" xr:uid="{5BF85361-6BEF-4029-A6B4-31A2721F2F6D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId11"/>
-  <drawing r:id="rId12"/>
+  <pageSetup orientation="portrait" r:id="rId13"/>
+  <drawing r:id="rId14"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
PerfectSquares - Mar 20th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BBD2303-1735-4F14-98C8-F796E8B2C0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08889E69-1F3F-4E9D-8257-190E9C0A2BF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="5" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="15" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="379">
   <si>
     <t>Statement</t>
   </si>
@@ -382,12 +382,6 @@
   </si>
   <si>
     <t>Bottom up solution - dp[m+1][n+1]</t>
-  </si>
-  <si>
-    <t>while iterating - if both chars are same call next itr ([i][j] = [i-1][j-1])</t>
-  </si>
-  <si>
-    <t>else min of 1 + (addn - [i-1][j], deletn - [i][j-1], replace - [i-1][j-1])</t>
   </si>
   <si>
     <t>97. Interleaving String</t>
@@ -1214,6 +1208,30 @@
   </si>
   <si>
     <t>return dfs for (i+1,j) + (i, j+1)</t>
+  </si>
+  <si>
+    <t>279. Perfect Squares</t>
+  </si>
+  <si>
+    <t>fill all with n and 0 with 0</t>
+  </si>
+  <si>
+    <t>iterate through all elements to find min combination for each</t>
+  </si>
+  <si>
+    <t>for each square posiible within i</t>
+  </si>
+  <si>
+    <t>dp[i] = min(dp[i], dp[i-square])</t>
+  </si>
+  <si>
+    <t>similarly dfs</t>
+  </si>
+  <si>
+    <t>while iterating - if both chars are same call next itr ([i][j] = [i+1][j+1])</t>
+  </si>
+  <si>
+    <t>else min of 1 + (addn : [i+1][j], deletn : [i][j+1], replace : [i+1][j+1])</t>
   </si>
 </sst>
 </file>
@@ -2420,6 +2438,50 @@
         <a:xfrm>
           <a:off x="2867025" y="21364575"/>
           <a:ext cx="4857750" cy="1609950"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1352550</xdr:colOff>
+      <xdr:row>123</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3429290</xdr:colOff>
+      <xdr:row>126</xdr:row>
+      <xdr:rowOff>123917</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Picture 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BAD39209-FC96-4BB4-B06C-BA51DE776A2A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4171950" y="23469600"/>
+          <a:ext cx="2076740" cy="657317"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4549,10 +4611,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="6" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -4560,30 +4622,30 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D7" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D9" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -4596,20 +4658,20 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="D24" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D25" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D26" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -4622,28 +4684,28 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="8" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D44" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D45" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D46" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D47" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -4656,20 +4718,20 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D51" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D52" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D53" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="70" spans="4:4" x14ac:dyDescent="0.25">
@@ -4682,35 +4744,35 @@
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="8" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D87" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D88" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D89" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D90" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D91" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D92" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
@@ -4723,15 +4785,15 @@
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="8" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D97" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D98" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
@@ -4797,15 +4859,15 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="D3" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -4818,34 +4880,34 @@
     </row>
     <row r="8" spans="1:4" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D8" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="D9" t="s">
         <v>236</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="D9" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="17" spans="3:4" x14ac:dyDescent="0.25">
@@ -4937,23 +4999,23 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="D3" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="D4" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -4961,22 +5023,22 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D9" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -5030,20 +5092,20 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -5051,12 +5113,12 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -5109,25 +5171,25 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="D3" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -5140,30 +5202,30 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="D18" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D19" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D20" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D21" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -5171,17 +5233,17 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D24" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D25" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D26" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -5206,7 +5268,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
-  <dimension ref="A1:D122"/>
+  <dimension ref="A1:D130"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -5275,12 +5337,20 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
-        <v>111</v>
+        <v>377</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D12" t="s">
-        <v>112</v>
+        <v>378</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D13" s="4"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D14" t="s">
+        <v>376</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -5293,30 +5363,30 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D18" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D19" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D20" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D21" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -5329,41 +5399,41 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="D33" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="D34" s="4"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C35" s="1" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="D35" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C36" s="1" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="D36" s="4"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D37" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -5376,25 +5446,25 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="8" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D40" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D41" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D42" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D43" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -5407,20 +5477,20 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D51" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D52" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D53" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -5433,23 +5503,23 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="D59" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C60" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="D60" t="s">
         <v>274</v>
-      </c>
-      <c r="D60" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D61" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -5462,15 +5532,15 @@
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="8" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="D69" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D70" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -5483,10 +5553,10 @@
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="8" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D75" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -5494,17 +5564,17 @@
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D77" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D78" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D79" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
@@ -5517,20 +5587,20 @@
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="D85" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D86" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D87" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
@@ -5538,7 +5608,7 @@
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D89" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
@@ -5551,33 +5621,33 @@
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="13" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="D93" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D94" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D95" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D96" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D97" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
@@ -5585,17 +5655,17 @@
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D99" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D100" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D101" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
@@ -5608,20 +5678,20 @@
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="8" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="D104" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D105" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D106" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
@@ -5629,7 +5699,7 @@
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D108" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
@@ -5642,37 +5712,73 @@
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="8" t="s">
+        <v>342</v>
+      </c>
+      <c r="D112" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D113" t="s">
         <v>344</v>
       </c>
-      <c r="D112" t="s">
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D114" t="s">
         <v>345</v>
       </c>
     </row>
-    <row r="113" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="D113" t="s">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D115" s="4"/>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D116" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="114" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="D114" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="115" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="D115" s="4"/>
-    </row>
-    <row r="116" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="D116" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="121" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D121" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="122" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C122" s="5"/>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A123" s="13" t="s">
+        <v>371</v>
+      </c>
+      <c r="D123" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D124" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D125" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D126" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D127" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="129" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D129" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="130" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C130" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -5703,10 +5809,11 @@
     <hyperlink ref="A94" r:id="rId25" xr:uid="{CE5BE0DF-21EC-4745-89A4-E000FF1A053F}"/>
     <hyperlink ref="A112" r:id="rId26" xr:uid="{3B73D3B5-CE16-4ED9-A68E-2CFE5F8AE2D8}"/>
     <hyperlink ref="D121" r:id="rId27" xr:uid="{C6CC741C-F1EF-403B-933A-047E364E457D}"/>
+    <hyperlink ref="A123" r:id="rId28" xr:uid="{E4F469FE-9B9E-44DD-BE4F-7E7E49F00709}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId28"/>
-  <drawing r:id="rId29"/>
+  <pageSetup orientation="portrait" r:id="rId29"/>
+  <drawing r:id="rId30"/>
 </worksheet>
 </file>
 
@@ -5742,30 +5849,30 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D3" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -5818,20 +5925,20 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="D3" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -5844,35 +5951,35 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="D9" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D12" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D13" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D14" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -5927,25 +6034,25 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -5958,35 +6065,35 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D11" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D12" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D13" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D14" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D15" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D16" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -5999,25 +6106,25 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D20" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D21" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D23" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -6074,25 +6181,25 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -6105,31 +6212,31 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D13" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C14" s="1" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="D14" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D15" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D16" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="18" spans="3:4" x14ac:dyDescent="0.25">
@@ -6184,35 +6291,35 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -6225,20 +6332,20 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="D17" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D18" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D19" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -6293,7 +6400,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D3" t="s">
         <v>90</v>
@@ -6306,7 +6413,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -6319,7 +6426,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -6334,7 +6441,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D12" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -6344,12 +6451,12 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D14" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D16" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -6385,25 +6492,25 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="D23" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D24" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D25" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D26" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -6416,25 +6523,25 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D30" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D31" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D32" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D33" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -6447,32 +6554,32 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="13" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="D36" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="C37" s="1" t="s">
         <v>365</v>
       </c>
-      <c r="C37" s="1" t="s">
-        <v>367</v>
-      </c>
       <c r="D37" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C38" s="1" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="D38" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -6534,7 +6641,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D3" t="s">
         <v>100</v>
@@ -6565,15 +6672,15 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="D21" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -6586,25 +6693,25 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="D31" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D32" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D33" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D34" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -6617,15 +6724,15 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="D47" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D48" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -6638,35 +6745,35 @@
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D79" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D80" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="81" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D81" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="82" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D82" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="83" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D83" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="84" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D84" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="85" spans="4:4" x14ac:dyDescent="0.25">
@@ -6674,22 +6781,22 @@
     </row>
     <row r="86" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D86" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="87" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D87" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="88" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D88" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="89" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D89" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
@@ -6702,25 +6809,25 @@
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="13" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="D100" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D101" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D102" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D103" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
@@ -6784,7 +6891,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D3" t="s">
         <v>45</v>
@@ -6815,7 +6922,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B17" t="s">
         <v>38</v>
@@ -6906,7 +7013,7 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D36" t="s">
         <v>55</v>
@@ -6952,7 +7059,7 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D49" t="s">
         <v>62</v>
@@ -6994,7 +7101,7 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D61" s="7" t="s">
         <v>44</v>
@@ -7043,7 +7150,7 @@
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="8" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C77" s="1" t="s">
         <v>80</v>
@@ -7093,7 +7200,7 @@
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="8" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D87" t="s">
         <v>83</v>
@@ -7197,7 +7304,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
@@ -7237,7 +7344,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B20" t="s">
         <v>8</v>
@@ -7306,7 +7413,7 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D36" t="s">
         <v>23</v>
@@ -7314,22 +7421,22 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D37" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D38" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D39" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D40" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -7375,7 +7482,7 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="9" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B51" t="s">
         <v>30</v>
@@ -7456,10 +7563,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -7472,10 +7579,10 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D11" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -7488,30 +7595,30 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="D19" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D20" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D21" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D26" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="27" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
DistinctSubsequences - Mar 20th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08889E69-1F3F-4E9D-8257-190E9C0A2BF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D68E33E5-F910-477F-91FD-7DD12CA473F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="15" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="379">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="385">
   <si>
     <t>Statement</t>
   </si>
@@ -1232,6 +1232,24 @@
   </si>
   <si>
     <t>else min of 1 + (addn : [i+1][j], deletn : [i][j+1], replace : [i+1][j+1])</t>
+  </si>
+  <si>
+    <t>115. Distinct Subsequences</t>
+  </si>
+  <si>
+    <t>start from 0,0</t>
+  </si>
+  <si>
+    <t>if t is at end return 1</t>
+  </si>
+  <si>
+    <t>if s is at end return 0</t>
+  </si>
+  <si>
+    <t>if current 2 chars are same call i+1, j+1 and get count</t>
+  </si>
+  <si>
+    <t>also get count for i+1, j</t>
   </si>
 </sst>
 </file>
@@ -1415,7 +1433,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3"/>
@@ -1432,6 +1450,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="6"/>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="2" xfId="7"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="3" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="3" applyFill="1"/>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="Bad" xfId="5" builtinId="27"/>
@@ -2482,6 +2501,50 @@
         <a:xfrm>
           <a:off x="4171950" y="23469600"/>
           <a:ext cx="2076740" cy="657317"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>142875</xdr:colOff>
+      <xdr:row>131</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4829829</xdr:colOff>
+      <xdr:row>138</xdr:row>
+      <xdr:rowOff>133551</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="Picture 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{69C5DDCF-090B-4412-AA59-E773A25EEBCA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2962275" y="24984075"/>
+          <a:ext cx="4686954" cy="1438476"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5268,7 +5331,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
-  <dimension ref="A1:D130"/>
+  <dimension ref="A1:D140"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -5772,13 +5835,54 @@
         <v>375</v>
       </c>
     </row>
-    <row r="129" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="D129" t="s">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D129" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="130" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C130" s="5"/>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A131" s="14" t="s">
+        <v>379</v>
+      </c>
+      <c r="D131" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D132" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D133" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D134" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D135" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D136" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D139" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C140" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -5810,10 +5914,13 @@
     <hyperlink ref="A112" r:id="rId26" xr:uid="{3B73D3B5-CE16-4ED9-A68E-2CFE5F8AE2D8}"/>
     <hyperlink ref="D121" r:id="rId27" xr:uid="{C6CC741C-F1EF-403B-933A-047E364E457D}"/>
     <hyperlink ref="A123" r:id="rId28" xr:uid="{E4F469FE-9B9E-44DD-BE4F-7E7E49F00709}"/>
+    <hyperlink ref="A131" r:id="rId29" xr:uid="{987A1555-C35C-4948-B108-C08BDC8FE9B0}"/>
+    <hyperlink ref="D129" r:id="rId30" xr:uid="{4F79E34E-15EB-4AD9-B828-473058090EC2}"/>
+    <hyperlink ref="D139" r:id="rId31" xr:uid="{9729ECE9-F78F-4E56-80C2-981532330ADE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId29"/>
-  <drawing r:id="rId30"/>
+  <pageSetup orientation="portrait" r:id="rId32"/>
+  <drawing r:id="rId33"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
22nd Mar - 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D68E33E5-F910-477F-91FD-7DD12CA473F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79A65F62-E28A-481B-98B2-EC4B43EC874D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="15" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="398">
   <si>
     <t>Statement</t>
   </si>
@@ -1250,6 +1250,57 @@
   </si>
   <si>
     <t>also get count for i+1, j</t>
+  </si>
+  <si>
+    <t>377. Combination Sum IV</t>
+  </si>
+  <si>
+    <t>for every num start over from start = 0, as even for start = 3 we need 1</t>
+  </si>
+  <si>
+    <t>return 1 if target == 0</t>
+  </si>
+  <si>
+    <t>return 0 if target &lt; 0</t>
+  </si>
+  <si>
+    <t>dp[target]</t>
+  </si>
+  <si>
+    <t>dp[0] = 1</t>
+  </si>
+  <si>
+    <t>for each i : target:</t>
+  </si>
+  <si>
+    <t>for each num : if i &gt;= num i += dp[i-num]</t>
+  </si>
+  <si>
+    <t>312. Burst Balloons</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">permutations - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>timeout</t>
+    </r>
+  </si>
+  <si>
+    <t>call backtrack</t>
+  </si>
+  <si>
+    <t>start from 0 all the time</t>
+  </si>
+  <si>
+    <t>use a set to track used ones</t>
   </si>
 </sst>
 </file>
@@ -2545,6 +2596,94 @@
         <a:xfrm>
           <a:off x="2962275" y="24984075"/>
           <a:ext cx="4686954" cy="1438476"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>161925</xdr:colOff>
+      <xdr:row>141</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4839353</xdr:colOff>
+      <xdr:row>153</xdr:row>
+      <xdr:rowOff>124160</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Picture 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FEE9D9BB-78B2-4D4C-BB67-C3DF0ADCADD8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2981325" y="26870025"/>
+          <a:ext cx="4677428" cy="2400635"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>695325</xdr:colOff>
+      <xdr:row>157</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4401067</xdr:colOff>
+      <xdr:row>162</xdr:row>
+      <xdr:rowOff>85867</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="Picture 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B7453641-1A08-4E19-BD26-8AEF2220D6CC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3514725" y="29927550"/>
+          <a:ext cx="3705742" cy="1019317"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5331,7 +5470,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
-  <dimension ref="A1:D140"/>
+  <dimension ref="A1:D170"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -5883,6 +6022,99 @@
     </row>
     <row r="140" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C140" s="5"/>
+    </row>
+    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A141" s="13" t="s">
+        <v>385</v>
+      </c>
+      <c r="D141" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D142" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D143" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D144" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D145" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D146" s="4"/>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D147" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D148" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D149" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D150" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D155" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C156" s="5"/>
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A157" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="D157" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D158" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D159" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D160" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="161" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D161" s="4"/>
+    </row>
+    <row r="169" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D169" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="170" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C170" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -5917,10 +6149,14 @@
     <hyperlink ref="A131" r:id="rId29" xr:uid="{987A1555-C35C-4948-B108-C08BDC8FE9B0}"/>
     <hyperlink ref="D129" r:id="rId30" xr:uid="{4F79E34E-15EB-4AD9-B828-473058090EC2}"/>
     <hyperlink ref="D139" r:id="rId31" xr:uid="{9729ECE9-F78F-4E56-80C2-981532330ADE}"/>
+    <hyperlink ref="A141" r:id="rId32" xr:uid="{E102098D-511B-4DF4-9B3A-95860EAFE1B8}"/>
+    <hyperlink ref="D155" r:id="rId33" xr:uid="{34DCD78E-0805-4EC0-AD2A-52F3FD1669BB}"/>
+    <hyperlink ref="A157" r:id="rId34" xr:uid="{E9DD9232-280B-4B8B-A729-20EB44C509B6}"/>
+    <hyperlink ref="D169" r:id="rId35" xr:uid="{B37792E6-28BA-4481-8374-9991E31B71D2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId32"/>
-  <drawing r:id="rId33"/>
+  <pageSetup orientation="portrait" r:id="rId36"/>
+  <drawing r:id="rId37"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
24 Mar 2022 - BurstBalloons
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79A65F62-E28A-481B-98B2-EC4B43EC874D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B9E26C6-5389-432B-BBD8-AC9BC0CDF198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="15" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="398">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="402">
   <si>
     <t>Statement</t>
   </si>
@@ -1301,6 +1301,18 @@
   </si>
   <si>
     <t>use a set to track used ones</t>
+  </si>
+  <si>
+    <t>create copy with edges as 1</t>
+  </si>
+  <si>
+    <t>use recursion</t>
+  </si>
+  <si>
+    <t>for each start and end assume they are last balloons - burst them and recurse for other ones</t>
+  </si>
+  <si>
+    <t>using map for memo won't work - timeout</t>
   </si>
 </sst>
 </file>
@@ -6108,6 +6120,24 @@
     <row r="161" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D161" s="4"/>
     </row>
+    <row r="162" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C162" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="D162" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="163" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D163" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="164" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D164" t="s">
+        <v>400</v>
+      </c>
+    </row>
     <row r="169" spans="3:4" x14ac:dyDescent="0.25">
       <c r="D169" s="2" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
PartitionEqualSubsetSum - Mar 25th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B9E26C6-5389-432B-BBD8-AC9BC0CDF198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA23285F-EE73-4E60-B020-AF9ECDBB73F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="15" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="411">
   <si>
     <t>Statement</t>
   </si>
@@ -1313,6 +1313,33 @@
   </si>
   <si>
     <t>using map for memo won't work - timeout</t>
+  </si>
+  <si>
+    <t>1911. Maximum Alternating Subsequence Sum</t>
+  </si>
+  <si>
+    <t>keep track of even and odd - 0,0 start will be even</t>
+  </si>
+  <si>
+    <t>call dfs using current and not using current</t>
+  </si>
+  <si>
+    <t>416. Partition Equal Subset Sum</t>
+  </si>
+  <si>
+    <t>find total sum</t>
+  </si>
+  <si>
+    <t>using dfs find if sum/2 can be formed</t>
+  </si>
+  <si>
+    <t>use set as dp</t>
+  </si>
+  <si>
+    <t>add element and sum to prev elements as well</t>
+  </si>
+  <si>
+    <t>if set at any point has sum/2 then return true</t>
   </si>
 </sst>
 </file>
@@ -2696,6 +2723,94 @@
         <a:xfrm>
           <a:off x="3514725" y="29927550"/>
           <a:ext cx="3705742" cy="1019317"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>171</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>174</xdr:row>
+      <xdr:rowOff>57234</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="19" name="Picture 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5288985C-424B-4DB9-B98E-7510244DF40A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2838450" y="32604075"/>
+          <a:ext cx="4905375" cy="600159"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>504825</xdr:colOff>
+      <xdr:row>178</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4486831</xdr:colOff>
+      <xdr:row>181</xdr:row>
+      <xdr:rowOff>38181</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="20" name="Picture 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{47968A35-8635-4AF5-BFB1-814AB1AEB038}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3324225" y="33937575"/>
+          <a:ext cx="3982006" cy="581106"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5482,7 +5597,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
-  <dimension ref="A1:D170"/>
+  <dimension ref="A1:D187"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -6117,10 +6232,10 @@
         <v>397</v>
       </c>
     </row>
-    <row r="161" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D161" s="4"/>
     </row>
-    <row r="162" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C162" s="1" t="s">
         <v>401</v>
       </c>
@@ -6128,23 +6243,93 @@
         <v>398</v>
       </c>
     </row>
-    <row r="163" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D163" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="164" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D164" t="s">
         <v>400</v>
       </c>
     </row>
-    <row r="169" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D169" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="170" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C170" s="5"/>
+    </row>
+    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A171" s="13" t="s">
+        <v>402</v>
+      </c>
+      <c r="D171" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D172" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D173" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D174" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D176" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="177" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C177" s="5"/>
+    </row>
+    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A178" s="13" t="s">
+        <v>405</v>
+      </c>
+      <c r="D178" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D179" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D180" s="4"/>
+    </row>
+    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D181" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D182" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D183" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="186" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D186" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="187" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C187" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -6183,10 +6368,14 @@
     <hyperlink ref="D155" r:id="rId33" xr:uid="{34DCD78E-0805-4EC0-AD2A-52F3FD1669BB}"/>
     <hyperlink ref="A157" r:id="rId34" xr:uid="{E9DD9232-280B-4B8B-A729-20EB44C509B6}"/>
     <hyperlink ref="D169" r:id="rId35" xr:uid="{B37792E6-28BA-4481-8374-9991E31B71D2}"/>
+    <hyperlink ref="A171" r:id="rId36" xr:uid="{77B17A77-30EE-459E-B7CD-147FBF0E8523}"/>
+    <hyperlink ref="D176" r:id="rId37" xr:uid="{6C2363E3-0E3A-4EBE-8D53-454DDE516888}"/>
+    <hyperlink ref="A178" r:id="rId38" xr:uid="{5EF8094F-0113-4F1C-9272-FD2A4007BC58}"/>
+    <hyperlink ref="D186" r:id="rId39" xr:uid="{B634781E-00FF-4F3E-B5F5-BC6FA60A5E7F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId36"/>
-  <drawing r:id="rId37"/>
+  <pageSetup orientation="portrait" r:id="rId40"/>
+  <drawing r:id="rId41"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
StickerstoSpellWord - Mar 26th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA23285F-EE73-4E60-B020-AF9ECDBB73F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A95049D3-82CB-4810-B6A5-2B9CC7567595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="15" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="411">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="419">
   <si>
     <t>Statement</t>
   </si>
@@ -1340,6 +1340,30 @@
   </si>
   <si>
     <t>if set at any point has sum/2 then return true</t>
+  </si>
+  <si>
+    <t>691. Stickers to Spell Word</t>
+  </si>
+  <si>
+    <t>keep char count of each sticker</t>
+  </si>
+  <si>
+    <t>use dfs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">use 1 sticker and add 1 to count if used sticker had any chars </t>
+  </si>
+  <si>
+    <t>call 1 + dfs with min recorded</t>
+  </si>
+  <si>
+    <t>338. Counting Bits</t>
+  </si>
+  <si>
+    <t>dp</t>
+  </si>
+  <si>
+    <t>i = i/2 + (i &amp; 2)</t>
   </si>
 </sst>
 </file>
@@ -1523,7 +1547,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3"/>
@@ -1541,6 +1565,7 @@
     <xf numFmtId="0" fontId="11" fillId="6" borderId="2" xfId="7"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="3" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="3" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="3" applyFill="1"/>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="Bad" xfId="5" builtinId="27"/>
@@ -2811,6 +2836,94 @@
         <a:xfrm>
           <a:off x="3324225" y="33937575"/>
           <a:ext cx="3982006" cy="581106"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>188</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4867275</xdr:colOff>
+      <xdr:row>193</xdr:row>
+      <xdr:rowOff>181129</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="21" name="Picture 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{571E0322-050B-4EFD-A219-DE4B575E7BFA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2857500" y="35842575"/>
+          <a:ext cx="4829175" cy="1105054"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1714500</xdr:colOff>
+      <xdr:row>196</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2762396</xdr:colOff>
+      <xdr:row>201</xdr:row>
+      <xdr:rowOff>171604</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="22" name="Picture 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{21FA816F-34B8-490E-8521-7A2CC47236B8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId21"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4533900" y="37357050"/>
+          <a:ext cx="1047896" cy="1105054"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5597,7 +5710,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
-  <dimension ref="A1:D187"/>
+  <dimension ref="A1:D204"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -6330,6 +6443,58 @@
     </row>
     <row r="187" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C187" s="5"/>
+    </row>
+    <row r="188" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A188" s="14" t="s">
+        <v>411</v>
+      </c>
+      <c r="D188" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="189" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D189" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="190" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D190" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="191" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D191" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="194" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D194" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="195" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C195" s="5"/>
+    </row>
+    <row r="196" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A196" s="15" t="s">
+        <v>416</v>
+      </c>
+      <c r="D196" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="197" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D197" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="203" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D203" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="204" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C204" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -6372,10 +6537,14 @@
     <hyperlink ref="D176" r:id="rId37" xr:uid="{6C2363E3-0E3A-4EBE-8D53-454DDE516888}"/>
     <hyperlink ref="A178" r:id="rId38" xr:uid="{5EF8094F-0113-4F1C-9272-FD2A4007BC58}"/>
     <hyperlink ref="D186" r:id="rId39" xr:uid="{B634781E-00FF-4F3E-B5F5-BC6FA60A5E7F}"/>
+    <hyperlink ref="A188" r:id="rId40" xr:uid="{27491F11-A710-4CCB-9017-F947DF6FEC44}"/>
+    <hyperlink ref="D194" r:id="rId41" xr:uid="{511FE57E-DCE1-410D-BD38-C4F43E785E3A}"/>
+    <hyperlink ref="A196" r:id="rId42" xr:uid="{33C8DB24-35DF-4AA2-A7F2-6187258CBF38}"/>
+    <hyperlink ref="D203" r:id="rId43" xr:uid="{085A29C3-E8EF-48CF-8410-9E7F6639072E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId40"/>
-  <drawing r:id="rId41"/>
+  <pageSetup orientation="portrait" r:id="rId44"/>
+  <drawing r:id="rId45"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
AllPossibleFullBinaryTrees - Mar 31st 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A95049D3-82CB-4810-B6A5-2B9CC7567595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60156392-1C4E-4DDB-8360-19F0F83453EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="15" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="419">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="440">
   <si>
     <t>Statement</t>
   </si>
@@ -1364,6 +1364,69 @@
   </si>
   <si>
     <t>i = i/2 + (i &amp; 2)</t>
+  </si>
+  <si>
+    <t>1553. Minimum Number of Days to Eat N Oranges</t>
+  </si>
+  <si>
+    <t xml:space="preserve">use dfs </t>
+  </si>
+  <si>
+    <t>if n &lt;= 2 return 2</t>
+  </si>
+  <si>
+    <t>memo = n -&gt; 1 + Math.min(n%2 + dfs(n/2), n%3 + dfs(n/3))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">not using n-1 because above will do that </t>
+  </si>
+  <si>
+    <t>as n%2 -&gt; 1 if odd to get it to divisible by 2</t>
+  </si>
+  <si>
+    <t>and n%3 -&gt; 2 if odd to get divisible by 3</t>
+  </si>
+  <si>
+    <t>64. Minimum Path Sum</t>
+  </si>
+  <si>
+    <t>call dfs for down and left</t>
+  </si>
+  <si>
+    <t>return current + min of two</t>
+  </si>
+  <si>
+    <t>edge case - return last if reached</t>
+  </si>
+  <si>
+    <t>118. Pascal's Triangle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">add 1 to start </t>
+  </si>
+  <si>
+    <t>from index 1 add current and next</t>
+  </si>
+  <si>
+    <t>use the list</t>
+  </si>
+  <si>
+    <t>894. All Possible Full Binary Trees</t>
+  </si>
+  <si>
+    <t>if n == 0 return empty list</t>
+  </si>
+  <si>
+    <t>if n == 1 return list with 1 node</t>
+  </si>
+  <si>
+    <t>if n == odd :</t>
+  </si>
+  <si>
+    <t>for 0 - n-1 =&gt; left = i, right = n - i - 1 as 1 will be root</t>
+  </si>
+  <si>
+    <t>call dfs for both left and right and add them to node</t>
   </si>
 </sst>
 </file>
@@ -2924,6 +2987,182 @@
         <a:xfrm>
           <a:off x="4533900" y="37357050"/>
           <a:ext cx="1047896" cy="1105054"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>205</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4763141</xdr:colOff>
+      <xdr:row>212</xdr:row>
+      <xdr:rowOff>162130</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="23" name="Picture 22">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E38090F0-D8BD-4609-A01C-35A93AB47334}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId22"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3095625" y="39081075"/>
+          <a:ext cx="4591691" cy="1467055"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>409575</xdr:colOff>
+      <xdr:row>215</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4563055</xdr:colOff>
+      <xdr:row>218</xdr:row>
+      <xdr:rowOff>19130</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="24" name="Picture 23">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E93534CA-3450-47ED-ABCB-B4289B9705CA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId23"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3333750" y="40976550"/>
+          <a:ext cx="4153480" cy="571580"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>857250</xdr:colOff>
+      <xdr:row>222</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4077149</xdr:colOff>
+      <xdr:row>239</xdr:row>
+      <xdr:rowOff>29027</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="25" name="Picture 24">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3D42DCB4-5BF5-4BAA-8C58-92E8C47C2F7F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId24"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3781425" y="42319575"/>
+          <a:ext cx="3219899" cy="3238952"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>241</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4895850</xdr:colOff>
+      <xdr:row>258</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="26" name="Picture 25">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C569B4F9-2695-4B28-8F66-DDBF23046450}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId25"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2981325" y="45986700"/>
+          <a:ext cx="4838700" cy="3181350"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5710,10 +5949,10 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
-  <dimension ref="A1:D204"/>
+  <dimension ref="A1:D259"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="1" max="1" width="43.85546875" customWidth="1"/>
     <col min="2" max="2" width="73.85546875" customWidth="1"/>
     <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
     <col min="4" max="4" width="91.7109375" customWidth="1"/>
@@ -6495,6 +6734,150 @@
     </row>
     <row r="204" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C204" s="5"/>
+    </row>
+    <row r="205" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A205" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="D205" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="206" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D206" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="207" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D207" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="208" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D208" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="209" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D209" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="210" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D210" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="213" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D213" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="214" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C214" s="5"/>
+    </row>
+    <row r="215" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A215" s="13" t="s">
+        <v>426</v>
+      </c>
+      <c r="D215" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="216" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D216" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="217" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D217" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="218" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D218" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="219" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D219" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="220" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D220" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="221" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C221" s="5"/>
+    </row>
+    <row r="222" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A222" s="15" t="s">
+        <v>430</v>
+      </c>
+      <c r="D222" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="223" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D223" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="224" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D224" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="239" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D239" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="240" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C240" s="5"/>
+    </row>
+    <row r="241" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A241" s="13" t="s">
+        <v>434</v>
+      </c>
+      <c r="D241" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="242" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D242" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="243" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D243" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="244" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D244" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="245" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D245" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="246" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D246" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="258" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D258" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="259" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C259" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -6541,10 +6924,18 @@
     <hyperlink ref="D194" r:id="rId41" xr:uid="{511FE57E-DCE1-410D-BD38-C4F43E785E3A}"/>
     <hyperlink ref="A196" r:id="rId42" xr:uid="{33C8DB24-35DF-4AA2-A7F2-6187258CBF38}"/>
     <hyperlink ref="D203" r:id="rId43" xr:uid="{085A29C3-E8EF-48CF-8410-9E7F6639072E}"/>
+    <hyperlink ref="A205" r:id="rId44" xr:uid="{813FCDE1-72F2-43D4-BDD8-5EA88939285E}"/>
+    <hyperlink ref="D213" r:id="rId45" xr:uid="{334D45A7-5E3E-4B7B-B039-FB4C9DB3FF94}"/>
+    <hyperlink ref="A215" r:id="rId46" xr:uid="{BFDB1641-E185-4361-A607-7E35D1DC2942}"/>
+    <hyperlink ref="D220" r:id="rId47" xr:uid="{9DFF0154-2033-447C-ABD2-6993BC3F9B2E}"/>
+    <hyperlink ref="A222" r:id="rId48" xr:uid="{643AA764-BB96-4681-85CC-769DB0BA512E}"/>
+    <hyperlink ref="D239" r:id="rId49" xr:uid="{6DFAE2A3-5069-49EC-9925-1ECFC205F63E}"/>
+    <hyperlink ref="A241" r:id="rId50" xr:uid="{BC1C5EF6-04BE-48CD-AEEA-481B1878B9DC}"/>
+    <hyperlink ref="D258" r:id="rId51" xr:uid="{CA10B727-4FB1-4F67-97A8-E69093F24599}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId44"/>
-  <drawing r:id="rId45"/>
+  <pageSetup orientation="portrait" r:id="rId52"/>
+  <drawing r:id="rId53"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
BestTimetoBuyandSellStockwithCooldown - Mar 31 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60156392-1C4E-4DDB-8360-19F0F83453EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A86D22D-CB41-4156-887A-28D6420A0C04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="15" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="457">
   <si>
     <t>Statement</t>
   </si>
@@ -1427,6 +1427,57 @@
   </si>
   <si>
     <t>call dfs for both left and right and add them to node</t>
+  </si>
+  <si>
+    <t>746. Min Cost Climbing Stairs</t>
+  </si>
+  <si>
+    <t>call for min of len-1 and len-2</t>
+  </si>
+  <si>
+    <t>if n &lt; 0 return 0</t>
+  </si>
+  <si>
+    <t>if n is 0 or 1 =&gt; return cost[n]</t>
+  </si>
+  <si>
+    <t>dfs for cost[n] + min (n-1, n-2)</t>
+  </si>
+  <si>
+    <t>877. Stone Game</t>
+  </si>
+  <si>
+    <t>task is to find if alice gets &gt; sum/2</t>
+  </si>
+  <si>
+    <t>call dfs with i=0 and j=n-1</t>
+  </si>
+  <si>
+    <t>if i &gt; j return 0</t>
+  </si>
+  <si>
+    <t>declare a boolean isAliceTurn = (j - i + 1)%2 == 0</t>
+  </si>
+  <si>
+    <t>if alice turn call dfs using first element and last element =&gt; return max among them</t>
+  </si>
+  <si>
+    <t>309. Best Time to Buy and Sell Stock with Cooldown</t>
+  </si>
+  <si>
+    <t>call with start and isBuy as boolean</t>
+  </si>
+  <si>
+    <t xml:space="preserve">if isBuy </t>
+  </si>
+  <si>
+    <t>minus current + dfs for start+1, not Buy  or buy at next</t>
+  </si>
+  <si>
+    <t xml:space="preserve">else sell at here </t>
+  </si>
+  <si>
+    <t>plus current + dfs for start + 2 as cooldown requires a gap or sell at next</t>
   </si>
 </sst>
 </file>
@@ -3163,6 +3214,138 @@
         <a:xfrm>
           <a:off x="2981325" y="45986700"/>
           <a:ext cx="4838700" cy="3181350"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1076325</xdr:colOff>
+      <xdr:row>260</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3991382</xdr:colOff>
+      <xdr:row>264</xdr:row>
+      <xdr:rowOff>152525</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="27" name="Picture 26">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E041024E-FBEB-4E9F-B8B3-C87D7002069C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId26"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4000500" y="49549050"/>
+          <a:ext cx="2915057" cy="895475"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>268</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4857750</xdr:colOff>
+      <xdr:row>276</xdr:row>
+      <xdr:rowOff>207</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="28" name="Picture 27">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C11FB259-6DDA-4B75-B6A5-79780F5EAD7B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId27"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2962275" y="51092100"/>
+          <a:ext cx="4819650" cy="1486107"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>600075</xdr:colOff>
+      <xdr:row>278</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4382028</xdr:colOff>
+      <xdr:row>281</xdr:row>
+      <xdr:rowOff>77</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="29" name="Picture 28">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F05D1BF0-A92E-4570-AD35-51ABF36A84E5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId28"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3638550" y="52978050"/>
+          <a:ext cx="3781953" cy="552527"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5949,10 +6132,10 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
-  <dimension ref="A1:D259"/>
+  <dimension ref="A1:D285"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="43.85546875" customWidth="1"/>
+    <col min="1" max="1" width="45.5703125" customWidth="1"/>
     <col min="2" max="2" width="73.85546875" customWidth="1"/>
     <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
     <col min="4" max="4" width="91.7109375" customWidth="1"/>
@@ -6871,13 +7054,126 @@
         <v>439</v>
       </c>
     </row>
-    <row r="258" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D258" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="259" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C259" s="5"/>
+    </row>
+    <row r="260" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A260" s="15" t="s">
+        <v>440</v>
+      </c>
+      <c r="D260" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="261" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D261" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="262" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D262" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="263" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D263" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="264" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D264" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="266" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D266" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="267" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C267" s="5"/>
+    </row>
+    <row r="268" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A268" s="13" t="s">
+        <v>445</v>
+      </c>
+      <c r="D268" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="269" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D269" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="270" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D270" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="271" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D271" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="272" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D272" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="276" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D276" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="277" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C277" s="5"/>
+    </row>
+    <row r="278" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A278" s="13" t="s">
+        <v>451</v>
+      </c>
+      <c r="D278" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="279" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D279" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="280" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D280" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="281" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D281" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="282" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D282" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="283" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D283" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="284" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D284" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="285" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C285" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -6932,10 +7228,16 @@
     <hyperlink ref="D239" r:id="rId49" xr:uid="{6DFAE2A3-5069-49EC-9925-1ECFC205F63E}"/>
     <hyperlink ref="A241" r:id="rId50" xr:uid="{BC1C5EF6-04BE-48CD-AEEA-481B1878B9DC}"/>
     <hyperlink ref="D258" r:id="rId51" xr:uid="{CA10B727-4FB1-4F67-97A8-E69093F24599}"/>
+    <hyperlink ref="A260" r:id="rId52" xr:uid="{EEB38988-4DFD-488C-8BEC-D357D7443E6A}"/>
+    <hyperlink ref="D266" r:id="rId53" xr:uid="{5CEB5CD5-DBF2-4064-9169-6F253C83AEDA}"/>
+    <hyperlink ref="A268" r:id="rId54" xr:uid="{E8300B63-8607-4507-A0C3-67C9AA08927A}"/>
+    <hyperlink ref="D276" r:id="rId55" xr:uid="{93B7C95F-272C-48E7-BBB9-31457ECAC32B}"/>
+    <hyperlink ref="A278" r:id="rId56" xr:uid="{290845DF-25B5-43FF-9BB5-90E2E5CCDD7F}"/>
+    <hyperlink ref="D284" r:id="rId57" xr:uid="{8C9BD488-C3CA-458E-8BDE-5ACF645C6262}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId52"/>
-  <drawing r:id="rId53"/>
+  <pageSetup orientation="portrait" r:id="rId58"/>
+  <drawing r:id="rId59"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
graphs - April 6th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A86D22D-CB41-4156-887A-28D6420A0C04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0C43D37-AB9A-4209-854C-734E64039FF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="15" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="457">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="463">
   <si>
     <t>Statement</t>
   </si>
@@ -1478,6 +1478,24 @@
   </si>
   <si>
     <t>plus current + dfs for start + 2 as cooldown requires a gap or sell at next</t>
+  </si>
+  <si>
+    <t>343. Integer Break</t>
+  </si>
+  <si>
+    <t>n == 3 =&gt; 2</t>
+  </si>
+  <si>
+    <t>n == 10 =&gt; 3 + 3 + 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">while n changes from initial value we can keep </t>
+  </si>
+  <si>
+    <t>min as n (we don't have to split it)</t>
+  </si>
+  <si>
+    <t>for each i &lt;  n call dfs for i and n - i</t>
   </si>
 </sst>
 </file>
@@ -3346,6 +3364,50 @@
         <a:xfrm>
           <a:off x="3638550" y="52978050"/>
           <a:ext cx="3781953" cy="552527"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>914400</xdr:colOff>
+      <xdr:row>286</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3877088</xdr:colOff>
+      <xdr:row>297</xdr:row>
+      <xdr:rowOff>114603</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="31" name="Picture 30">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2BD4233A-D6AA-41D0-8AB6-9EA9AB452F6B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId29"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3952875" y="54521100"/>
+          <a:ext cx="2962688" cy="2172003"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6132,7 +6194,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
-  <dimension ref="A1:D285"/>
+  <dimension ref="A1:D298"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45.5703125" customWidth="1"/>
@@ -7174,6 +7236,43 @@
     </row>
     <row r="285" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C285" s="5"/>
+    </row>
+    <row r="286" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A286" s="13" t="s">
+        <v>457</v>
+      </c>
+      <c r="C286" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="D286" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="287" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C287" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="D287" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="288" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C288" s="1" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="289" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C289" s="1" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="297" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D297" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="298" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C298" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -7234,10 +7333,12 @@
     <hyperlink ref="D276" r:id="rId55" xr:uid="{93B7C95F-272C-48E7-BBB9-31457ECAC32B}"/>
     <hyperlink ref="A278" r:id="rId56" xr:uid="{290845DF-25B5-43FF-9BB5-90E2E5CCDD7F}"/>
     <hyperlink ref="D284" r:id="rId57" xr:uid="{8C9BD488-C3CA-458E-8BDE-5ACF645C6262}"/>
+    <hyperlink ref="A286" r:id="rId58" xr:uid="{07895363-8E1D-4116-81C2-518ED1B24D0E}"/>
+    <hyperlink ref="D297" r:id="rId59" xr:uid="{FA74ABFB-C411-4F4B-B1EA-5857007451A4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId58"/>
-  <drawing r:id="rId59"/>
+  <pageSetup orientation="portrait" r:id="rId60"/>
+  <drawing r:id="rId61"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
7th April 2022 - WordLadder
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25028"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0C43D37-AB9A-4209-854C-734E64039FF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF0B0600-AC43-4F11-B3A6-BF15B3B3669A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="15" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="9" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="463">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="469">
   <si>
     <t>Statement</t>
   </si>
@@ -1496,6 +1496,24 @@
   </si>
   <si>
     <t>for each i &lt;  n call dfs for i and n - i</t>
+  </si>
+  <si>
+    <t>127. Word Ladder</t>
+  </si>
+  <si>
+    <t>use BFS</t>
+  </si>
+  <si>
+    <t>find all transforms of current transformed set - i.e. a-z for all indexes</t>
+  </si>
+  <si>
+    <t>create a transformed set - init with beginWord</t>
+  </si>
+  <si>
+    <t>if any transform is in wordSet add it to newTransform set - which we'll point to ald transform set after checking for all</t>
+  </si>
+  <si>
+    <t>do this till we find endWord in transform set or newTransform is empty</t>
   </si>
 </sst>
 </file>
@@ -5130,6 +5148,50 @@
         <a:xfrm>
           <a:off x="2838451" y="18488025"/>
           <a:ext cx="4876800" cy="2838846"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>114</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4905375</xdr:colOff>
+      <xdr:row>117</xdr:row>
+      <xdr:rowOff>171550</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{60A39EF4-22B6-4A41-8ACA-FBBF4A4D89DE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2857500" y="21745575"/>
+          <a:ext cx="4867275" cy="714475"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5507,13 +5569,13 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E87A3A0-D815-41F9-954B-826D58641E2B}">
-  <dimension ref="A1:D113"/>
+  <dimension ref="A1:D121"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
     <col min="2" max="2" width="73.85546875" customWidth="1"/>
     <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="4" max="4" width="103.5703125" customWidth="1"/>
     <col min="13" max="13" width="6.7109375" customWidth="1"/>
     <col min="14" max="14" width="8.5703125" customWidth="1"/>
   </cols>
@@ -5727,8 +5789,44 @@
         <v>9</v>
       </c>
     </row>
-    <row r="113" spans="3:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C113" s="5"/>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A114" s="14" t="s">
+        <v>463</v>
+      </c>
+      <c r="D114" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D115" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D116" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D117" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D118" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D120" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C121" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -5746,10 +5844,12 @@
     <hyperlink ref="D95" r:id="rId12" xr:uid="{8872328D-61D7-4547-8FF7-479ED08BFBCC}"/>
     <hyperlink ref="A97" r:id="rId13" xr:uid="{FFC83952-6DF4-4D2B-9794-7BE41DB5095E}"/>
     <hyperlink ref="D111" r:id="rId14" xr:uid="{3EE638A9-17A4-457C-9C53-D2E84457850F}"/>
+    <hyperlink ref="A114" r:id="rId15" xr:uid="{5883B364-0547-4DEE-A083-E8C5AD44B8DA}"/>
+    <hyperlink ref="D120" r:id="rId16" xr:uid="{5B9A9308-2E60-45F9-8E47-F28B42801351}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId15"/>
-  <drawing r:id="rId16"/>
+  <pageSetup orientation="portrait" r:id="rId17"/>
+  <drawing r:id="rId18"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
PacificAtlanticWaterFlow - Apr 9th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF0B0600-AC43-4F11-B3A6-BF15B3B3669A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F930B8B-41FD-4ACF-8117-DE9B41DD5503}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="9" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="474">
   <si>
     <t>Statement</t>
   </si>
@@ -1514,6 +1514,21 @@
   </si>
   <si>
     <t>do this till we find endWord in transform set or newTransform is empty</t>
+  </si>
+  <si>
+    <t>417. Pacific Atlantic Water Flow</t>
+  </si>
+  <si>
+    <t>start from 4 sides and add if any cells reach pacific or atlantic</t>
+  </si>
+  <si>
+    <t>i.e. dfs from 0th row will find all cells reaching pacific</t>
+  </si>
+  <si>
+    <t>add cells to pacific set</t>
+  </si>
+  <si>
+    <t>finally take conjunction of pacific and atlantic set</t>
   </si>
 </sst>
 </file>
@@ -5192,6 +5207,50 @@
         <a:xfrm>
           <a:off x="2857500" y="21745575"/>
           <a:ext cx="4867275" cy="714475"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>95251</xdr:colOff>
+      <xdr:row>122</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4857750</xdr:colOff>
+      <xdr:row>151</xdr:row>
+      <xdr:rowOff>19821</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4E4E6FA5-5F05-408D-AA76-F6652CDBF762}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2914651" y="23260050"/>
+          <a:ext cx="4762499" cy="5525271"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5569,7 +5628,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E87A3A0-D815-41F9-954B-826D58641E2B}">
-  <dimension ref="A1:D121"/>
+  <dimension ref="A1:D152"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -5827,6 +5886,42 @@
     </row>
     <row r="121" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C121" s="5"/>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A122" s="13" t="s">
+        <v>469</v>
+      </c>
+      <c r="D122" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D123" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D124" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D125" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D127" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="151" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D151" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="152" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C152" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -5846,10 +5941,12 @@
     <hyperlink ref="D111" r:id="rId14" xr:uid="{3EE638A9-17A4-457C-9C53-D2E84457850F}"/>
     <hyperlink ref="A114" r:id="rId15" xr:uid="{5883B364-0547-4DEE-A083-E8C5AD44B8DA}"/>
     <hyperlink ref="D120" r:id="rId16" xr:uid="{5B9A9308-2E60-45F9-8E47-F28B42801351}"/>
+    <hyperlink ref="A122" r:id="rId17" xr:uid="{18422908-9300-4EE6-ACE5-39C538727C2D}"/>
+    <hyperlink ref="D151" r:id="rId18" xr:uid="{E1BF700E-EF66-4530-8D26-D16D6426F368}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId17"/>
-  <drawing r:id="rId18"/>
+  <pageSetup orientation="portrait" r:id="rId19"/>
+  <drawing r:id="rId20"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Apr 11th - 2022, WordSearch
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F930B8B-41FD-4ACF-8117-DE9B41DD5503}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B05939ED-D4CF-4BF2-87C6-A5F8C67A829C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="9" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="474">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="480">
   <si>
     <t>Statement</t>
   </si>
@@ -1529,6 +1529,24 @@
   </si>
   <si>
     <t>finally take conjunction of pacific and atlantic set</t>
+  </si>
+  <si>
+    <t>79. Word Search</t>
+  </si>
+  <si>
+    <t>iterate m*n indexes to find first match</t>
+  </si>
+  <si>
+    <t>if idx == word.length return true</t>
+  </si>
+  <si>
+    <t>if first matched find dfs with idx = 0, i=0, j=0</t>
+  </si>
+  <si>
+    <t>if inbounds and char at i,j != word[idx] return true</t>
+  </si>
+  <si>
+    <t>call dfs on all 4 sides (make word[i][j] = ' ' before and set later - backtrack to avoid loop or false positive)</t>
   </si>
 </sst>
 </file>
@@ -5251,6 +5269,50 @@
         <a:xfrm>
           <a:off x="2914651" y="23260050"/>
           <a:ext cx="4762499" cy="5525271"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>153</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4791075</xdr:colOff>
+      <xdr:row>167</xdr:row>
+      <xdr:rowOff>86095</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BD955182-1C37-4A51-B1FF-8EFC33B71113}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2914650" y="29251275"/>
+          <a:ext cx="4695825" cy="2648320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5628,7 +5690,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E87A3A0-D815-41F9-954B-826D58641E2B}">
-  <dimension ref="A1:D152"/>
+  <dimension ref="A1:D169"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -5915,13 +5977,54 @@
         <v>473</v>
       </c>
     </row>
-    <row r="151" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D151" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="152" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C152" s="5"/>
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A153" s="13" t="s">
+        <v>474</v>
+      </c>
+      <c r="D153" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D154" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D155" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D156" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D157" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D158" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="168" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D168" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="169" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C169" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -5943,10 +6046,12 @@
     <hyperlink ref="D120" r:id="rId16" xr:uid="{5B9A9308-2E60-45F9-8E47-F28B42801351}"/>
     <hyperlink ref="A122" r:id="rId17" xr:uid="{18422908-9300-4EE6-ACE5-39C538727C2D}"/>
     <hyperlink ref="D151" r:id="rId18" xr:uid="{E1BF700E-EF66-4530-8D26-D16D6426F368}"/>
+    <hyperlink ref="A153" r:id="rId19" xr:uid="{4AEC5EBB-1857-4C61-B7F1-20E90FF745CC}"/>
+    <hyperlink ref="D168" r:id="rId20" xr:uid="{C1167FED-6135-4C66-94EF-863171E02AE8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId19"/>
-  <drawing r:id="rId20"/>
+  <pageSetup orientation="portrait" r:id="rId21"/>
+  <drawing r:id="rId22"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
april 13th 2022 - ReorderRoutestoMakeAllPathsLeadtotheCityZero
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B05939ED-D4CF-4BF2-87C6-A5F8C67A829C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EFD9D4D-9FC3-47FE-925F-CE4F07050327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="9" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="480">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="660" uniqueCount="489">
   <si>
     <t>Statement</t>
   </si>
@@ -1547,6 +1547,33 @@
   </si>
   <si>
     <t>call dfs on all 4 sides (make word[i][j] = ' ' before and set later - backtrack to avoid loop or false positive)</t>
+  </si>
+  <si>
+    <t>1466. Reorder Routes to Make All Paths Lead to the City Zero</t>
+  </si>
+  <si>
+    <t>create adj with  1 -&gt; 2 means 1 to 2 ans 2 -&gt; -1 means 1 to 2</t>
+  </si>
+  <si>
+    <t>if visited return 0</t>
+  </si>
+  <si>
+    <t>else</t>
+  </si>
+  <si>
+    <t>add current vertex to visited</t>
+  </si>
+  <si>
+    <t>call dfs v=0 with visited set</t>
+  </si>
+  <si>
+    <t>for all its neighbours</t>
+  </si>
+  <si>
+    <t>add 1 to changed if they are in positive (because we are moving far from 0 -&gt; positive means should change direction)</t>
+  </si>
+  <si>
+    <t>call dfs for neighbor</t>
   </si>
 </sst>
 </file>
@@ -5313,6 +5340,50 @@
         <a:xfrm>
           <a:off x="2914650" y="29251275"/>
           <a:ext cx="4695825" cy="2648320"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>85725</xdr:colOff>
+      <xdr:row>170</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4781550</xdr:colOff>
+      <xdr:row>183</xdr:row>
+      <xdr:rowOff>124179</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Picture 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D4227938-2A3F-4A13-9E2A-DA967BDD95B8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3657600" y="32451675"/>
+          <a:ext cx="4695825" cy="2534004"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5690,10 +5761,10 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E87A3A0-D815-41F9-954B-826D58641E2B}">
-  <dimension ref="A1:D169"/>
+  <dimension ref="A1:D185"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="1" max="1" width="45.85546875" customWidth="1"/>
     <col min="2" max="2" width="73.85546875" customWidth="1"/>
     <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
     <col min="4" max="4" width="103.5703125" customWidth="1"/>
@@ -6018,13 +6089,64 @@
         <v>479</v>
       </c>
     </row>
-    <row r="168" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D168" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="169" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C169" s="5"/>
+    </row>
+    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A170" s="13" t="s">
+        <v>480</v>
+      </c>
+      <c r="D170" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D171" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D172" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D173" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D174" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D175" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D176" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="177" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D177" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="184" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D184" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="185" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C185" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -6048,10 +6170,12 @@
     <hyperlink ref="D151" r:id="rId18" xr:uid="{E1BF700E-EF66-4530-8D26-D16D6426F368}"/>
     <hyperlink ref="A153" r:id="rId19" xr:uid="{4AEC5EBB-1857-4C61-B7F1-20E90FF745CC}"/>
     <hyperlink ref="D168" r:id="rId20" xr:uid="{C1167FED-6135-4C66-94EF-863171E02AE8}"/>
+    <hyperlink ref="A170" r:id="rId21" xr:uid="{B99FBD60-EEEB-406D-93B1-4A82D01C21EB}"/>
+    <hyperlink ref="D184" r:id="rId22" xr:uid="{F5AE28A4-CA7C-4221-881E-BE3AA9433D50}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId21"/>
-  <drawing r:id="rId22"/>
+  <pageSetup orientation="portrait" r:id="rId23"/>
+  <drawing r:id="rId24"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
April16th 2022 - WordSearchII
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDD89F7D-E91F-4062-8182-53497F51BFE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52605163-097E-4B54-B24A-85590A103B18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" activeTab="9" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="503">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="511">
   <si>
     <t>Statement</t>
   </si>
@@ -1616,6 +1616,30 @@
   </si>
   <si>
     <t>684. Redundant Connection</t>
+  </si>
+  <si>
+    <t>212. Word Search II</t>
+  </si>
+  <si>
+    <t>create Trie for all words</t>
+  </si>
+  <si>
+    <t>for each letter in matrix call dfs</t>
+  </si>
+  <si>
+    <t>return if not inbounds or current char is *</t>
+  </si>
+  <si>
+    <t>add current char to str</t>
+  </si>
+  <si>
+    <t>dfs i,  j, str=""</t>
+  </si>
+  <si>
+    <t>return if trie doesn't have str, add to res if str is present</t>
+  </si>
+  <si>
+    <t>recurse all 4 sides (trackback with * for avoiding cycles)</t>
   </si>
 </sst>
 </file>
@@ -5472,6 +5496,50 @@
         <a:xfrm>
           <a:off x="3095625" y="35490150"/>
           <a:ext cx="4876800" cy="2771775"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>203</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4886325</xdr:colOff>
+      <xdr:row>221</xdr:row>
+      <xdr:rowOff>143367</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Picture 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0646556D-69B7-4B0E-9BDD-BAFE0A9B358B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3114675" y="38719125"/>
+          <a:ext cx="4829175" cy="3524742"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5849,7 +5917,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E87A3A0-D815-41F9-954B-826D58641E2B}">
-  <dimension ref="A1:D202"/>
+  <dimension ref="A1:D223"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45.85546875" customWidth="1"/>
@@ -6284,33 +6352,79 @@
         <v>496</v>
       </c>
     </row>
-    <row r="193" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D193" t="s">
         <v>497</v>
       </c>
     </row>
-    <row r="194" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D194" t="s">
         <v>498</v>
       </c>
     </row>
-    <row r="195" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D195" t="s">
         <v>500</v>
       </c>
     </row>
-    <row r="196" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D196" t="s">
         <v>499</v>
       </c>
     </row>
-    <row r="201" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D201" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="202" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C202" s="5"/>
+    </row>
+    <row r="203" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A203" s="14" t="s">
+        <v>503</v>
+      </c>
+      <c r="D203" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="204" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D204" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="205" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D205" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="206" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D206" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="207" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D207" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="208" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D208" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="209" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D209" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="222" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D222" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="223" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C223" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -6341,10 +6455,12 @@
     <hyperlink ref="D201" r:id="rId25" xr:uid="{BC0BA31D-AB96-433F-AC27-1A2A21D063D8}"/>
     <hyperlink ref="C187" r:id="rId26" xr:uid="{40FCD56A-49F4-4E23-B056-A8720EFE565E}"/>
     <hyperlink ref="C188" r:id="rId27" xr:uid="{3559E797-6B4E-4E5D-BE6A-16C6DDBB1A99}"/>
+    <hyperlink ref="A203" r:id="rId28" xr:uid="{30F69B60-91AB-47CC-90C1-3046AB318383}"/>
+    <hyperlink ref="D222" r:id="rId29" xr:uid="{8B7A0763-215F-4803-A93D-BA9ECF465E5F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId28"/>
-  <drawing r:id="rId29"/>
+  <pageSetup orientation="portrait" r:id="rId30"/>
+  <drawing r:id="rId31"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
17th Apr 2022 - SwiminRisingWater
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52605163-097E-4B54-B24A-85590A103B18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4DEFC37-83DA-4189-A7E4-A70289A6644F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" activeTab="9" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="511">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="523">
   <si>
     <t>Statement</t>
   </si>
@@ -1640,6 +1640,42 @@
   </si>
   <si>
     <t>recurse all 4 sides (trackback with * for avoiding cycles)</t>
+  </si>
+  <si>
+    <t>1905. Count Sub Islands</t>
+  </si>
+  <si>
+    <t>start dfs if grid2 has 1 and non-visited</t>
+  </si>
+  <si>
+    <t>dfs i, j</t>
+  </si>
+  <si>
+    <t>if out of bounds or grid2[i][j] == 0 return true</t>
+  </si>
+  <si>
+    <t>since grid2 has 1, if grid1 has 0 return false</t>
+  </si>
+  <si>
+    <t>do dfs on 4 sides completely as we want to cover all indexes</t>
+  </si>
+  <si>
+    <t>778. Swim in Rising Water</t>
+  </si>
+  <si>
+    <t>use priority queue -minHeap (maxElevation, row, col)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">remove top </t>
+  </si>
+  <si>
+    <t>endcase</t>
+  </si>
+  <si>
+    <t>if row &amp; col reach n-1, n-1 then return weight</t>
+  </si>
+  <si>
+    <t>add from all its 4 directions - (maxtillNow, nextrow, nextcol) - check outofbounds before adding</t>
   </si>
 </sst>
 </file>
@@ -5540,6 +5576,94 @@
         <a:xfrm>
           <a:off x="3114675" y="38719125"/>
           <a:ext cx="4829175" cy="3524742"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>224</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4800600</xdr:colOff>
+      <xdr:row>239</xdr:row>
+      <xdr:rowOff>143284</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Picture 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B968BC98-AF7F-4A32-AE72-6A93ADE943CF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3124200" y="42738675"/>
+          <a:ext cx="4733925" cy="2934109"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>242</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4886325</xdr:colOff>
+      <xdr:row>254</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Picture 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A7D8D6BC-8A8E-45F0-888F-608B517BA22C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3086100" y="46167675"/>
+          <a:ext cx="4857750" cy="2238375"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5917,7 +6041,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E87A3A0-D815-41F9-954B-826D58641E2B}">
-  <dimension ref="A1:D223"/>
+  <dimension ref="A1:D255"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45.85546875" customWidth="1"/>
@@ -6413,18 +6537,95 @@
         <v>509</v>
       </c>
     </row>
-    <row r="209" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D209" t="s">
         <v>510</v>
       </c>
     </row>
-    <row r="222" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D222" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="223" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C223" s="5"/>
+    </row>
+    <row r="224" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A224" s="13" t="s">
+        <v>511</v>
+      </c>
+      <c r="D224" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="225" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D225" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="226" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D226" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="227" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D227" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="228" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D228" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="240" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D240" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="241" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C241" s="5"/>
+    </row>
+    <row r="242" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A242" s="14" t="s">
+        <v>517</v>
+      </c>
+      <c r="D242" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="243" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D243" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="244" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D244" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="245" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D245" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="246" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D246" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="247" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D247" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="254" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D254" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="255" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C255" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -6457,10 +6658,14 @@
     <hyperlink ref="C188" r:id="rId27" xr:uid="{3559E797-6B4E-4E5D-BE6A-16C6DDBB1A99}"/>
     <hyperlink ref="A203" r:id="rId28" xr:uid="{30F69B60-91AB-47CC-90C1-3046AB318383}"/>
     <hyperlink ref="D222" r:id="rId29" xr:uid="{8B7A0763-215F-4803-A93D-BA9ECF465E5F}"/>
+    <hyperlink ref="A224" r:id="rId30" xr:uid="{E677433C-0F25-4705-988B-294731FA1D56}"/>
+    <hyperlink ref="D240" r:id="rId31" xr:uid="{883C3C91-146C-405D-B816-2AF87712403E}"/>
+    <hyperlink ref="A242" r:id="rId32" xr:uid="{D2D391B6-840C-44EB-A74D-EE8C8039341C}"/>
+    <hyperlink ref="D254" r:id="rId33" xr:uid="{78DC200C-E07B-43F2-AEF3-6EBDA0D042AC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId30"/>
-  <drawing r:id="rId31"/>
+  <pageSetup orientation="portrait" r:id="rId34"/>
+  <drawing r:id="rId35"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
18th April 2022 - RottingOranges
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD5F08DD-3A69-4E64-9008-D1717E8099A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3029348A-1368-43AD-B70F-382D1AD39A31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" activeTab="9" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="705" uniqueCount="527">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="539">
   <si>
     <t>Statement</t>
   </si>
@@ -1688,6 +1688,42 @@
   </si>
   <si>
     <t>call dfs on 4 sides and add to area</t>
+  </si>
+  <si>
+    <t>994. Rotting Oranges</t>
+  </si>
+  <si>
+    <t>bfs</t>
+  </si>
+  <si>
+    <t>add current fresh and rotten ones to 2 sets</t>
+  </si>
+  <si>
+    <t>while fresh are empty - for each minute take out possible fresh getting rotten from current rotten</t>
+  </si>
+  <si>
+    <t>newRotten becomes rotten now</t>
+  </si>
+  <si>
+    <t>at any point if newRotten is empty - means some fresh cannot be rotten</t>
+  </si>
+  <si>
+    <t>329. Longest Increasing Path in a Matrix</t>
+  </si>
+  <si>
+    <t>iterate all indices</t>
+  </si>
+  <si>
+    <t>dfs i, j, prev = -1</t>
+  </si>
+  <si>
+    <t>if out of bounds or current &lt;= prev, return 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">if cached return </t>
+  </si>
+  <si>
+    <t>init max = 1, find the max on 1 + all 4 directions</t>
   </si>
 </sst>
 </file>
@@ -5720,6 +5756,94 @@
         <a:xfrm>
           <a:off x="3114675" y="48806100"/>
           <a:ext cx="4743450" cy="2543175"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>272</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4905375</xdr:colOff>
+      <xdr:row>279</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Picture 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2E4FFD2E-2556-42FE-9857-8400169CCE07}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3076575" y="51825525"/>
+          <a:ext cx="4886325" cy="1476375"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>495300</xdr:colOff>
+      <xdr:row>282</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4401095</xdr:colOff>
+      <xdr:row>296</xdr:row>
+      <xdr:rowOff>143266</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="Picture 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D649ED91-3EF4-4464-BA5B-0C6A90C0C5BE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3552825" y="53730525"/>
+          <a:ext cx="3905795" cy="2800741"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6097,7 +6221,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E87A3A0-D815-41F9-954B-826D58641E2B}">
-  <dimension ref="A1:D271"/>
+  <dimension ref="A1:D298"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45.85546875" customWidth="1"/>
@@ -6691,23 +6815,95 @@
         <v>524</v>
       </c>
     </row>
-    <row r="257" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D257" t="s">
         <v>525</v>
       </c>
     </row>
-    <row r="258" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D258" t="s">
         <v>526</v>
       </c>
     </row>
-    <row r="270" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D270" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="271" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C271" s="5"/>
+    </row>
+    <row r="272" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A272" s="13" t="s">
+        <v>527</v>
+      </c>
+      <c r="D272" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="273" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D273" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="274" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D274" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="275" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D275" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="276" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D276" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="280" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D280" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="281" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C281" s="5"/>
+    </row>
+    <row r="282" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A282" s="14" t="s">
+        <v>533</v>
+      </c>
+      <c r="D282" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="283" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D283" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="284" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D284" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="285" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D285" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="286" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D286" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="297" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D297" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="298" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C298" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -6746,10 +6942,14 @@
     <hyperlink ref="D254" r:id="rId33" xr:uid="{78DC200C-E07B-43F2-AEF3-6EBDA0D042AC}"/>
     <hyperlink ref="A256" r:id="rId34" xr:uid="{A57E2B92-8D8F-466F-B082-6F4B35EA576F}"/>
     <hyperlink ref="D270" r:id="rId35" xr:uid="{83748603-B7B9-43B2-A36E-0A5FD228D90F}"/>
+    <hyperlink ref="A272" r:id="rId36" xr:uid="{7AD933DF-B23F-44D4-A088-337AD9776914}"/>
+    <hyperlink ref="D280" r:id="rId37" xr:uid="{BE07BF23-068F-4DE1-B128-262FB713EB09}"/>
+    <hyperlink ref="A282" r:id="rId38" xr:uid="{DD1DE91A-CC47-4CFA-BF31-9151AE92485A}"/>
+    <hyperlink ref="D297" r:id="rId39" xr:uid="{67C6FD54-EE22-419C-A9AF-70895311C893}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId36"/>
-  <drawing r:id="rId37"/>
+  <pageSetup orientation="portrait" r:id="rId40"/>
+  <drawing r:id="rId41"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
April 27th - 2022 - snakesAndLadders
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3029348A-1368-43AD-B70F-382D1AD39A31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{842DADEE-5D63-46BB-9A0F-88778000A8BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" activeTab="9" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" activeTab="10" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="539">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="547">
   <si>
     <t>Statement</t>
   </si>
@@ -1724,6 +1724,30 @@
   </si>
   <si>
     <t>init max = 1, find the max on 1 + all 4 directions</t>
+  </si>
+  <si>
+    <t>909. Snakes and Ladders</t>
+  </si>
+  <si>
+    <t>use queue [currentSquare, jumps]</t>
+  </si>
+  <si>
+    <t>init with [1, 0]</t>
+  </si>
+  <si>
+    <t>while queue is not empty - while adding all next 6 combinations, check</t>
+  </si>
+  <si>
+    <t>if not reached n^2</t>
+  </si>
+  <si>
+    <t>if ladder or snake</t>
+  </si>
+  <si>
+    <t>if not visited add next ones</t>
+  </si>
+  <si>
+    <t>Topological sorting</t>
   </si>
 </sst>
 </file>
@@ -5844,6 +5868,94 @@
         <a:xfrm>
           <a:off x="3552825" y="53730525"/>
           <a:ext cx="3905795" cy="2800741"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>299</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2847975</xdr:colOff>
+      <xdr:row>306</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="19" name="Picture 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EEBE657C-1B6A-4D05-87F5-BD8D07508341}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8010525" y="57016650"/>
+          <a:ext cx="2819400" cy="1400175"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>299</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4857750</xdr:colOff>
+      <xdr:row>320</xdr:row>
+      <xdr:rowOff>105343</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="20" name="Picture 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E9C2D92D-8FEB-4ED0-8BFD-F641865138D8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3086100" y="56997600"/>
+          <a:ext cx="4829175" cy="4067743"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6221,7 +6333,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E87A3A0-D815-41F9-954B-826D58641E2B}">
-  <dimension ref="A1:D298"/>
+  <dimension ref="A1:D322"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45.85546875" customWidth="1"/>
@@ -6897,13 +7009,59 @@
         <v>538</v>
       </c>
     </row>
-    <row r="297" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D297" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="298" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C298" s="5"/>
+    </row>
+    <row r="299" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A299" s="13" t="s">
+        <v>539</v>
+      </c>
+      <c r="D299" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="300" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D300" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="301" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D301" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="302" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D302" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="303" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D303" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="304" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D304" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="305" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D305" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="321" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D321" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="322" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C322" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -6946,10 +7104,12 @@
     <hyperlink ref="D280" r:id="rId37" xr:uid="{BE07BF23-068F-4DE1-B128-262FB713EB09}"/>
     <hyperlink ref="A282" r:id="rId38" xr:uid="{DD1DE91A-CC47-4CFA-BF31-9151AE92485A}"/>
     <hyperlink ref="D297" r:id="rId39" xr:uid="{67C6FD54-EE22-419C-A9AF-70895311C893}"/>
+    <hyperlink ref="A299" r:id="rId40" xr:uid="{BA8DDBEE-9C57-4B91-8079-9FEE4DB75B33}"/>
+    <hyperlink ref="D321" r:id="rId41" xr:uid="{6C86F891-320C-4279-B08D-7840657DD50D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId40"/>
-  <drawing r:id="rId41"/>
+  <pageSetup orientation="portrait" r:id="rId42"/>
+  <drawing r:id="rId43"/>
 </worksheet>
 </file>
 
@@ -7032,6 +7192,9 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C11" s="1" t="s">
+        <v>546</v>
+      </c>
       <c r="D11" t="s">
         <v>238</v>
       </c>

</xml_diff>

<commit_message>
May 1st 2022 - longestValidParentheses
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{842DADEE-5D63-46BB-9A0F-88778000A8BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67E41791-E6CD-4C0C-A67D-64A0488279E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" activeTab="10" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" activeTab="1" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="547">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="552">
   <si>
     <t>Statement</t>
   </si>
@@ -1748,6 +1748,21 @@
   </si>
   <si>
     <t>Topological sorting</t>
+  </si>
+  <si>
+    <t>32. Longest Valid Parentheses</t>
+  </si>
+  <si>
+    <t>dp[n]</t>
+  </si>
+  <si>
+    <t>for each parentheses, if ')' and -</t>
+  </si>
+  <si>
+    <t>dp[i-1] == '(' then dp[i] = 2 + dp[i-2]</t>
+  </si>
+  <si>
+    <t>else if charAt[i - dp[i-1] - 1] == ')' then dp[i] = dp[i-1] + dp[i-dp[i-1]-2] + 2</t>
   </si>
 </sst>
 </file>
@@ -2097,6 +2112,50 @@
         <a:xfrm>
           <a:off x="3181350" y="3867150"/>
           <a:ext cx="3829584" cy="485843"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4391590</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>38181</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A61B0CA3-859C-4F2C-A4F6-4B0B0E649A4A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3162300" y="5172075"/>
+          <a:ext cx="4048690" cy="581106"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -8892,7 +8951,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AAA3DB6-B181-432C-9183-F47857237DA8}">
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -9023,6 +9082,37 @@
     <row r="26" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C26" s="5"/>
     </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="14" t="s">
+        <v>547</v>
+      </c>
+      <c r="D27" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D28" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D29" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D30" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D32" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="3:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C33" s="5"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" xr:uid="{A24F529E-D0E4-4D7C-8940-2EF8A048917C}"/>
@@ -9031,9 +9121,11 @@
     <hyperlink ref="D18" r:id="rId4" xr:uid="{305DB711-02E8-46A6-A4B2-FBE63ADC1454}"/>
     <hyperlink ref="A20" r:id="rId5" xr:uid="{8CA448EC-D236-455D-8BAE-429EDAA19260}"/>
     <hyperlink ref="D25" r:id="rId6" xr:uid="{E0D5FDE7-5097-47AC-89CC-3DD086203364}"/>
+    <hyperlink ref="A27" r:id="rId7" xr:uid="{062EB6D1-B6C8-4E86-BC47-6B515EB90A7C}"/>
+    <hyperlink ref="D32" r:id="rId8" xr:uid="{AADFAA3D-E8F3-4A0F-8516-9B9143A6E576}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId7"/>
+  <drawing r:id="rId9"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
LowestCommonAncestorofaBinaryTree - May 3rd 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5108D2D3-7342-4C12-8B44-29B7D0A9B817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{199E6D4B-E760-44A6-907C-88D88D513750}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="16" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="741" uniqueCount="557">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="758" uniqueCount="572">
   <si>
     <t>Statement</t>
   </si>
@@ -1778,6 +1778,51 @@
   </si>
   <si>
     <t>else return root</t>
+  </si>
+  <si>
+    <t>236. Lowest Common Ancestor of a Binary Tree</t>
+  </si>
+  <si>
+    <t>recursive - dfs</t>
+  </si>
+  <si>
+    <t>if root is null or == left or == right, return root</t>
+  </si>
+  <si>
+    <t>take recursive result from left and right</t>
+  </si>
+  <si>
+    <t>if both are not null then return root</t>
+  </si>
+  <si>
+    <t>else return which is not null</t>
+  </si>
+  <si>
+    <t>iterative</t>
+  </si>
+  <si>
+    <t>create parent map till we have both elements parents</t>
+  </si>
+  <si>
+    <t>for p add all parents till root to a set</t>
+  </si>
+  <si>
+    <t>for q iterate till set has ancestor</t>
+  </si>
+  <si>
+    <t>2096. Step-By-Step Directions From a Binary Tree Node to Another</t>
+  </si>
+  <si>
+    <t>get root to start node and left node routes</t>
+  </si>
+  <si>
+    <t>trim prefix till lowest common ancestor</t>
+  </si>
+  <si>
+    <t>and append trimmed root to dest string</t>
+  </si>
+  <si>
+    <t>replace trimmed root to start string with U</t>
   </si>
 </sst>
 </file>
@@ -3829,6 +3874,94 @@
         <a:xfrm>
           <a:off x="3409950" y="3124200"/>
           <a:ext cx="3667637" cy="2286319"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>657225</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4410599</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>95573</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0D842A49-D771-64F0-F991-2E2C98CBECAC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3476625" y="5972175"/>
+          <a:ext cx="3753374" cy="2314898"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>466725</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4534468</xdr:colOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>133653</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30EABA92-CFBE-68B4-2A88-D5A60EF8E2D7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3286125" y="8820150"/>
+          <a:ext cx="4067743" cy="2172003"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -8825,7 +8958,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36268CC4-0AC5-4653-846F-9B607EC203E4}">
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D59"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -8897,28 +9030,118 @@
         <v>553</v>
       </c>
     </row>
-    <row r="17" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D17" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="18" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D18" t="s">
         <v>555</v>
       </c>
     </row>
-    <row r="19" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D19" t="s">
         <v>556</v>
       </c>
     </row>
-    <row r="29" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D29" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C30" s="5"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="13" t="s">
+        <v>557</v>
+      </c>
+      <c r="D31" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D32" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D33" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D34" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D35" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D36" s="4"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D37" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D38" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D39" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D40" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D44" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C45" s="5"/>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="13" t="s">
+        <v>567</v>
+      </c>
+      <c r="D46" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D47" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D48" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="49" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D49" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="58" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D58" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C59" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -8926,9 +9149,13 @@
     <hyperlink ref="D14" r:id="rId2" xr:uid="{16097345-4A31-47BC-92C1-D1A6FA33CDED}"/>
     <hyperlink ref="A16" r:id="rId3" xr:uid="{4EED7F04-D037-4FF2-B603-15D08ED992C6}"/>
     <hyperlink ref="D29" r:id="rId4" xr:uid="{89A86ED2-73BD-4675-852A-DB40234EFA26}"/>
+    <hyperlink ref="A31" r:id="rId5" xr:uid="{B05B6041-5A9E-4149-A338-71A512161B90}"/>
+    <hyperlink ref="D44" r:id="rId6" xr:uid="{4523B996-1EEE-47FD-BCC3-99CEC22CC731}"/>
+    <hyperlink ref="A46" r:id="rId7" xr:uid="{B34586CF-8F8E-44AA-8095-2C8B73B52E9A}"/>
+    <hyperlink ref="D58" r:id="rId8" xr:uid="{22300045-E647-415F-8A9A-969002EEDD97}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId5"/>
+  <drawing r:id="rId9"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
PartitiontoKEqualSumSubsets - May 5th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{199E6D4B-E760-44A6-907C-88D88D513750}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2429AF28-9F42-40F8-A26F-08370C424DDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="16" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="4" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="758" uniqueCount="572">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="766" uniqueCount="579">
   <si>
     <t>Statement</t>
   </si>
@@ -1823,6 +1823,27 @@
   </si>
   <si>
     <t>replace trimmed root to start string with U</t>
+  </si>
+  <si>
+    <t>698. Partition to K Equal Sum Subsets</t>
+  </si>
+  <si>
+    <t>if k == 0 return true</t>
+  </si>
+  <si>
+    <t>use trackback and keep visited set</t>
+  </si>
+  <si>
+    <t>dfs(start=0, k, target = avg i.e.(sum/k), currentSum)</t>
+  </si>
+  <si>
+    <t>if currentSum == taget call all over again with k-1</t>
+  </si>
+  <si>
+    <t>call dfs from start of each element</t>
+  </si>
+  <si>
+    <t>check currentSum + nums[i] before callling (should be less than target)</t>
   </si>
 </sst>
 </file>
@@ -4466,6 +4487,50 @@
         <a:xfrm>
           <a:off x="3419475" y="6877050"/>
           <a:ext cx="4886325" cy="628738"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4914900</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>104859</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{22FAFFAB-8026-0449-9C30-C2F4DD4F2DEA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3400425" y="8077200"/>
+          <a:ext cx="4905375" cy="600159"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -9669,7 +9734,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDA924A8-9114-46BA-B39C-6743F04F80F3}">
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50.85546875" customWidth="1"/>
@@ -9889,6 +9954,47 @@
     <row r="41" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C41" s="5"/>
     </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="13" t="s">
+        <v>572</v>
+      </c>
+      <c r="D42" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D43" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D44" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D45" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D46" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D47" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="49" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D49" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C50" s="5"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" display="Find First and Last Position of Element in Sorted Array" xr:uid="{1078431E-90B5-490C-89E2-631EC2FC986D}"/>
@@ -9902,9 +10008,11 @@
     <hyperlink ref="A23" r:id="rId9" xr:uid="{F16EB101-F0CB-48DB-8CC1-4B777907F79A}"/>
     <hyperlink ref="D40" r:id="rId10" xr:uid="{1392FFB3-5685-43A8-8CC5-71556F981E6A}"/>
     <hyperlink ref="A37" r:id="rId11" xr:uid="{E12E6C6B-5CBE-4336-9DD7-AB14B0F9585C}"/>
+    <hyperlink ref="A42" r:id="rId12" xr:uid="{8FB4A6A6-111C-48EE-A168-45CC4FAD248E}"/>
+    <hyperlink ref="D49" r:id="rId13" xr:uid="{EE41CC91-2B69-498C-8FCA-D221C021F81C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId12"/>
+  <drawing r:id="rId14"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
SizeOfMaxBSTInBinaryTree - Nay 8th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2429AF28-9F42-40F8-A26F-08370C424DDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{677D87F4-3120-45A4-BBB3-6CD2165D8B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="4" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="16" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="766" uniqueCount="579">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="584">
   <si>
     <t>Statement</t>
   </si>
@@ -1844,6 +1844,21 @@
   </si>
   <si>
     <t>check currentSum + nums[i] before callling (should be less than target)</t>
+  </si>
+  <si>
+    <t>98. Validate Binary Search Tree</t>
+  </si>
+  <si>
+    <t>dfs (max, min)</t>
+  </si>
+  <si>
+    <t>if root is null return true</t>
+  </si>
+  <si>
+    <t>if currNode.val &lt; min or &gt; max, return false</t>
+  </si>
+  <si>
+    <t>call dfs for left and right</t>
   </si>
 </sst>
 </file>
@@ -3983,6 +3998,50 @@
         <a:xfrm>
           <a:off x="3286125" y="8820150"/>
           <a:ext cx="4067743" cy="2172003"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>971550</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3734186</xdr:colOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>295</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1C3917B0-D601-AF6D-017A-C82904D7F218}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3790950" y="11410950"/>
+          <a:ext cx="2762636" cy="2114845"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -9023,7 +9082,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36268CC4-0AC5-4653-846F-9B607EC203E4}">
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:D72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -9195,18 +9254,49 @@
         <v>571</v>
       </c>
     </row>
-    <row r="49" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D49" t="s">
         <v>570</v>
       </c>
     </row>
-    <row r="58" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D58" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="59" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C59" s="5"/>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="13" t="s">
+        <v>579</v>
+      </c>
+      <c r="D60" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D61" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D62" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D63" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="71" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D71" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C72" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -9218,9 +9308,11 @@
     <hyperlink ref="D44" r:id="rId6" xr:uid="{4523B996-1EEE-47FD-BCC3-99CEC22CC731}"/>
     <hyperlink ref="A46" r:id="rId7" xr:uid="{B34586CF-8F8E-44AA-8095-2C8B73B52E9A}"/>
     <hyperlink ref="D58" r:id="rId8" xr:uid="{22300045-E647-415F-8A9A-969002EEDD97}"/>
+    <hyperlink ref="A60" r:id="rId9" xr:uid="{E71D1802-6DE8-472B-955E-068B2E908329}"/>
+    <hyperlink ref="D71" r:id="rId10" xr:uid="{E4D3E62A-5D0C-43E7-81E1-D06ADCFC6A65}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId9"/>
+  <drawing r:id="rId11"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
RotateArray - May 18th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{677D87F4-3120-45A4-BBB3-6CD2165D8B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC7C6101-10CE-49AD-96B4-EFC5ABB932FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="16" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="4" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="584">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="781" uniqueCount="590">
   <si>
     <t>Statement</t>
   </si>
@@ -1859,6 +1859,24 @@
   </si>
   <si>
     <t>call dfs for left and right</t>
+  </si>
+  <si>
+    <t>122. Best Time to Buy and Sell Stock II</t>
+  </si>
+  <si>
+    <t>if next is greater than current, add next and subtract current to profit</t>
+  </si>
+  <si>
+    <t>189. Rotate Array</t>
+  </si>
+  <si>
+    <t>reverse array</t>
+  </si>
+  <si>
+    <t>reverse 0, k-1</t>
+  </si>
+  <si>
+    <t>reverse k, n-1</t>
   </si>
 </sst>
 </file>
@@ -3825,6 +3843,50 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>299</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>303</xdr:row>
+      <xdr:rowOff>181101</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="30" name="Picture 29">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{56C7BB26-7F09-8A55-247C-EEDDDA3C6BB2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId30"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3076575" y="56997600"/>
+          <a:ext cx="4886325" cy="905001"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -4590,6 +4652,50 @@
         <a:xfrm>
           <a:off x="3400425" y="8077200"/>
           <a:ext cx="4905375" cy="600159"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>866775</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3810411</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>181133</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DA6027B5-B9A0-F602-8635-2F889C765AEA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4257675" y="9715500"/>
+          <a:ext cx="2943636" cy="1133633"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -7932,7 +8038,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
-  <dimension ref="A1:D298"/>
+  <dimension ref="A1:D305"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45.5703125" customWidth="1"/>
@@ -8999,18 +9105,39 @@
         <v>460</v>
       </c>
     </row>
-    <row r="289" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C289" s="1" t="s">
         <v>461</v>
       </c>
     </row>
-    <row r="297" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D297" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="298" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C298" s="5"/>
+    </row>
+    <row r="299" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A299" s="13" t="s">
+        <v>584</v>
+      </c>
+      <c r="D299" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="300" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D300" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="304" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D304" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="305" spans="3:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C305" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -9073,10 +9200,12 @@
     <hyperlink ref="D284" r:id="rId57" xr:uid="{8C9BD488-C3CA-458E-8BDE-5ACF645C6262}"/>
     <hyperlink ref="A286" r:id="rId58" xr:uid="{07895363-8E1D-4116-81C2-518ED1B24D0E}"/>
     <hyperlink ref="D297" r:id="rId59" xr:uid="{FA74ABFB-C411-4F4B-B1EA-5857007451A4}"/>
+    <hyperlink ref="A299" r:id="rId60" xr:uid="{1FCAE6AE-0B3F-47E1-9767-971F723B2E83}"/>
+    <hyperlink ref="D304" r:id="rId61" xr:uid="{4E6A4A67-63BB-4DA4-ACE0-DE299D79DF74}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId60"/>
-  <drawing r:id="rId61"/>
+  <pageSetup orientation="portrait" r:id="rId62"/>
+  <drawing r:id="rId63"/>
 </worksheet>
 </file>
 
@@ -9347,7 +9476,7 @@
       <c r="C2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="13" t="s">
         <v>288</v>
       </c>
       <c r="D3" t="s">
@@ -9826,7 +9955,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDA924A8-9114-46BA-B39C-6743F04F80F3}">
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50.85546875" customWidth="1"/>
@@ -10079,13 +10208,39 @@
         <v>578</v>
       </c>
     </row>
-    <row r="49" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D49" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="50" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C50" s="5"/>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="13" t="s">
+        <v>586</v>
+      </c>
+      <c r="D51" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D52" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D53" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D57" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C58" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -10102,9 +10257,11 @@
     <hyperlink ref="A37" r:id="rId11" xr:uid="{E12E6C6B-5CBE-4336-9DD7-AB14B0F9585C}"/>
     <hyperlink ref="A42" r:id="rId12" xr:uid="{8FB4A6A6-111C-48EE-A168-45CC4FAD248E}"/>
     <hyperlink ref="D49" r:id="rId13" xr:uid="{EE41CC91-2B69-498C-8FCA-D221C021F81C}"/>
+    <hyperlink ref="A51" r:id="rId14" xr:uid="{BE66F050-01A5-4862-90DF-2B9B4114BE8E}"/>
+    <hyperlink ref="D57" r:id="rId15" xr:uid="{D42D7A59-E6C3-4502-9E9E-BE38080EC9D1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId14"/>
+  <drawing r:id="rId16"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
CountGoodNodesinBinaryTree - May 19th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC7C6101-10CE-49AD-96B4-EFC5ABB932FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42D7EF8F-4964-45B8-8E24-0E6C23D43B90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="4" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="16" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="781" uniqueCount="590">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="786" uniqueCount="594">
   <si>
     <t>Statement</t>
   </si>
@@ -1877,6 +1877,18 @@
   </si>
   <si>
     <t>reverse k, n-1</t>
+  </si>
+  <si>
+    <t>1448. Count Good Nodes in Binary Tree</t>
+  </si>
+  <si>
+    <t>if root is null return 0</t>
+  </si>
+  <si>
+    <t>dfs root, maxInPath = Integer.MIN_VALUE</t>
+  </si>
+  <si>
+    <t>else return 1 if root.val &gt;= maxInPath else 0, and sum dfs of left and right children</t>
   </si>
 </sst>
 </file>
@@ -4104,6 +4116,50 @@
         <a:xfrm>
           <a:off x="3790950" y="11410950"/>
           <a:ext cx="2762636" cy="2114845"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1057275</xdr:colOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3657963</xdr:colOff>
+      <xdr:row>82</xdr:row>
+      <xdr:rowOff>181238</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A0EABD2C-82EB-1FA8-17B8-34D9A231978C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3876675" y="13916025"/>
+          <a:ext cx="2600688" cy="1886213"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -9211,7 +9267,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36268CC4-0AC5-4653-846F-9B607EC203E4}">
-  <dimension ref="A1:D72"/>
+  <dimension ref="A1:D84"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -9419,13 +9475,39 @@
         <v>583</v>
       </c>
     </row>
-    <row r="71" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D71" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="72" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C72" s="5"/>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" s="13" t="s">
+        <v>590</v>
+      </c>
+      <c r="D73" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D74" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D75" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="83" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D83" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C84" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -9439,9 +9521,11 @@
     <hyperlink ref="D58" r:id="rId8" xr:uid="{22300045-E647-415F-8A9A-969002EEDD97}"/>
     <hyperlink ref="A60" r:id="rId9" xr:uid="{E71D1802-6DE8-472B-955E-068B2E908329}"/>
     <hyperlink ref="D71" r:id="rId10" xr:uid="{E4D3E62A-5D0C-43E7-81E1-D06ADCFC6A65}"/>
+    <hyperlink ref="A73" r:id="rId11" xr:uid="{2EE4C200-CFE1-4C5B-9E3B-162FCF083A8E}"/>
+    <hyperlink ref="D83" r:id="rId12" xr:uid="{1559CE54-3E65-43EB-BF5B-D49C6184A518}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId11"/>
+  <drawing r:id="rId13"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
BasicCalculator - May 21st 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42D7EF8F-4964-45B8-8E24-0E6C23D43B90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CDC4F29-1373-4794-9B0F-06222CC1FCA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="16" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="17" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="786" uniqueCount="594">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="798" uniqueCount="604">
   <si>
     <t>Statement</t>
   </si>
@@ -1889,6 +1889,36 @@
   </si>
   <si>
     <t>else return 1 if root.val &gt;= maxInPath else 0, and sum dfs of left and right children</t>
+  </si>
+  <si>
+    <t>224. Basic Calculator</t>
+  </si>
+  <si>
+    <t>while loop till the end</t>
+  </si>
+  <si>
+    <t>if + sign = 1, if - sign = -1</t>
+  </si>
+  <si>
+    <t>if char is digit collect the number, put total += sign * number</t>
+  </si>
+  <si>
+    <t>if ( put current total to stack, and sign before (</t>
+  </si>
+  <si>
+    <t>if ), pop sign and multiply by current total (i.e. total in parenthesis)</t>
+  </si>
+  <si>
+    <t>then pop old total and add it to current total</t>
+  </si>
+  <si>
+    <t>227. Basic Calculator II</t>
+  </si>
+  <si>
+    <t>if prev operator is + or -, push num with sign to stack</t>
+  </si>
+  <si>
+    <t>if prev operator is * or /, push solved expression to stack</t>
   </si>
 </sst>
 </file>
@@ -4253,6 +4283,94 @@
         <a:xfrm>
           <a:off x="3381375" y="1743075"/>
           <a:ext cx="3867690" cy="628738"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1019175</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3610337</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>76575</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{811B344E-6837-A01F-FA45-82541185DDC5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3838575" y="3486150"/>
+          <a:ext cx="2591162" cy="2686425"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1419225</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3295912</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>57524</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{412BF0E3-B9B9-D686-3C88-769B47553381}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4238625" y="6715125"/>
+          <a:ext cx="1876687" cy="2676899"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -9531,7 +9649,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BDF4E8D-D4E1-4180-9015-2E66B34CBB41}">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -9623,8 +9741,70 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="3:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C17" s="5"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="14" t="s">
+        <v>594</v>
+      </c>
+      <c r="D18" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D19" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D20" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D21" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D22" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D23" t="s">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D33" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C34" s="5"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="13" t="s">
+        <v>601</v>
+      </c>
+      <c r="D35" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D36" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="49" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D49" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C50" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -9632,9 +9812,14 @@
     <hyperlink ref="D7" r:id="rId2" xr:uid="{B5902076-F258-44B7-A10E-28D7D53892DD}"/>
     <hyperlink ref="A9" r:id="rId3" xr:uid="{41CA7DEA-C842-4838-AA5B-416057A8B26C}"/>
     <hyperlink ref="D16" r:id="rId4" xr:uid="{7D78E185-BD0C-42CC-955B-A30BB33C24AE}"/>
+    <hyperlink ref="A18" r:id="rId5" xr:uid="{303D85E8-A243-45E0-AB2B-F650E00882D7}"/>
+    <hyperlink ref="D33" r:id="rId6" xr:uid="{20E93955-F6EE-4945-AF7A-5E21E68FD72A}"/>
+    <hyperlink ref="A35" r:id="rId7" xr:uid="{EBEB57E2-D61C-429F-9ED4-13410C4795F5}"/>
+    <hyperlink ref="D49" r:id="rId8" xr:uid="{E33833DE-847A-4DF8-93F7-4EAA9509A09E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId5"/>
+  <pageSetup orientation="portrait" r:id="rId9"/>
+  <drawing r:id="rId10"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
InfixToPostfix, InfixToPrefix, PostfixToExpressionTree - May 22nd 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CDC4F29-1373-4794-9B0F-06222CC1FCA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{824A7C0C-E61F-408F-ADC9-0D9A3B20257B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="17" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="4" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="798" uniqueCount="604">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="803" uniqueCount="608">
   <si>
     <t>Statement</t>
   </si>
@@ -1919,6 +1919,18 @@
   </si>
   <si>
     <t>if prev operator is * or /, push solved expression to stack</t>
+  </si>
+  <si>
+    <t>75. Sort Colors</t>
+  </si>
+  <si>
+    <t>declare 2 pointers zeroIndex=0, twoIndex=n-1</t>
+  </si>
+  <si>
+    <t>iterate while i&lt;=twoIndex</t>
+  </si>
+  <si>
+    <t>if nums[i]==0, swap it with zeroIndex++ and i++, similarly twoIndex--, not i++</t>
   </si>
 </sst>
 </file>
@@ -4338,15 +4350,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1419225</xdr:colOff>
+      <xdr:colOff>1304925</xdr:colOff>
       <xdr:row>35</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:rowOff>9525</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>3295912</xdr:colOff>
+      <xdr:colOff>3181612</xdr:colOff>
       <xdr:row>49</xdr:row>
-      <xdr:rowOff>57524</xdr:rowOff>
+      <xdr:rowOff>19424</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4369,7 +4381,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4238625" y="6715125"/>
+          <a:off x="4124325" y="6677025"/>
           <a:ext cx="1876687" cy="2676899"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4870,6 +4882,50 @@
         <a:xfrm>
           <a:off x="4257675" y="9715500"/>
           <a:ext cx="2943636" cy="1133633"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1200150</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3038732</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>76260</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{866B424D-FCDB-8B74-40DD-6E13462C3727}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4591050" y="11268075"/>
+          <a:ext cx="1838582" cy="428685"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -10224,7 +10280,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDA924A8-9114-46BA-B39C-6743F04F80F3}">
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50.85546875" customWidth="1"/>
@@ -10510,6 +10566,32 @@
     </row>
     <row r="58" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C58" s="5"/>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="13" t="s">
+        <v>604</v>
+      </c>
+      <c r="D59" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D60" t="s">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D61" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D62" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C63" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -10528,9 +10610,11 @@
     <hyperlink ref="D49" r:id="rId13" xr:uid="{EE41CC91-2B69-498C-8FCA-D221C021F81C}"/>
     <hyperlink ref="A51" r:id="rId14" xr:uid="{BE66F050-01A5-4862-90DF-2B9B4114BE8E}"/>
     <hyperlink ref="D57" r:id="rId15" xr:uid="{D42D7A59-E6C3-4502-9E9E-BE38080EC9D1}"/>
+    <hyperlink ref="A59" r:id="rId16" xr:uid="{015C1AC1-D3A1-414E-BCC0-D586E7FD26CA}"/>
+    <hyperlink ref="D62" r:id="rId17" xr:uid="{F43C7C50-4691-47C3-BA28-55C6EE02BB1B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId16"/>
+  <drawing r:id="rId18"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
update excel - May 25th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{824A7C0C-E61F-408F-ADC9-0D9A3B20257B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F4AA096-7732-4AE7-8501-1F852D5ADC16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="4" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="15" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="803" uniqueCount="608">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="613">
   <si>
     <t>Statement</t>
   </si>
@@ -1931,6 +1931,21 @@
   </si>
   <si>
     <t>if nums[i]==0, swap it with zeroIndex++ and i++, similarly twoIndex--, not i++</t>
+  </si>
+  <si>
+    <t>Intuitive</t>
+  </si>
+  <si>
+    <t>find product from left and right</t>
+  </si>
+  <si>
+    <t>and take max in each index</t>
+  </si>
+  <si>
+    <t xml:space="preserve">if zero at any point </t>
+  </si>
+  <si>
+    <t>reinitalize to 1</t>
   </si>
 </sst>
 </file>
@@ -8091,7 +8106,7 @@
       <c r="C2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="13" t="s">
         <v>225</v>
       </c>
       <c r="D3" t="s">
@@ -8297,7 +8312,7 @@
       <c r="C2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="13" t="s">
         <v>104</v>
       </c>
       <c r="D3" t="s">
@@ -8323,7 +8338,7 @@
       <c r="C8" s="5"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="14" t="s">
         <v>108</v>
       </c>
       <c r="D9" t="s">
@@ -8362,7 +8377,7 @@
       <c r="C17" s="5"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="13" t="s">
         <v>111</v>
       </c>
       <c r="D18" t="s">
@@ -8398,7 +8413,7 @@
       <c r="C32" s="5"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
+      <c r="A33" s="15" t="s">
         <v>261</v>
       </c>
       <c r="C33" s="1" t="s">
@@ -8445,7 +8460,7 @@
       <c r="C39" s="5"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="8" t="s">
+      <c r="A40" s="13" t="s">
         <v>264</v>
       </c>
       <c r="D40" t="s">
@@ -9432,10 +9447,11 @@
     <hyperlink ref="D297" r:id="rId59" xr:uid="{FA74ABFB-C411-4F4B-B1EA-5857007451A4}"/>
     <hyperlink ref="A299" r:id="rId60" xr:uid="{1FCAE6AE-0B3F-47E1-9767-971F723B2E83}"/>
     <hyperlink ref="D304" r:id="rId61" xr:uid="{4E6A4A67-63BB-4DA4-ACE0-DE299D79DF74}"/>
+    <hyperlink ref="D7" r:id="rId62" xr:uid="{440ECE85-1159-4668-8AED-B2DAB74583B5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId62"/>
-  <drawing r:id="rId63"/>
+  <pageSetup orientation="portrait" r:id="rId63"/>
+  <drawing r:id="rId64"/>
 </worksheet>
 </file>
 
@@ -10309,7 +10325,7 @@
       <c r="C2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="13" t="s">
         <v>156</v>
       </c>
       <c r="D3" t="s">
@@ -10404,23 +10420,40 @@
       <c r="A23" s="13" t="s">
         <v>321</v>
       </c>
+      <c r="C23" s="1" t="s">
+        <v>608</v>
+      </c>
       <c r="D23" t="s">
         <v>322</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C24" s="1" t="s">
+        <v>609</v>
+      </c>
       <c r="D24" t="s">
         <v>323</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C25" s="1" t="s">
+        <v>610</v>
+      </c>
       <c r="D25" t="s">
         <v>324</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C26" s="1" t="s">
+        <v>611</v>
+      </c>
       <c r="D26" t="s">
         <v>325</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C27" s="1" t="s">
+        <v>612</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -10595,7 +10628,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" display="Find First and Last Position of Element in Sorted Array" xr:uid="{1078431E-90B5-490C-89E2-631EC2FC986D}"/>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{1078431E-90B5-490C-89E2-631EC2FC986D}"/>
     <hyperlink ref="D7" r:id="rId2" xr:uid="{A82BE56D-8664-44EF-9D97-3B9B32089A10}"/>
     <hyperlink ref="A9" r:id="rId3" display="Median of Two Sorted Arrays" xr:uid="{E9DDCB05-35C4-411A-9E11-5D6F3CC3AF96}"/>
     <hyperlink ref="D21" r:id="rId4" xr:uid="{3402BAFA-50FF-4A91-9C05-9F6AEAC01303}"/>

</xml_diff>

<commit_message>
update excel - May 26th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F4AA096-7732-4AE7-8501-1F852D5ADC16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6A5A9CC-3FA9-4777-A191-3F4AC744D0B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="15" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -8491,7 +8491,7 @@
       <c r="C50" s="5"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="4" t="s">
+      <c r="A51" s="15" t="s">
         <v>268</v>
       </c>
       <c r="D51" t="s">
@@ -8517,7 +8517,7 @@
       <c r="C58" s="5"/>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="8" t="s">
+      <c r="A59" s="13" t="s">
         <v>271</v>
       </c>
       <c r="D59" t="s">
@@ -8546,7 +8546,7 @@
       <c r="C68" s="5"/>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="8" t="s">
+      <c r="A69" s="13" t="s">
         <v>275</v>
       </c>
       <c r="D69" t="s">
@@ -8567,7 +8567,7 @@
       <c r="C74" s="5"/>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="8" t="s">
+      <c r="A75" s="13" t="s">
         <v>278</v>
       </c>
       <c r="D75" t="s">
@@ -8601,7 +8601,7 @@
       <c r="C84" s="5"/>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="8" t="s">
+      <c r="A85" s="13" t="s">
         <v>283</v>
       </c>
       <c r="D85" t="s">
@@ -8692,7 +8692,7 @@
       <c r="C103" s="5"/>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A104" s="8" t="s">
+      <c r="A104" s="13" t="s">
         <v>311</v>
       </c>
       <c r="D104" t="s">
@@ -8726,7 +8726,7 @@
       <c r="C111" s="5"/>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A112" s="8" t="s">
+      <c r="A112" s="13" t="s">
         <v>342</v>
       </c>
       <c r="D112" t="s">

</xml_diff>

<commit_message>
May 27th 2022 - Update excel
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25225"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6A5A9CC-3FA9-4777-A191-3F4AC744D0B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99843D92-A11B-4EB5-9433-BF165035B802}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="15" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="1" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -1612,9 +1612,6 @@
     <t>if not equal - make one with higher rank parent of other, return 1 (means no common nodes)</t>
   </si>
   <si>
-    <t>same problem</t>
-  </si>
-  <si>
     <t>684. Redundant Connection</t>
   </si>
   <si>
@@ -1946,6 +1943,9 @@
   </si>
   <si>
     <t>reinitalize to 1</t>
+  </si>
+  <si>
+    <t>similar problem</t>
   </si>
 </sst>
 </file>
@@ -2140,16 +2140,16 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="4"/>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="5"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="4" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="6"/>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="2" xfId="7"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="3" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="3" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="3" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="3" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="3" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="3" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="Bad" xfId="5" builtinId="27"/>
@@ -5226,94 +5226,6 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>47625</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>4886325</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>9243</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C9F7CC6B-BDB7-4468-864C-90E88BE74687}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2867025" y="609600"/>
-          <a:ext cx="4838700" cy="2257143"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>28575</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>4876800</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>190124</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{78B8743F-FCDF-4982-B850-38C307B790CF}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2847975" y="3276600"/>
-          <a:ext cx="4848225" cy="3009524"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
       <xdr:colOff>771525</xdr:colOff>
       <xdr:row>36</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
@@ -5338,7 +5250,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5358,22 +5270,110 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>180975</xdr:colOff>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>28576</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4906053</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>161926</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{85D2CA75-0A77-8EC3-1D39-CCA2CB2A9381}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2867025" y="600076"/>
+          <a:ext cx="4858428" cy="2228850"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4886325</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8A533D10-1887-F677-8875-2F66CA700A64}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2857500" y="3324225"/>
+          <a:ext cx="4848225" cy="3076575"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>314325</xdr:colOff>
       <xdr:row>49</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>4723832</xdr:colOff>
-      <xdr:row>59</xdr:row>
-      <xdr:rowOff>56910</xdr:rowOff>
+      <xdr:colOff>4372541</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 4">
+        <xdr:cNvPr id="11" name="Picture 10">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{69180342-896B-4276-AA66-4AC691C87E15}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{69529BC8-CD02-9037-0AA8-903FE999D7AC}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5389,8 +5389,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3000375" y="9372600"/>
-          <a:ext cx="4542857" cy="1923810"/>
+          <a:off x="3133725" y="9372600"/>
+          <a:ext cx="4058216" cy="1838325"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5402,22 +5402,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>790575</xdr:colOff>
-      <xdr:row>61</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:colOff>952500</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>3904861</xdr:colOff>
+      <xdr:colOff>3810399</xdr:colOff>
       <xdr:row>74</xdr:row>
-      <xdr:rowOff>28271</xdr:rowOff>
+      <xdr:rowOff>152768</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Picture 5">
+        <xdr:cNvPr id="12" name="Picture 11">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7EFC80A3-43EE-4640-94DE-5DFA8D43746B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C361F852-06CE-6607-4349-D657927C53FB}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5433,8 +5433,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3609975" y="11696700"/>
-          <a:ext cx="3114286" cy="2428571"/>
+          <a:off x="3771900" y="11610975"/>
+          <a:ext cx="2857899" cy="2638793"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5446,22 +5446,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
-      <xdr:row>77</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:colOff>361950</xdr:colOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>4914900</xdr:colOff>
+      <xdr:colOff>4725009</xdr:colOff>
       <xdr:row>84</xdr:row>
-      <xdr:rowOff>171267</xdr:rowOff>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Picture 6">
+        <xdr:cNvPr id="13" name="Picture 12">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{07C4DDB7-29D4-45BF-B6D9-6A1ACCCF81AE}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{613257E7-C7D3-CEB7-B05F-BA64B1F79D33}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5477,8 +5477,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2838450" y="14706600"/>
-          <a:ext cx="4895850" cy="1466667"/>
+          <a:off x="3181350" y="14649450"/>
+          <a:ext cx="4363059" cy="1504950"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5490,22 +5490,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
+      <xdr:colOff>38100</xdr:colOff>
       <xdr:row>87</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>4914900</xdr:colOff>
+      <xdr:colOff>4905375</xdr:colOff>
       <xdr:row>98</xdr:row>
-      <xdr:rowOff>161648</xdr:rowOff>
+      <xdr:rowOff>171450</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="Picture 7">
+        <xdr:cNvPr id="14" name="Picture 13">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{72C369ED-CB3E-414B-AA88-1A97F9A9B26F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A1A89F36-2068-08CA-C3DE-E3CCA530AB16}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5521,8 +5521,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2838450" y="16611600"/>
-          <a:ext cx="4895850" cy="2219048"/>
+          <a:off x="2857500" y="16592550"/>
+          <a:ext cx="4867275" cy="2247900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5539,22 +5539,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
+      <xdr:colOff>66675</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>133350</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>4914899</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>28214</xdr:rowOff>
+      <xdr:colOff>4886325</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
+        <xdr:cNvPr id="7" name="Picture 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EB62B418-DC22-44ED-8807-345A5BA65F21}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4AC79A22-E60E-8843-4E67-45DCD0FDCA98}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5570,8 +5570,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2838450" y="571500"/>
-          <a:ext cx="4895849" cy="2885714"/>
+          <a:off x="2886075" y="704850"/>
+          <a:ext cx="4819650" cy="2676525"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5583,22 +5583,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>438150</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>4438150</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>95052</xdr:rowOff>
+      <xdr:colOff>4914900</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>162247</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
+        <xdr:cNvPr id="8" name="Picture 7">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{19768BBE-BA6F-4378-8C5C-C958B2CBC7F1}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{11F4C685-B63F-AFD6-643D-0ADA26C2ED24}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5614,8 +5614,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3257550" y="3848100"/>
-          <a:ext cx="4000000" cy="1580952"/>
+          <a:off x="2867025" y="4143375"/>
+          <a:ext cx="4867275" cy="2305372"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5627,22 +5627,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>28576</xdr:colOff>
+      <xdr:colOff>19050</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>4905376</xdr:colOff>
+      <xdr:colOff>4905375</xdr:colOff>
       <xdr:row>48</xdr:row>
-      <xdr:rowOff>171145</xdr:rowOff>
+      <xdr:rowOff>161925</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
+        <xdr:cNvPr id="9" name="Picture 8">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{04A1031B-C790-4A68-9CE9-B0DE59F8E2C0}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{01CEB0C1-CDDC-46BE-3EA6-0D099286D0E4}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5658,8 +5658,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2847976" y="6877050"/>
-          <a:ext cx="4876800" cy="2438095"/>
+          <a:off x="2838450" y="6905625"/>
+          <a:ext cx="4886325" cy="2400300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5671,22 +5671,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>457200</xdr:colOff>
+      <xdr:colOff>38101</xdr:colOff>
       <xdr:row>51</xdr:row>
       <xdr:rowOff>9525</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>4371486</xdr:colOff>
-      <xdr:row>67</xdr:row>
-      <xdr:rowOff>123430</xdr:rowOff>
+      <xdr:colOff>4895851</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 4">
+        <xdr:cNvPr id="10" name="Picture 9">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{263344B6-54B1-4702-BA39-ECBB86150295}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A4E022EA-EDFB-B752-2CDF-3B61CAB57409}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5702,8 +5702,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3276600" y="9725025"/>
-          <a:ext cx="3914286" cy="3161905"/>
+          <a:off x="2857501" y="9725025"/>
+          <a:ext cx="4857750" cy="3009900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -7099,7 +7099,7 @@
       <c r="C6" s="5"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="12" t="s">
         <v>170</v>
       </c>
       <c r="D7" t="s">
@@ -7135,7 +7135,7 @@
       <c r="C23" s="5"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="8" t="s">
+      <c r="A24" s="12" t="s">
         <v>176</v>
       </c>
       <c r="D24" t="s">
@@ -7161,7 +7161,7 @@
       <c r="C43" s="5"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="8" t="s">
+      <c r="A44" s="12" t="s">
         <v>180</v>
       </c>
       <c r="D44" t="s">
@@ -7195,7 +7195,7 @@
       <c r="C50" s="5"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="8" t="s">
+      <c r="A51" s="12" t="s">
         <v>186</v>
       </c>
       <c r="D51" t="s">
@@ -7221,7 +7221,7 @@
       <c r="C86" s="5"/>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="13" t="s">
+      <c r="A87" s="12" t="s">
         <v>190</v>
       </c>
       <c r="D87" t="s">
@@ -7262,7 +7262,7 @@
       <c r="C96" s="5"/>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A97" s="8" t="s">
+      <c r="A97" s="12" t="s">
         <v>196</v>
       </c>
       <c r="D97" t="s">
@@ -7283,7 +7283,7 @@
       <c r="C113" s="5"/>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A114" s="14" t="s">
+      <c r="A114" s="13" t="s">
         <v>463</v>
       </c>
       <c r="D114" t="s">
@@ -7319,7 +7319,7 @@
       <c r="C121" s="5"/>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A122" s="13" t="s">
+      <c r="A122" s="12" t="s">
         <v>469</v>
       </c>
       <c r="D122" t="s">
@@ -7355,7 +7355,7 @@
       <c r="C152" s="5"/>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A153" s="13" t="s">
+      <c r="A153" s="12" t="s">
         <v>474</v>
       </c>
       <c r="D153" t="s">
@@ -7396,7 +7396,7 @@
       <c r="C169" s="5"/>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A170" s="13" t="s">
+      <c r="A170" s="12" t="s">
         <v>480</v>
       </c>
       <c r="D170" t="s">
@@ -7447,11 +7447,11 @@
       <c r="C185" s="5"/>
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A186" s="13" t="s">
+      <c r="A186" s="12" t="s">
         <v>489</v>
       </c>
       <c r="C186" s="1" t="s">
-        <v>501</v>
+        <v>612</v>
       </c>
       <c r="D186" t="s">
         <v>491</v>
@@ -7461,15 +7461,15 @@
       <c r="A187" s="2" t="s">
         <v>490</v>
       </c>
-      <c r="C187" s="17" t="s">
-        <v>502</v>
+      <c r="C187" s="16" t="s">
+        <v>501</v>
       </c>
       <c r="D187" t="s">
         <v>492</v>
       </c>
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C188" s="16" t="s">
+      <c r="C188" s="15" t="s">
         <v>9</v>
       </c>
       <c r="D188" t="s">
@@ -7523,41 +7523,41 @@
       <c r="C202" s="5"/>
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A203" s="14" t="s">
+      <c r="A203" s="13" t="s">
+        <v>502</v>
+      </c>
+      <c r="D203" t="s">
         <v>503</v>
-      </c>
-      <c r="D203" t="s">
-        <v>504</v>
       </c>
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D204" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D205" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D206" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D207" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D208" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D209" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.25">
@@ -7569,31 +7569,31 @@
       <c r="C223" s="5"/>
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A224" s="13" t="s">
+      <c r="A224" s="12" t="s">
+        <v>510</v>
+      </c>
+      <c r="D224" t="s">
         <v>511</v>
-      </c>
-      <c r="D224" t="s">
-        <v>512</v>
       </c>
     </row>
     <row r="225" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D225" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
     </row>
     <row r="226" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D226" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="227" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D227" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
     </row>
     <row r="228" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D228" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
     </row>
     <row r="240" spans="4:4" x14ac:dyDescent="0.25">
@@ -7605,11 +7605,11 @@
       <c r="C241" s="5"/>
     </row>
     <row r="242" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A242" s="14" t="s">
+      <c r="A242" s="13" t="s">
+        <v>516</v>
+      </c>
+      <c r="D242" t="s">
         <v>517</v>
-      </c>
-      <c r="D242" t="s">
-        <v>518</v>
       </c>
     </row>
     <row r="243" spans="1:4" x14ac:dyDescent="0.25">
@@ -7619,22 +7619,22 @@
     </row>
     <row r="244" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D244" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="245" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D245" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="246" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D246" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="247" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D247" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
     </row>
     <row r="254" spans="1:4" x14ac:dyDescent="0.25">
@@ -7646,21 +7646,21 @@
       <c r="C255" s="5"/>
     </row>
     <row r="256" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A256" s="13" t="s">
+      <c r="A256" s="12" t="s">
+        <v>522</v>
+      </c>
+      <c r="D256" t="s">
         <v>523</v>
-      </c>
-      <c r="D256" t="s">
-        <v>524</v>
       </c>
     </row>
     <row r="257" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D257" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
     </row>
     <row r="258" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D258" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
     </row>
     <row r="270" spans="1:4" x14ac:dyDescent="0.25">
@@ -7672,31 +7672,31 @@
       <c r="C271" s="5"/>
     </row>
     <row r="272" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A272" s="13" t="s">
+      <c r="A272" s="12" t="s">
+        <v>526</v>
+      </c>
+      <c r="D272" t="s">
         <v>527</v>
-      </c>
-      <c r="D272" t="s">
-        <v>528</v>
       </c>
     </row>
     <row r="273" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D273" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
     </row>
     <row r="274" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D274" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
     </row>
     <row r="275" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D275" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
     </row>
     <row r="276" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D276" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
     </row>
     <row r="280" spans="1:4" x14ac:dyDescent="0.25">
@@ -7708,31 +7708,31 @@
       <c r="C281" s="5"/>
     </row>
     <row r="282" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A282" s="14" t="s">
+      <c r="A282" s="13" t="s">
+        <v>532</v>
+      </c>
+      <c r="D282" t="s">
         <v>533</v>
-      </c>
-      <c r="D282" t="s">
-        <v>534</v>
       </c>
     </row>
     <row r="283" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D283" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
     </row>
     <row r="284" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D284" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
     </row>
     <row r="285" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D285" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
     </row>
     <row r="286" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D286" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
     </row>
     <row r="297" spans="1:4" x14ac:dyDescent="0.25">
@@ -7744,41 +7744,41 @@
       <c r="C298" s="5"/>
     </row>
     <row r="299" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A299" s="13" t="s">
-        <v>539</v>
+      <c r="A299" s="12" t="s">
+        <v>538</v>
       </c>
       <c r="D299" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
     </row>
     <row r="300" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D300" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
     </row>
     <row r="301" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D301" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
     </row>
     <row r="302" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D302" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
     </row>
     <row r="303" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D303" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
     </row>
     <row r="304" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D304" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="305" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D305" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
     </row>
     <row r="321" spans="3:4" x14ac:dyDescent="0.25">
@@ -7891,7 +7891,7 @@
       <c r="C7" s="5"/>
     </row>
     <row r="8" spans="1:4" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="11" t="s">
         <v>231</v>
       </c>
       <c r="C8" s="1" t="s">
@@ -7919,7 +7919,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C11" s="1" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="D11" t="s">
         <v>238</v>
@@ -8106,7 +8106,7 @@
       <c r="C2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="12" t="s">
         <v>225</v>
       </c>
       <c r="D3" t="s">
@@ -8312,7 +8312,7 @@
       <c r="C2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="12" t="s">
         <v>104</v>
       </c>
       <c r="D3" t="s">
@@ -8338,7 +8338,7 @@
       <c r="C8" s="5"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="13" t="s">
         <v>108</v>
       </c>
       <c r="D9" t="s">
@@ -8377,7 +8377,7 @@
       <c r="C17" s="5"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="13" t="s">
+      <c r="A18" s="12" t="s">
         <v>111</v>
       </c>
       <c r="D18" t="s">
@@ -8413,7 +8413,7 @@
       <c r="C32" s="5"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="15" t="s">
+      <c r="A33" s="14" t="s">
         <v>261</v>
       </c>
       <c r="C33" s="1" t="s">
@@ -8460,7 +8460,7 @@
       <c r="C39" s="5"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="13" t="s">
+      <c r="A40" s="12" t="s">
         <v>264</v>
       </c>
       <c r="D40" t="s">
@@ -8491,7 +8491,7 @@
       <c r="C50" s="5"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="15" t="s">
+      <c r="A51" s="14" t="s">
         <v>268</v>
       </c>
       <c r="D51" t="s">
@@ -8517,7 +8517,7 @@
       <c r="C58" s="5"/>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="13" t="s">
+      <c r="A59" s="12" t="s">
         <v>271</v>
       </c>
       <c r="D59" t="s">
@@ -8546,7 +8546,7 @@
       <c r="C68" s="5"/>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="13" t="s">
+      <c r="A69" s="12" t="s">
         <v>275</v>
       </c>
       <c r="D69" t="s">
@@ -8567,7 +8567,7 @@
       <c r="C74" s="5"/>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="13" t="s">
+      <c r="A75" s="12" t="s">
         <v>278</v>
       </c>
       <c r="D75" t="s">
@@ -8601,7 +8601,7 @@
       <c r="C84" s="5"/>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="13" t="s">
+      <c r="A85" s="12" t="s">
         <v>283</v>
       </c>
       <c r="D85" t="s">
@@ -8635,7 +8635,7 @@
       <c r="C92" s="5"/>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A93" s="13" t="s">
+      <c r="A93" s="12" t="s">
         <v>318</v>
       </c>
       <c r="D93" t="s">
@@ -8692,7 +8692,7 @@
       <c r="C103" s="5"/>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A104" s="13" t="s">
+      <c r="A104" s="12" t="s">
         <v>311</v>
       </c>
       <c r="D104" t="s">
@@ -8726,7 +8726,7 @@
       <c r="C111" s="5"/>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A112" s="13" t="s">
+      <c r="A112" s="12" t="s">
         <v>342</v>
       </c>
       <c r="D112" t="s">
@@ -8760,7 +8760,7 @@
       <c r="C122" s="5"/>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A123" s="13" t="s">
+      <c r="A123" s="12" t="s">
         <v>371</v>
       </c>
       <c r="D123" t="s">
@@ -8796,7 +8796,7 @@
       <c r="C130" s="5"/>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A131" s="14" t="s">
+      <c r="A131" s="13" t="s">
         <v>379</v>
       </c>
       <c r="D131" t="s">
@@ -8837,7 +8837,7 @@
       <c r="C140" s="5"/>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A141" s="13" t="s">
+      <c r="A141" s="12" t="s">
         <v>385</v>
       </c>
       <c r="D141" t="s">
@@ -8896,7 +8896,7 @@
       <c r="C156" s="5"/>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A157" s="14" t="s">
+      <c r="A157" s="13" t="s">
         <v>393</v>
       </c>
       <c r="D157" t="s">
@@ -8948,7 +8948,7 @@
       <c r="C170" s="5"/>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A171" s="13" t="s">
+      <c r="A171" s="12" t="s">
         <v>402</v>
       </c>
       <c r="D171" t="s">
@@ -8979,7 +8979,7 @@
       <c r="C177" s="5"/>
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A178" s="13" t="s">
+      <c r="A178" s="12" t="s">
         <v>405</v>
       </c>
       <c r="D178" t="s">
@@ -9018,7 +9018,7 @@
       <c r="C187" s="5"/>
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A188" s="14" t="s">
+      <c r="A188" s="13" t="s">
         <v>411</v>
       </c>
       <c r="D188" t="s">
@@ -9049,7 +9049,7 @@
       <c r="C195" s="5"/>
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A196" s="15" t="s">
+      <c r="A196" s="14" t="s">
         <v>416</v>
       </c>
       <c r="D196" t="s">
@@ -9070,7 +9070,7 @@
       <c r="C204" s="5"/>
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A205" s="14" t="s">
+      <c r="A205" s="13" t="s">
         <v>419</v>
       </c>
       <c r="D205" t="s">
@@ -9111,7 +9111,7 @@
       <c r="C214" s="5"/>
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A215" s="13" t="s">
+      <c r="A215" s="12" t="s">
         <v>426</v>
       </c>
       <c r="D215" t="s">
@@ -9147,7 +9147,7 @@
       <c r="C221" s="5"/>
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A222" s="15" t="s">
+      <c r="A222" s="14" t="s">
         <v>430</v>
       </c>
       <c r="D222" t="s">
@@ -9173,7 +9173,7 @@
       <c r="C240" s="5"/>
     </row>
     <row r="241" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A241" s="13" t="s">
+      <c r="A241" s="12" t="s">
         <v>434</v>
       </c>
       <c r="D241" t="s">
@@ -9214,7 +9214,7 @@
       <c r="C259" s="5"/>
     </row>
     <row r="260" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A260" s="15" t="s">
+      <c r="A260" s="14" t="s">
         <v>440</v>
       </c>
       <c r="D260" t="s">
@@ -9250,7 +9250,7 @@
       <c r="C267" s="5"/>
     </row>
     <row r="268" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A268" s="13" t="s">
+      <c r="A268" s="12" t="s">
         <v>445</v>
       </c>
       <c r="D268" t="s">
@@ -9286,7 +9286,7 @@
       <c r="C277" s="5"/>
     </row>
     <row r="278" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A278" s="13" t="s">
+      <c r="A278" s="12" t="s">
         <v>451</v>
       </c>
       <c r="D278" t="s">
@@ -9327,7 +9327,7 @@
       <c r="C285" s="5"/>
     </row>
     <row r="286" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A286" s="13" t="s">
+      <c r="A286" s="12" t="s">
         <v>457</v>
       </c>
       <c r="C286" s="1" t="s">
@@ -9364,16 +9364,16 @@
       <c r="C298" s="5"/>
     </row>
     <row r="299" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A299" s="13" t="s">
-        <v>584</v>
+      <c r="A299" s="12" t="s">
+        <v>583</v>
       </c>
       <c r="D299" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="300" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D300" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="304" spans="1:4" x14ac:dyDescent="0.25">
@@ -9522,26 +9522,26 @@
       <c r="C15" s="5"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="15" t="s">
+      <c r="A16" s="14" t="s">
+        <v>551</v>
+      </c>
+      <c r="D16" t="s">
         <v>552</v>
-      </c>
-      <c r="D16" t="s">
-        <v>553</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D17" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D18" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D19" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -9553,31 +9553,31 @@
       <c r="C30" s="5"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="13" t="s">
+      <c r="A31" s="12" t="s">
+        <v>556</v>
+      </c>
+      <c r="D31" t="s">
         <v>557</v>
-      </c>
-      <c r="D31" t="s">
-        <v>558</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D32" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D33" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D34" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D35" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -9585,22 +9585,22 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D37" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D38" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D39" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D40" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -9612,26 +9612,26 @@
       <c r="C45" s="5"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="13" t="s">
+      <c r="A46" s="12" t="s">
+        <v>566</v>
+      </c>
+      <c r="D46" t="s">
         <v>567</v>
-      </c>
-      <c r="D46" t="s">
-        <v>568</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D47" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D48" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D49" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -9643,26 +9643,26 @@
       <c r="C59" s="5"/>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="13" t="s">
+      <c r="A60" s="12" t="s">
+        <v>578</v>
+      </c>
+      <c r="D60" t="s">
         <v>579</v>
-      </c>
-      <c r="D60" t="s">
-        <v>580</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D61" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D62" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D63" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
@@ -9674,21 +9674,21 @@
       <c r="C72" s="5"/>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="13" t="s">
-        <v>590</v>
+      <c r="A73" s="12" t="s">
+        <v>589</v>
       </c>
       <c r="D73" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D74" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D75" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="83" spans="3:4" x14ac:dyDescent="0.25">
@@ -9750,7 +9750,7 @@
       <c r="C2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="12" t="s">
         <v>288</v>
       </c>
       <c r="D3" t="s">
@@ -9817,36 +9817,36 @@
       <c r="C17" s="5"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="14" t="s">
+      <c r="A18" s="13" t="s">
+        <v>593</v>
+      </c>
+      <c r="D18" t="s">
         <v>594</v>
-      </c>
-      <c r="D18" t="s">
-        <v>595</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D19" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D20" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D21" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D23" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -9858,16 +9858,16 @@
       <c r="C34" s="5"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="13" t="s">
+      <c r="A35" s="12" t="s">
+        <v>600</v>
+      </c>
+      <c r="D35" t="s">
         <v>601</v>
-      </c>
-      <c r="D35" t="s">
-        <v>602</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D36" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
     </row>
     <row r="49" spans="3:4" x14ac:dyDescent="0.25">
@@ -9926,7 +9926,7 @@
       <c r="C2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="14" t="s">
         <v>117</v>
       </c>
       <c r="D3" t="s">
@@ -9957,7 +9957,7 @@
       <c r="C10" s="5"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="17" t="s">
         <v>122</v>
       </c>
       <c r="D11" t="s">
@@ -9998,7 +9998,7 @@
       <c r="C19" s="5"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="12" t="s">
         <v>141</v>
       </c>
       <c r="D20" t="s">
@@ -10029,26 +10029,26 @@
       <c r="C26" s="5"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="14" t="s">
+      <c r="A27" s="13" t="s">
+        <v>546</v>
+      </c>
+      <c r="D27" t="s">
         <v>547</v>
-      </c>
-      <c r="D27" t="s">
-        <v>548</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D28" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D29" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D30" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -10325,7 +10325,7 @@
       <c r="C2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="12" t="s">
         <v>156</v>
       </c>
       <c r="D3" t="s">
@@ -10417,11 +10417,11 @@
       <c r="C22" s="5"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="13" t="s">
+      <c r="A23" s="12" t="s">
         <v>321</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D23" t="s">
         <v>322</v>
@@ -10429,7 +10429,7 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C24" s="1" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="D24" t="s">
         <v>323</v>
@@ -10437,7 +10437,7 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C25" s="1" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D25" t="s">
         <v>324</v>
@@ -10445,7 +10445,7 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C26" s="1" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="D26" t="s">
         <v>325</v>
@@ -10453,7 +10453,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C27" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -10496,7 +10496,7 @@
       <c r="C35" s="5"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="13" t="s">
+      <c r="A36" s="12" t="s">
         <v>359</v>
       </c>
       <c r="C36" s="1" t="s">
@@ -10534,36 +10534,36 @@
       <c r="C41" s="5"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="13" t="s">
-        <v>572</v>
+      <c r="A42" s="12" t="s">
+        <v>571</v>
       </c>
       <c r="D42" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D43" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D44" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D45" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D46" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D47" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -10575,21 +10575,21 @@
       <c r="C50" s="5"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="13" t="s">
+      <c r="A51" s="12" t="s">
+        <v>585</v>
+      </c>
+      <c r="D51" t="s">
         <v>586</v>
-      </c>
-      <c r="D51" t="s">
-        <v>587</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D52" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D53" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -10601,21 +10601,21 @@
       <c r="C58" s="5"/>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="13" t="s">
+      <c r="A59" s="12" t="s">
+        <v>603</v>
+      </c>
+      <c r="D59" t="s">
         <v>604</v>
-      </c>
-      <c r="D59" t="s">
-        <v>605</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D60" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D61" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -10850,7 +10850,7 @@
       <c r="C99" s="5"/>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A100" s="13" t="s">
+      <c r="A100" s="12" t="s">
         <v>367</v>
       </c>
       <c r="D100" t="s">
@@ -10932,7 +10932,7 @@
       <c r="C2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="12" t="s">
         <v>159</v>
       </c>
       <c r="D3" t="s">
@@ -10963,7 +10963,7 @@
       <c r="C16" s="5"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="14" t="s">
         <v>160</v>
       </c>
       <c r="B17" t="s">
@@ -11054,7 +11054,7 @@
       <c r="C35" s="5"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="9" t="s">
+      <c r="A36" s="13" t="s">
         <v>161</v>
       </c>
       <c r="D36" t="s">
@@ -11100,7 +11100,7 @@
       <c r="C48" s="5"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="8" t="s">
+      <c r="A49" s="12" t="s">
         <v>162</v>
       </c>
       <c r="D49" t="s">
@@ -11142,7 +11142,7 @@
       <c r="C60" s="5"/>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="4" t="s">
+      <c r="A61" s="14" t="s">
         <v>163</v>
       </c>
       <c r="D61" s="7" t="s">
@@ -11191,7 +11191,7 @@
       <c r="C76" s="5"/>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="8" t="s">
+      <c r="A77" s="12" t="s">
         <v>164</v>
       </c>
       <c r="C77" s="1" t="s">
@@ -11241,7 +11241,7 @@
       <c r="C86" s="5"/>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="8" t="s">
+      <c r="A87" s="12" t="s">
         <v>165</v>
       </c>
       <c r="D87" t="s">
@@ -11293,19 +11293,19 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" display="Remove Nth Node From End of List" xr:uid="{7DFF2091-3C94-4306-9948-C02C8450916F}"/>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{7DFF2091-3C94-4306-9948-C02C8450916F}"/>
     <hyperlink ref="D15" r:id="rId2" xr:uid="{EACB1A9A-0E1F-40EF-A8DA-3D41720EFE9D}"/>
-    <hyperlink ref="A17" r:id="rId3" display="Merge Two Sorted Lists" xr:uid="{29D47218-0B99-4D27-92EB-96B8A53BF540}"/>
+    <hyperlink ref="A17" r:id="rId3" xr:uid="{29D47218-0B99-4D27-92EB-96B8A53BF540}"/>
     <hyperlink ref="D34" r:id="rId4" xr:uid="{E6B50439-28D8-4A43-A31B-CA26FE7F6665}"/>
-    <hyperlink ref="A36" r:id="rId5" display="Merge k Sorted Lists" xr:uid="{B469572D-F03A-49A5-BB95-40D77AF73B8F}"/>
+    <hyperlink ref="A36" r:id="rId5" xr:uid="{B469572D-F03A-49A5-BB95-40D77AF73B8F}"/>
     <hyperlink ref="D47" r:id="rId6" xr:uid="{B5EB827D-B21A-4924-9D01-9B55F99EE74F}"/>
-    <hyperlink ref="A49" r:id="rId7" display="Rotate List" xr:uid="{9991CCC5-947C-47FA-94E2-F9C4DC8AEE2F}"/>
+    <hyperlink ref="A49" r:id="rId7" xr:uid="{9991CCC5-947C-47FA-94E2-F9C4DC8AEE2F}"/>
     <hyperlink ref="D59" r:id="rId8" xr:uid="{E43457D5-A59A-4E1A-8DBF-788129276609}"/>
-    <hyperlink ref="A61" r:id="rId9" display="Remove Duplicates from Sorted List" xr:uid="{87233EE7-0EC1-4307-9FBD-D575CDBE8312}"/>
+    <hyperlink ref="A61" r:id="rId9" xr:uid="{87233EE7-0EC1-4307-9FBD-D575CDBE8312}"/>
     <hyperlink ref="D75" r:id="rId10" xr:uid="{15CFEFB2-0626-4422-8C73-8889EDAD581A}"/>
-    <hyperlink ref="A77" r:id="rId11" display="Remove Duplicates from Sorted List II" xr:uid="{989B3ECE-514E-404A-8626-396B08E7CC8E}"/>
+    <hyperlink ref="A77" r:id="rId11" xr:uid="{989B3ECE-514E-404A-8626-396B08E7CC8E}"/>
     <hyperlink ref="D85" r:id="rId12" xr:uid="{0B825229-A326-4F0A-98C7-177795F408C9}"/>
-    <hyperlink ref="A87" r:id="rId13" display="Partition List" xr:uid="{48BB70FF-A8ED-42E4-8A11-752AF2EB04DC}"/>
+    <hyperlink ref="A87" r:id="rId13" xr:uid="{48BB70FF-A8ED-42E4-8A11-752AF2EB04DC}"/>
     <hyperlink ref="D99" r:id="rId14" xr:uid="{C55579BE-756D-40BA-A7A4-EA1ABF78C0AC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11345,7 +11345,7 @@
       <c r="C2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="12" t="s">
         <v>166</v>
       </c>
       <c r="B3" t="s">
@@ -11385,7 +11385,7 @@
       <c r="C19" s="5"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="9" t="s">
+      <c r="A20" s="13" t="s">
         <v>167</v>
       </c>
       <c r="B20" t="s">
@@ -11454,7 +11454,7 @@
       <c r="C35" s="5"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="9" t="s">
+      <c r="A36" s="13" t="s">
         <v>168</v>
       </c>
       <c r="D36" t="s">
@@ -11485,32 +11485,32 @@
       <c r="D41" s="8"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D42" s="11" t="s">
+      <c r="D42" s="10" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D43" s="11" t="s">
+      <c r="D43" s="10" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D44" s="11" t="s">
+      <c r="D44" s="10" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D45" s="11" t="s">
+      <c r="D45" s="10" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D46" s="11" t="s">
+      <c r="D46" s="10" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D47" s="11" t="s">
+      <c r="D47" s="10" t="s">
         <v>29</v>
       </c>
     </row>
@@ -11523,7 +11523,7 @@
       <c r="C50" s="5"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="9" t="s">
+      <c r="A51" s="13" t="s">
         <v>169</v>
       </c>
       <c r="B51" t="s">
@@ -11558,13 +11558,13 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" display="Container with most water" xr:uid="{F4D67A5D-744F-4C81-957E-33D3253297A2}"/>
-    <hyperlink ref="A20" r:id="rId2" display="Trapping Rain Water" xr:uid="{CDAA1F07-861A-43F8-806E-CBF196F42093}"/>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{F4D67A5D-744F-4C81-957E-33D3253297A2}"/>
+    <hyperlink ref="A20" r:id="rId2" xr:uid="{CDAA1F07-861A-43F8-806E-CBF196F42093}"/>
     <hyperlink ref="D18" r:id="rId3" xr:uid="{30328AA2-76F9-472A-BAB3-B3B0C7802963}"/>
     <hyperlink ref="D34" r:id="rId4" xr:uid="{FBB1B328-6337-43BB-960F-5B6CAE89E813}"/>
-    <hyperlink ref="A36" r:id="rId5" display="Largest Rectangle in Histogram" xr:uid="{33CB1418-814A-466E-8725-5800B98469F7}"/>
+    <hyperlink ref="A36" r:id="rId5" xr:uid="{33CB1418-814A-466E-8725-5800B98469F7}"/>
     <hyperlink ref="D49" r:id="rId6" xr:uid="{6329D858-D8F3-4698-AF57-250A8ABB78A2}"/>
-    <hyperlink ref="A51" r:id="rId7" display="Maximal Rectangle" xr:uid="{C5538507-5156-4F6A-800E-694A86C1DE83}"/>
+    <hyperlink ref="A51" r:id="rId7" xr:uid="{C5538507-5156-4F6A-800E-694A86C1DE83}"/>
     <hyperlink ref="D67" r:id="rId8" xr:uid="{A272D98F-93C2-491D-BEBC-54FFA0BBC858}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
nextGreaterElement - May 28th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99843D92-A11B-4EB5-9433-BF165035B802}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D57299DC-295B-4244-B9BF-53D83DB7AE42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="1" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="2" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="613">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="825" uniqueCount="627">
   <si>
     <t>Statement</t>
   </si>
@@ -1947,12 +1947,82 @@
   <si>
     <t>similar problem</t>
   </si>
+  <si>
+    <t>496. Next Greater Element I</t>
+  </si>
+  <si>
+    <t>use stack to find next greater element for nums2</t>
+  </si>
+  <si>
+    <t>if stack is empty just add</t>
+  </si>
+  <si>
+    <t>else while peek element is &lt; current, means nge of peek = current</t>
+  </si>
+  <si>
+    <t>503. Next Greater Element II</t>
+  </si>
+  <si>
+    <t>556. Next Greater Element III</t>
+  </si>
+  <si>
+    <t>find i for which i &lt; i+1 from right</t>
+  </si>
+  <si>
+    <r>
+      <t>for 3</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>476</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>find k for which k &gt; i from right, swap i and k -&gt; 3</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>674</t>
+    </r>
+  </si>
+  <si>
+    <t>reverse chars from i+1 to end</t>
+  </si>
+  <si>
+    <t>71. Simplify Path</t>
+  </si>
+  <si>
+    <t>split by /</t>
+  </si>
+  <si>
+    <t>if dir is .. and non empty stack - pop</t>
+  </si>
+  <si>
+    <t>else if dir not in . .. Or '' add to stack</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2042,6 +2112,15 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -4499,6 +4578,50 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>152488</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C1AA3435-2DEC-7A9E-3EA8-54C18FC52C43}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2857500" y="3905250"/>
+          <a:ext cx="4886325" cy="628738"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -4941,6 +5064,94 @@
         <a:xfrm>
           <a:off x="4591050" y="11268075"/>
           <a:ext cx="1838582" cy="428685"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>171607</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{251DF39B-64BC-D685-3D54-94F4ED362B57}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3448050" y="12382500"/>
+          <a:ext cx="4867275" cy="1124107"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1476375</xdr:colOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2610008</xdr:colOff>
+      <xdr:row>75</xdr:row>
+      <xdr:rowOff>181033</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Picture 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BBFCD468-B742-8264-2174-F835A46EE88D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4867275" y="14049375"/>
+          <a:ext cx="1133633" cy="419158"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -10077,7 +10288,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5D8A62A-F83B-49C3-B94F-89CCE841A84E}">
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -10106,7 +10317,7 @@
       <c r="C2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="12" t="s">
         <v>129</v>
       </c>
       <c r="D3" t="s">
@@ -10137,7 +10348,7 @@
       <c r="C12" s="5"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="12" t="s">
         <v>206</v>
       </c>
       <c r="C13" s="1" t="s">
@@ -10165,13 +10376,39 @@
         <v>210</v>
       </c>
     </row>
-    <row r="18" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D18" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C19" s="5"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
+        <v>623</v>
+      </c>
+      <c r="D20" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D21" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D22" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D24" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C25" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -10179,9 +10416,11 @@
     <hyperlink ref="D11" r:id="rId2" xr:uid="{9F89C3A2-3C08-4ECF-9472-88C559CBD6E0}"/>
     <hyperlink ref="A13" r:id="rId3" xr:uid="{9B0E0792-F2BF-4326-AE22-484FC8152DDE}"/>
     <hyperlink ref="D18" r:id="rId4" xr:uid="{E62DF899-E1F2-4263-802D-E6519B60DC6C}"/>
+    <hyperlink ref="A20" r:id="rId5" xr:uid="{499A2B7E-6455-4752-801A-9309F08B80E1}"/>
+    <hyperlink ref="D24" r:id="rId6" xr:uid="{7172E2DF-D336-440F-BC8C-431F8A8501AB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId5"/>
+  <drawing r:id="rId7"/>
 </worksheet>
 </file>
 
@@ -10296,7 +10535,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDA924A8-9114-46BA-B39C-6743F04F80F3}">
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D78"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50.85546875" customWidth="1"/>
@@ -10625,6 +10864,66 @@
     </row>
     <row r="63" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C63" s="5"/>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="14" t="s">
+        <v>613</v>
+      </c>
+      <c r="C64" s="16" t="s">
+        <v>617</v>
+      </c>
+      <c r="D64" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D65" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D66" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D71" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C72" s="5"/>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" s="12" t="s">
+        <v>618</v>
+      </c>
+      <c r="D73" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D74" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D75" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D76" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D77" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C78" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -10645,9 +10944,15 @@
     <hyperlink ref="D57" r:id="rId15" xr:uid="{D42D7A59-E6C3-4502-9E9E-BE38080EC9D1}"/>
     <hyperlink ref="A59" r:id="rId16" xr:uid="{015C1AC1-D3A1-414E-BCC0-D586E7FD26CA}"/>
     <hyperlink ref="D62" r:id="rId17" xr:uid="{F43C7C50-4691-47C3-BA28-55C6EE02BB1B}"/>
+    <hyperlink ref="A64" r:id="rId18" xr:uid="{5EBCDE01-A923-4AAA-B4EA-6753EA278488}"/>
+    <hyperlink ref="D71" r:id="rId19" xr:uid="{22C37FA6-306B-4EE7-A240-9248366C0007}"/>
+    <hyperlink ref="C64" r:id="rId20" xr:uid="{E66C42DF-1C90-4082-AE05-B49055644FDA}"/>
+    <hyperlink ref="A73" r:id="rId21" xr:uid="{02DCB243-3895-4B62-B9BD-D9D4A1D7091F}"/>
+    <hyperlink ref="D77" r:id="rId22" xr:uid="{31F07A9C-A9D1-4B48-B801-6FECB16DE579}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId18"/>
+  <pageSetup orientation="portrait" r:id="rId23"/>
+  <drawing r:id="rId24"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
binary search - May 31 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D57299DC-295B-4244-B9BF-53D83DB7AE42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5163D05-5D7A-48F8-BB1C-F58C2ADF7C88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="2" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="825" uniqueCount="627">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="640">
   <si>
     <t>Statement</t>
   </si>
@@ -2016,6 +2016,45 @@
   </si>
   <si>
     <t>else if dir not in . .. Or '' add to stack</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/explore/learn/card/binary-search/125/template-i/938/</t>
+  </si>
+  <si>
+    <t>69. Sqrt(x)</t>
+  </si>
+  <si>
+    <t>binary search</t>
+  </si>
+  <si>
+    <t>lo &lt; hi, lo = mid and not mid + 1 as lo will be sqrt many times</t>
+  </si>
+  <si>
+    <t>33. Search in Rotated Sorted Array</t>
+  </si>
+  <si>
+    <t>binary search by,</t>
+  </si>
+  <si>
+    <t>finding the sorted part of array,</t>
+  </si>
+  <si>
+    <t>if target is between find in that, else other part</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/find-minimum-in-rotated-sorted-array/submissions/</t>
+  </si>
+  <si>
+    <t>735. Asteroid Collision</t>
+  </si>
+  <si>
+    <t>if prev is +ve i.e. right and curr is -ve left</t>
+  </si>
+  <si>
+    <t>then - if both equal pop one and change curr to 0 to get out of while loop, ~ for sum &lt; 0 and &gt; 0</t>
+  </si>
+  <si>
+    <t>else just add curr</t>
   </si>
 </sst>
 </file>
@@ -2577,13 +2616,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>847725</xdr:colOff>
-      <xdr:row>3</xdr:row>
+      <xdr:row>7</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>3600834</xdr:colOff>
-      <xdr:row>5</xdr:row>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>142945</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2609,6 +2648,94 @@
         <a:xfrm>
           <a:off x="3667125" y="590550"/>
           <a:ext cx="2753109" cy="504895"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1838325</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2829063</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>171501</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7D303A96-EAC2-1DE9-E2C0-96A1F0F87A85}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4657725" y="3238500"/>
+          <a:ext cx="990738" cy="362001"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1038225</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3648439</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>161982</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A443A49B-11C6-6BE8-D365-A8757EDC4FCE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3857625" y="4133850"/>
+          <a:ext cx="2610214" cy="409632"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4614,6 +4741,50 @@
         <a:xfrm>
           <a:off x="2857500" y="3905250"/>
           <a:ext cx="4886325" cy="628738"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>681</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>181052</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E2AA94F9-12F9-FB17-2C93-A77CFE80AD22}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2867025" y="4962525"/>
+          <a:ext cx="4877481" cy="552527"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -8288,7 +8459,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC70315-55E0-46CA-8156-25A8AD92E211}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -8317,51 +8488,115 @@
       <c r="C2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="2" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="5"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
         <v>225</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D7" t="s">
         <v>226</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D4" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D5" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="8"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D10" s="8"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D11" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D12" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D11" s="2" t="s">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D15" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C12" s="5"/>
+    <row r="16" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C16" s="5"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="14" t="s">
+        <v>628</v>
+      </c>
+      <c r="D17" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D18" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D19" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C20" s="5"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="12" t="s">
+        <v>631</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>635</v>
+      </c>
+      <c r="D21" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D22" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D23" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D24" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C25" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" xr:uid="{D15C5DE0-706A-4DBB-8F74-06E5036954E1}"/>
-    <hyperlink ref="D11" r:id="rId2" xr:uid="{78DAAF07-C11E-4A2F-B6D7-95F5F0D44DB8}"/>
+    <hyperlink ref="A7" r:id="rId1" xr:uid="{D15C5DE0-706A-4DBB-8F74-06E5036954E1}"/>
+    <hyperlink ref="D15" r:id="rId2" xr:uid="{78DAAF07-C11E-4A2F-B6D7-95F5F0D44DB8}"/>
+    <hyperlink ref="A3" r:id="rId3" xr:uid="{120F531C-3655-4C6A-83BF-32B2B57C07DF}"/>
+    <hyperlink ref="A17" r:id="rId4" xr:uid="{6D9D4EF2-6D20-4F15-9D04-9092739727C0}"/>
+    <hyperlink ref="D19" r:id="rId5" xr:uid="{DBFF9B81-CC27-4956-AE88-20783AA99FBA}"/>
+    <hyperlink ref="A21" r:id="rId6" xr:uid="{6D55850C-3F55-4C03-A6A3-DAEFF4B91148}"/>
+    <hyperlink ref="D24" r:id="rId7" xr:uid="{8EB59B02-D364-4F82-9E04-6EDEDB3D3A53}"/>
+    <hyperlink ref="C21" r:id="rId8" xr:uid="{B9649E71-3665-4367-A2FE-B1CC5126F04B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId3"/>
+  <drawing r:id="rId9"/>
 </worksheet>
 </file>
 
@@ -10288,7 +10523,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5D8A62A-F83B-49C3-B94F-89CCE841A84E}">
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -10410,6 +10645,32 @@
     <row r="25" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C25" s="5"/>
     </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="12" t="s">
+        <v>636</v>
+      </c>
+      <c r="D26" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D27" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D28" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D29" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C30" s="5"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" xr:uid="{6AAE33F8-490C-4B54-A064-DB29A73C2FC0}"/>
@@ -10418,9 +10679,11 @@
     <hyperlink ref="D18" r:id="rId4" xr:uid="{E62DF899-E1F2-4263-802D-E6519B60DC6C}"/>
     <hyperlink ref="A20" r:id="rId5" xr:uid="{499A2B7E-6455-4752-801A-9309F08B80E1}"/>
     <hyperlink ref="D24" r:id="rId6" xr:uid="{7172E2DF-D336-440F-BC8C-431F8A8501AB}"/>
+    <hyperlink ref="A26" r:id="rId7" xr:uid="{BB7B6230-0434-40F3-8748-35F5AB2DF0F8}"/>
+    <hyperlink ref="D29" r:id="rId8" xr:uid="{CD7A3958-5EBA-4ED1-AC04-A420C63A0A8D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId7"/>
+  <drawing r:id="rId9"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
MaximumSubarrayMin-Product - June 1st 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5163D05-5D7A-48F8-BB1C-F58C2ADF7C88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B7B13AE-5A62-4BEE-93E4-141D1EE2E5D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="2" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="640">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="847" uniqueCount="645">
   <si>
     <t>Statement</t>
   </si>
@@ -2055,6 +2055,21 @@
   </si>
   <si>
     <t>else just add curr</t>
+  </si>
+  <si>
+    <t>1856. Maximum Subarray Min-Product</t>
+  </si>
+  <si>
+    <t>if current element not &gt; peek</t>
+  </si>
+  <si>
+    <t>monotonic incr stack [value, index]</t>
+  </si>
+  <si>
+    <t>then pop last find msmp that it's part of, prefixSum(i-j) * val</t>
+  </si>
+  <si>
+    <t>find max among remaining elements in stack</t>
   </si>
 </sst>
 </file>
@@ -4785,6 +4800,50 @@
         <a:xfrm>
           <a:off x="2867025" y="4962525"/>
           <a:ext cx="4877481" cy="552527"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4886325</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>142985</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BFAA9585-C2A4-55D6-13D6-E9D7DECFD51C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2857500" y="6019800"/>
+          <a:ext cx="4848225" cy="790685"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -10523,7 +10582,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5D8A62A-F83B-49C3-B94F-89CCE841A84E}">
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -10671,6 +10730,37 @@
     <row r="30" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C30" s="5"/>
     </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="12" t="s">
+        <v>640</v>
+      </c>
+      <c r="D31" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D32" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="33" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D33" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="34" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D34" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="36" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D36" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C37" s="5"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" xr:uid="{6AAE33F8-490C-4B54-A064-DB29A73C2FC0}"/>
@@ -10681,9 +10771,11 @@
     <hyperlink ref="D24" r:id="rId6" xr:uid="{7172E2DF-D336-440F-BC8C-431F8A8501AB}"/>
     <hyperlink ref="A26" r:id="rId7" xr:uid="{BB7B6230-0434-40F3-8748-35F5AB2DF0F8}"/>
     <hyperlink ref="D29" r:id="rId8" xr:uid="{CD7A3958-5EBA-4ED1-AC04-A420C63A0A8D}"/>
+    <hyperlink ref="A31" r:id="rId9" xr:uid="{9D816F80-3F49-404D-A2A5-6F7368A89D5B}"/>
+    <hyperlink ref="D36" r:id="rId10" xr:uid="{A6350A69-B75B-483D-9A23-5B1F63BBA43D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId9"/>
+  <drawing r:id="rId11"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
OnlineStockSpan - June 4th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B7B13AE-5A62-4BEE-93E4-141D1EE2E5D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EB53D6B-B3B2-4B5E-869D-D62CFAEB825B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="2" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="847" uniqueCount="645">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="862" uniqueCount="657">
   <si>
     <t>Statement</t>
   </si>
@@ -2070,6 +2070,42 @@
   </si>
   <si>
     <t>find max among remaining elements in stack</t>
+  </si>
+  <si>
+    <t>901. Online Stock Span</t>
+  </si>
+  <si>
+    <t>monotonic decreasing stack</t>
+  </si>
+  <si>
+    <t>stack [value, span]</t>
+  </si>
+  <si>
+    <t>if empty add to stack with span as 1</t>
+  </si>
+  <si>
+    <t>else pop till peek &gt; current, and add its span to current-span</t>
+  </si>
+  <si>
+    <t>150. Evaluate Reverse Polish Notation</t>
+  </si>
+  <si>
+    <t>stack</t>
+  </si>
+  <si>
+    <t>add if operand</t>
+  </si>
+  <si>
+    <t>else pop 2 and perform operation</t>
+  </si>
+  <si>
+    <t>895. Maximum Frequency Stack</t>
+  </si>
+  <si>
+    <t>use val to count map</t>
+  </si>
+  <si>
+    <t>and count to stack of values map</t>
   </si>
 </sst>
 </file>
@@ -4844,6 +4880,138 @@
         <a:xfrm>
           <a:off x="2857500" y="6019800"/>
           <a:ext cx="4848225" cy="790685"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>247650</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4772656</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>162062</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D73C6B54-4E5C-60B8-D50B-C1544ECF4E81}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3067050" y="7372350"/>
+          <a:ext cx="4525006" cy="981212"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1200150</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3676996</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>19131</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E0C5D565-7AE5-C617-AE12-B91C21EFA79E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4019550" y="8772525"/>
+          <a:ext cx="2476846" cy="581106"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>66676</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4867276</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>152548</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{53725081-F31F-2A14-E800-0D24044F4A3A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2886076" y="9763125"/>
+          <a:ext cx="4800600" cy="1057423"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -10582,7 +10750,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5D8A62A-F83B-49C3-B94F-89CCE841A84E}">
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -10743,23 +10911,101 @@
         <v>641</v>
       </c>
     </row>
-    <row r="33" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D33" t="s">
         <v>643</v>
       </c>
     </row>
-    <row r="34" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D34" t="s">
         <v>644</v>
       </c>
     </row>
-    <row r="36" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D36" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="37" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C37" s="5"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="12" t="s">
+        <v>645</v>
+      </c>
+      <c r="D38" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D39" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D40" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D41" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D44" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C45" s="5"/>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="12" t="s">
+        <v>650</v>
+      </c>
+      <c r="D46" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D47" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D48" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D49" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C50" s="5"/>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="13" t="s">
+        <v>654</v>
+      </c>
+      <c r="D51" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D52" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D57" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C58" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -10773,9 +11019,15 @@
     <hyperlink ref="D29" r:id="rId8" xr:uid="{CD7A3958-5EBA-4ED1-AC04-A420C63A0A8D}"/>
     <hyperlink ref="A31" r:id="rId9" xr:uid="{9D816F80-3F49-404D-A2A5-6F7368A89D5B}"/>
     <hyperlink ref="D36" r:id="rId10" xr:uid="{A6350A69-B75B-483D-9A23-5B1F63BBA43D}"/>
+    <hyperlink ref="A38" r:id="rId11" xr:uid="{06184409-1A85-41F0-8E67-5A1271756EF6}"/>
+    <hyperlink ref="D44" r:id="rId12" xr:uid="{0E5037C5-B4C0-4A0C-BD52-FCCB66069C0C}"/>
+    <hyperlink ref="A46" r:id="rId13" xr:uid="{196C90E9-478C-48E5-858B-841013361D70}"/>
+    <hyperlink ref="D49" r:id="rId14" xr:uid="{7A49C60D-CF07-482B-88E8-BACCE2595D8E}"/>
+    <hyperlink ref="A51" r:id="rId15" xr:uid="{20507E66-8AEE-4B9C-850A-CA9238583EC3}"/>
+    <hyperlink ref="D57" r:id="rId16" xr:uid="{79F280B3-41CF-4A9A-A469-C35B9DB33B8A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId11"/>
+  <drawing r:id="rId17"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
FindMedianfromDataStream - June 7th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EB53D6B-B3B2-4B5E-869D-D62CFAEB825B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{227E235B-5C9D-4AD6-8BCE-241180C89681}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="2" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="3" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="862" uniqueCount="657">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="865" uniqueCount="659">
   <si>
     <t>Statement</t>
   </si>
@@ -2106,6 +2106,12 @@
   </si>
   <si>
     <t>and count to stack of values map</t>
+  </si>
+  <si>
+    <t>295. Find Median from Data Stream</t>
+  </si>
+  <si>
+    <t>Declare max heap and min heap to store first half and second half of sorted array</t>
   </si>
 </sst>
 </file>
@@ -5105,6 +5111,50 @@
         <a:xfrm>
           <a:off x="2847975" y="3286125"/>
           <a:ext cx="4876800" cy="1200318"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4772670</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>134</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C8FB4233-64A5-0450-CC3A-53F3CA2356FA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2971800" y="4943475"/>
+          <a:ext cx="4620270" cy="962159"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -11033,7 +11083,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51C4CDD9-9363-46B2-A2D8-BE11DE99714D}">
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -11062,7 +11112,7 @@
       <c r="C2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="13" t="s">
         <v>134</v>
       </c>
       <c r="D3" t="s">
@@ -11103,7 +11153,7 @@
       <c r="C16" s="5"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="12" t="s">
         <v>245</v>
       </c>
       <c r="D17" t="s">
@@ -11127,6 +11177,22 @@
     </row>
     <row r="25" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C25" s="5"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="13" t="s">
+        <v>657</v>
+      </c>
+      <c r="D26" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D31" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C32" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -11134,9 +11200,12 @@
     <hyperlink ref="D15" r:id="rId2" xr:uid="{8A4FF2B5-4B6B-44D6-AA37-2257F9852D45}"/>
     <hyperlink ref="A17" r:id="rId3" xr:uid="{528F5FE6-1479-40BB-A002-8A1E7211AB8C}"/>
     <hyperlink ref="D24" r:id="rId4" xr:uid="{DE2913A7-D3DA-46B3-83F9-C18D6E3ED24C}"/>
+    <hyperlink ref="A26" r:id="rId5" xr:uid="{E015E512-E9F6-4616-8A1F-85BBEAE8C64B}"/>
+    <hyperlink ref="D31" r:id="rId6" xr:uid="{39EBFCD6-D777-42F7-A268-B858B216B9BF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId5"/>
+  <pageSetup orientation="portrait" r:id="rId7"/>
+  <drawing r:id="rId8"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
AllNodesDistanceKinBinaryTree - June 8th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{227E235B-5C9D-4AD6-8BCE-241180C89681}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B387D73A-A77C-4F93-881C-7A5CD65568FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="3" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="16" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="865" uniqueCount="659">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="875" uniqueCount="667">
   <si>
     <t>Statement</t>
   </si>
@@ -2112,6 +2112,30 @@
   </si>
   <si>
     <t>Declare max heap and min heap to store first half and second half of sorted array</t>
+  </si>
+  <si>
+    <t>105. Construct Binary Tree from Preorder and Inorder Traversal</t>
+  </si>
+  <si>
+    <t>use inorder arr to keep track of number of nodes in left and right subtree</t>
+  </si>
+  <si>
+    <t>dfs 0, n-1</t>
+  </si>
+  <si>
+    <t>call dfs for left and right tree</t>
+  </si>
+  <si>
+    <t>iterate from preorder arr</t>
+  </si>
+  <si>
+    <t>863. All Nodes Distance K in Binary Tree</t>
+  </si>
+  <si>
+    <t>get parent map from dfs</t>
+  </si>
+  <si>
+    <t>do bfs using queue till k==0</t>
   </si>
 </sst>
 </file>
@@ -2304,7 +2328,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3"/>
@@ -2325,6 +2349,7 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="3" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="4" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="Bad" xfId="5" builtinId="27"/>
@@ -4480,6 +4505,94 @@
         <a:xfrm>
           <a:off x="3876675" y="13916025"/>
           <a:ext cx="2600688" cy="1886213"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>638175</xdr:colOff>
+      <xdr:row>85</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4286759</xdr:colOff>
+      <xdr:row>101</xdr:row>
+      <xdr:rowOff>133785</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9DBA0465-4634-AE68-4EB7-10339BF3D9DE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3457575" y="16259175"/>
+          <a:ext cx="3648584" cy="3115110"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>238125</xdr:colOff>
+      <xdr:row>104</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4648816</xdr:colOff>
+      <xdr:row>125</xdr:row>
+      <xdr:rowOff>172030</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CBDA63E5-67C6-A016-61DC-60A29CB513E2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3057525" y="19831050"/>
+          <a:ext cx="4410691" cy="4153480"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -10180,7 +10293,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36268CC4-0AC5-4653-846F-9B607EC203E4}">
-  <dimension ref="A1:D84"/>
+  <dimension ref="A1:D127"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -10414,13 +10527,65 @@
         <v>592</v>
       </c>
     </row>
-    <row r="83" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D83" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="84" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C84" s="5"/>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" s="12" t="s">
+        <v>659</v>
+      </c>
+      <c r="D85" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D86" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D87" t="s">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D88" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D102" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C103" s="5"/>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A104" s="12" t="s">
+        <v>664</v>
+      </c>
+      <c r="D104" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D105" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="126" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D126" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="127" spans="3:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C127" s="18"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -10436,9 +10601,13 @@
     <hyperlink ref="D71" r:id="rId10" xr:uid="{E4D3E62A-5D0C-43E7-81E1-D06ADCFC6A65}"/>
     <hyperlink ref="A73" r:id="rId11" xr:uid="{2EE4C200-CFE1-4C5B-9E3B-162FCF083A8E}"/>
     <hyperlink ref="D83" r:id="rId12" xr:uid="{1559CE54-3E65-43EB-BF5B-D49C6184A518}"/>
+    <hyperlink ref="A85" r:id="rId13" xr:uid="{66262CAD-2CF3-4CE1-8FBF-B87E227AE1CF}"/>
+    <hyperlink ref="D102" r:id="rId14" xr:uid="{A245F17E-5E8A-4545-8DB6-83AA1593FBF1}"/>
+    <hyperlink ref="A104" r:id="rId15" xr:uid="{7AC22602-C2D3-4582-9D2E-6C59BDD601DF}"/>
+    <hyperlink ref="D126" r:id="rId16" xr:uid="{00B99E80-16F3-405D-A7D3-4D641851B2D8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId13"/>
+  <drawing r:id="rId17"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
RemoveAllAdjacentDuplicatesinStringII - June 9th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B387D73A-A77C-4F93-881C-7A5CD65568FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ABA8F6A-4AC5-40C3-99B2-3F198F6ABB69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="16" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="2" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="875" uniqueCount="667">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="891" uniqueCount="680">
   <si>
     <t>Statement</t>
   </si>
@@ -2136,6 +2136,45 @@
   </si>
   <si>
     <t>do bfs using queue till k==0</t>
+  </si>
+  <si>
+    <t>Inorder Successor in BST</t>
+  </si>
+  <si>
+    <t>leetcode-premium</t>
+  </si>
+  <si>
+    <t>use queue to do inorder traversal</t>
+  </si>
+  <si>
+    <t>return next element when you get x while iterating - O(n) so bad, expected O(logn)</t>
+  </si>
+  <si>
+    <t>if x has right child then -</t>
+  </si>
+  <si>
+    <t>move 1 right and return left most child</t>
+  </si>
+  <si>
+    <t>else -</t>
+  </si>
+  <si>
+    <t>return latest left most while iterating from the root to x</t>
+  </si>
+  <si>
+    <t>173. Binary Search Tree Iterator</t>
+  </si>
+  <si>
+    <t>inorder traversal - iterative</t>
+  </si>
+  <si>
+    <t>1209. Remove All Adjacent Duplicates in String II</t>
+  </si>
+  <si>
+    <t>keep track of char count till now in stack</t>
+  </si>
+  <si>
+    <t>if count till now is k-1 and current char is same as prev pop else just add this</t>
   </si>
 </sst>
 </file>
@@ -4601,6 +4640,94 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>876300</xdr:colOff>
+      <xdr:row>128</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4172410</xdr:colOff>
+      <xdr:row>140</xdr:row>
+      <xdr:rowOff>314</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{049DFD97-7632-F84C-3D27-8EE15D50031B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3695700" y="24422100"/>
+          <a:ext cx="3296110" cy="2248214"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>142</xdr:row>
+      <xdr:rowOff>19051</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4857750</xdr:colOff>
+      <xdr:row>151</xdr:row>
+      <xdr:rowOff>152401</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Picture 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EDBE552B-C911-3FBA-1433-E7A6C0A5E342}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2847975" y="27070051"/>
+          <a:ext cx="4829175" cy="1847850"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -5131,6 +5258,50 @@
         <a:xfrm>
           <a:off x="2886076" y="9763125"/>
           <a:ext cx="4800600" cy="1057423"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1123950</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3724638</xdr:colOff>
+      <xdr:row>62</xdr:row>
+      <xdr:rowOff>162010</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{023658CC-E503-45F1-CF8E-914F7A55A204}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3943350" y="11363325"/>
+          <a:ext cx="2600688" cy="609685"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -10293,7 +10464,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36268CC4-0AC5-4653-846F-9B607EC203E4}">
-  <dimension ref="A1:D127"/>
+  <dimension ref="A1:D153"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -10579,13 +10750,76 @@
         <v>666</v>
       </c>
     </row>
-    <row r="126" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D126" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="127" spans="3:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C127" s="18"/>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A128" s="14" t="s">
+        <v>667</v>
+      </c>
+      <c r="D128" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A129" s="2" t="s">
+        <v>668</v>
+      </c>
+      <c r="D129" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D130" s="4"/>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D131" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D132" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D133" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D134" t="s">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D140" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C141" s="5"/>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A142" s="12" t="s">
+        <v>675</v>
+      </c>
+      <c r="D142" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="152" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D152" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="153" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C153" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -10605,9 +10839,14 @@
     <hyperlink ref="D102" r:id="rId14" xr:uid="{A245F17E-5E8A-4545-8DB6-83AA1593FBF1}"/>
     <hyperlink ref="A104" r:id="rId15" xr:uid="{7AC22602-C2D3-4582-9D2E-6C59BDD601DF}"/>
     <hyperlink ref="D126" r:id="rId16" xr:uid="{00B99E80-16F3-405D-A7D3-4D641851B2D8}"/>
+    <hyperlink ref="A129" r:id="rId17" xr:uid="{EF880B29-FD9F-4125-8881-D6F398964EA3}"/>
+    <hyperlink ref="A128" r:id="rId18" xr:uid="{350A241D-6AA2-4062-8132-6F907333AEA3}"/>
+    <hyperlink ref="D140" r:id="rId19" xr:uid="{EAE54D37-109D-4231-B46E-AE213D8D5674}"/>
+    <hyperlink ref="A142" r:id="rId20" xr:uid="{208DBEE3-DC36-4BCC-839D-302642CE3DB9}"/>
+    <hyperlink ref="D152" r:id="rId21" xr:uid="{A293AB57-9F78-405F-830B-16419EF6197E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId17"/>
+  <drawing r:id="rId22"/>
 </worksheet>
 </file>
 
@@ -10969,7 +11208,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5D8A62A-F83B-49C3-B94F-89CCE841A84E}">
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -11225,6 +11464,27 @@
     </row>
     <row r="58" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C58" s="5"/>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="12" t="s">
+        <v>677</v>
+      </c>
+      <c r="D59" t="s">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D60" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D63" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C64" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -11244,9 +11504,11 @@
     <hyperlink ref="D49" r:id="rId14" xr:uid="{7A49C60D-CF07-482B-88E8-BACCE2595D8E}"/>
     <hyperlink ref="A51" r:id="rId15" xr:uid="{20507E66-8AEE-4B9C-850A-CA9238583EC3}"/>
     <hyperlink ref="D57" r:id="rId16" xr:uid="{79F280B3-41CF-4A9A-A469-C35B9DB33B8A}"/>
+    <hyperlink ref="A59" r:id="rId17" xr:uid="{FC8EB95F-8A6C-4A54-A458-0553E36DE4B7}"/>
+    <hyperlink ref="D63" r:id="rId18" xr:uid="{E7F78474-1A2A-4D71-AE53-3FA1D5BD4142}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId17"/>
+  <drawing r:id="rId19"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
SumofSubarrayMinimums - June 18th
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A7C0C57-5855-4169-A9AF-0CFC953CD575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED269AA6-FF11-43B6-B9A5-9DDD9E4A0079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="2" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="5" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="greedy" sheetId="10" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="904" uniqueCount="687">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="910" uniqueCount="692">
   <si>
     <t>Statement</t>
   </si>
@@ -2197,6 +2197,21 @@
   </si>
   <si>
     <t>numerator and denominator should be converted to long</t>
+  </si>
+  <si>
+    <t>907. Sum of Subarray Minimums</t>
+  </si>
+  <si>
+    <t>for each element we should find the next least element on both sides</t>
+  </si>
+  <si>
+    <t>for 3 its 3 * (0-1) * (1-0)</t>
+  </si>
+  <si>
+    <t>for 1 its 1 * (1-(-1)) * (n-1)</t>
+  </si>
+  <si>
+    <t>i.e. 1 is part of sub-arrays that have elements greater than 1 on right and left</t>
   </si>
 </sst>
 </file>
@@ -6840,6 +6855,50 @@
         <a:xfrm>
           <a:off x="4867275" y="14049375"/>
           <a:ext cx="1133633" cy="419158"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>79</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4914900</xdr:colOff>
+      <xdr:row>85</xdr:row>
+      <xdr:rowOff>152566</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Picture 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6C942BAB-8547-939C-C936-76E33B968FE1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3448050" y="15154275"/>
+          <a:ext cx="4857750" cy="1190791"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -11953,7 +12012,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDA924A8-9114-46BA-B39C-6743F04F80F3}">
-  <dimension ref="A1:D78"/>
+  <dimension ref="A1:D87"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50.85546875" customWidth="1"/>
@@ -12342,6 +12401,37 @@
     </row>
     <row r="78" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C78" s="5"/>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" s="12" t="s">
+        <v>687</v>
+      </c>
+      <c r="D79" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D80" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="81" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D81" t="s">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="82" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D82" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="86" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D86" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C87" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -12367,10 +12457,12 @@
     <hyperlink ref="C64" r:id="rId20" xr:uid="{E66C42DF-1C90-4082-AE05-B49055644FDA}"/>
     <hyperlink ref="A73" r:id="rId21" xr:uid="{02DCB243-3895-4B62-B9BD-D9D4A1D7091F}"/>
     <hyperlink ref="D77" r:id="rId22" xr:uid="{31F07A9C-A9D1-4B48-B801-6FECB16DE579}"/>
+    <hyperlink ref="A79" r:id="rId23" xr:uid="{3A9D7590-CAC7-4070-98C6-D190FF2D0A06}"/>
+    <hyperlink ref="D86" r:id="rId24" xr:uid="{89FCF0CB-FB19-4DF1-9317-7405B8920DCD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId23"/>
-  <drawing r:id="rId24"/>
+  <pageSetup orientation="portrait" r:id="rId25"/>
+  <drawing r:id="rId26"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
SubarraySumEqualsK - June 21st 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,30 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED269AA6-FF11-43B6-B9A5-9DDD9E4A0079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3BBA9B4-FB6E-4A37-B185-DCA3C2CBCB16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="5" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="4" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
-    <sheet name="greedy" sheetId="10" r:id="rId1"/>
-    <sheet name="Parenthesis" sheetId="7" r:id="rId2"/>
-    <sheet name="Stack" sheetId="8" r:id="rId3"/>
-    <sheet name="Math" sheetId="20" r:id="rId4"/>
-    <sheet name="Queue" sheetId="9" r:id="rId5"/>
-    <sheet name="Array" sheetId="4" r:id="rId6"/>
-    <sheet name="Matrix" sheetId="5" r:id="rId7"/>
-    <sheet name="Linked list" sheetId="3" r:id="rId8"/>
-    <sheet name="Rain water trap" sheetId="1" r:id="rId9"/>
-    <sheet name="Low level design" sheetId="11" r:id="rId10"/>
-    <sheet name="Graph" sheetId="12" r:id="rId11"/>
-    <sheet name="Dictionary" sheetId="13" r:id="rId12"/>
-    <sheet name="template" sheetId="2" r:id="rId13"/>
-    <sheet name="Sorting Algorithms" sheetId="15" r:id="rId14"/>
-    <sheet name="Binary search" sheetId="16" r:id="rId15"/>
-    <sheet name="dfs" sheetId="17" r:id="rId16"/>
-    <sheet name="dp" sheetId="6" r:id="rId17"/>
-    <sheet name="Tree" sheetId="19" r:id="rId18"/>
-    <sheet name="String" sheetId="18" r:id="rId19"/>
+    <sheet name="Parenthesis" sheetId="7" r:id="rId1"/>
+    <sheet name="Stack" sheetId="8" r:id="rId2"/>
+    <sheet name="Math" sheetId="20" r:id="rId3"/>
+    <sheet name="Queue" sheetId="9" r:id="rId4"/>
+    <sheet name="Array" sheetId="4" r:id="rId5"/>
+    <sheet name="Matrix" sheetId="5" r:id="rId6"/>
+    <sheet name="Linked list" sheetId="3" r:id="rId7"/>
+    <sheet name="Rain water trap" sheetId="1" r:id="rId8"/>
+    <sheet name="Low level design" sheetId="11" r:id="rId9"/>
+    <sheet name="Graph" sheetId="12" r:id="rId10"/>
+    <sheet name="Dictionary" sheetId="13" r:id="rId11"/>
+    <sheet name="template" sheetId="2" r:id="rId12"/>
+    <sheet name="Sorting Algorithms" sheetId="15" r:id="rId13"/>
+    <sheet name="Binary search" sheetId="16" r:id="rId14"/>
+    <sheet name="dfs" sheetId="17" r:id="rId15"/>
+    <sheet name="dp" sheetId="6" r:id="rId16"/>
+    <sheet name="Tree" sheetId="19" r:id="rId17"/>
+    <sheet name="String" sheetId="18" r:id="rId18"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -50,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="910" uniqueCount="692">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="934" uniqueCount="715">
   <si>
     <t>Statement</t>
   </si>
@@ -2212,6 +2211,75 @@
   </si>
   <si>
     <t>i.e. 1 is part of sub-arrays that have elements greater than 1 on right and left</t>
+  </si>
+  <si>
+    <t>1504. Count Submatrices With All Ones</t>
+  </si>
+  <si>
+    <t>find histogram possible at each row</t>
+  </si>
+  <si>
+    <t>find corresponding array subArray minimums</t>
+  </si>
+  <si>
+    <t>688. Knight Probability in Chessboard</t>
+  </si>
+  <si>
+    <t>there will be 8^k steps possible</t>
+  </si>
+  <si>
+    <t>dfs(k, r, c)</t>
+  </si>
+  <si>
+    <t>if outofbounds return 0</t>
+  </si>
+  <si>
+    <t>if k == 0 return 1</t>
+  </si>
+  <si>
+    <t>dfs in 8 directions like r+2, c+1 …</t>
+  </si>
+  <si>
+    <t>1268. Search Suggestions System</t>
+  </si>
+  <si>
+    <t>keep maxHeap</t>
+  </si>
+  <si>
+    <t>for each letter from searchWord iterate compare through products</t>
+  </si>
+  <si>
+    <t>and add to maxHeap with maxSize == 3</t>
+  </si>
+  <si>
+    <t>52. N-Queens II</t>
+  </si>
+  <si>
+    <t>start dfs from row=0</t>
+  </si>
+  <si>
+    <t>if row reaches n return 1</t>
+  </si>
+  <si>
+    <t>if col is used or diagonal1 is used or diagonal2 is used continue</t>
+  </si>
+  <si>
+    <t>for each column</t>
+  </si>
+  <si>
+    <t>backtrack with set for col, row-col, row+col (row-col is same for d1 and r+c is same for d2)</t>
+  </si>
+  <si>
+    <t>dfs with r+1</t>
+  </si>
+  <si>
+    <t>560. Subarray Sum Equals K</t>
+  </si>
+  <si>
+    <t>keep in hashMap prefix sums till now</t>
+  </si>
+  <si>
+    <t>if map has sum - k then there is k possible</t>
   </si>
 </sst>
 </file>
@@ -5787,6 +5855,50 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>47626</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4867276</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>171733</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{82DE80EC-4634-862C-9195-D13B53048FE0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2867026" y="9763125"/>
+          <a:ext cx="4819650" cy="2029108"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -6907,6 +7019,50 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1314450</xdr:colOff>
+      <xdr:row>88</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3438821</xdr:colOff>
+      <xdr:row>97</xdr:row>
+      <xdr:rowOff>162183</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Picture 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ACD8ECCE-F543-3A47-C0F2-F62C28195183}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4705350" y="16792575"/>
+          <a:ext cx="2124371" cy="1848108"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -7168,6 +7324,138 @@
         <a:xfrm>
           <a:off x="3409950" y="19097625"/>
           <a:ext cx="3886742" cy="2200582"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1209675</xdr:colOff>
+      <xdr:row>113</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3886574</xdr:colOff>
+      <xdr:row>127</xdr:row>
+      <xdr:rowOff>152768</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D6CDDBD4-CFEC-934C-8442-1C4EFA7C3A30}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4029075" y="21707475"/>
+          <a:ext cx="2676899" cy="2638793"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>130</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4905375</xdr:colOff>
+      <xdr:row>158</xdr:row>
+      <xdr:rowOff>86471</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{70391740-A5E9-333A-1209-830FA7BBCACF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2857500" y="24841200"/>
+          <a:ext cx="4867275" cy="5344271"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>161</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4857750</xdr:colOff>
+      <xdr:row>177</xdr:row>
+      <xdr:rowOff>114733</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0467847F-B86A-2F28-716B-A51B6727CE1F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2847975" y="30727650"/>
+          <a:ext cx="4829175" cy="3105583"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -8140,8 +8428,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55C26914-8137-4079-AF30-EE7EDC55D866}">
-  <dimension ref="A1:D2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AAA3DB6-B181-432C-9183-F47857237DA8}">
+  <dimension ref="A1:D33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -8169,119 +8457,157 @@
     <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C2" s="5"/>
     </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="D3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D9" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C10" s="5"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="D11" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D12" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D13" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D14" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D15" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D16" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D18" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C19" s="5"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="D20" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D21" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D22" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D23" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D25" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C26" s="5"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="13" t="s">
+        <v>546</v>
+      </c>
+      <c r="D27" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D28" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D29" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D30" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D32" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="3:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C33" s="5"/>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{A24F529E-D0E4-4D7C-8940-2EF8A048917C}"/>
+    <hyperlink ref="D9" r:id="rId2" xr:uid="{3733EA6B-CA32-4A95-A915-04BBA49179CD}"/>
+    <hyperlink ref="A11" r:id="rId3" xr:uid="{DF0AC1E1-3EA5-40DA-A2FC-0C7AB70D8D78}"/>
+    <hyperlink ref="D18" r:id="rId4" xr:uid="{305DB711-02E8-46A6-A4B2-FBE63ADC1454}"/>
+    <hyperlink ref="A20" r:id="rId5" xr:uid="{8CA448EC-D236-455D-8BAE-429EDAA19260}"/>
+    <hyperlink ref="D25" r:id="rId6" xr:uid="{E0D5FDE7-5097-47AC-89CC-3DD086203364}"/>
+    <hyperlink ref="A27" r:id="rId7" xr:uid="{062EB6D1-B6C8-4E86-BC47-6B515EB90A7C}"/>
+    <hyperlink ref="D32" r:id="rId8" xr:uid="{AADFAA3D-E8F3-4A0F-8516-9B9143A6E576}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId9"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7BE8B5F-B3C3-43A1-BD9C-D35CE748D483}">
-  <dimension ref="A1:D27"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="42.28515625" customWidth="1"/>
-    <col min="2" max="2" width="73.85546875" customWidth="1"/>
-    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="91.7109375" customWidth="1"/>
-    <col min="13" max="13" width="6.7109375" customWidth="1"/>
-    <col min="14" max="14" width="8.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C2" s="5"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="D3" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D9" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C10" s="5"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="D11" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D17" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C18" s="5"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
-        <v>239</v>
-      </c>
-      <c r="D19" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D20" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D21" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D22" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D26" s="2" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C27" s="5"/>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" xr:uid="{976A6329-CE7B-45FA-9EC8-39B157036788}"/>
-    <hyperlink ref="D9" r:id="rId2" xr:uid="{60C7CCA8-6DFD-471B-BE7B-FBA6AA3D39EF}"/>
-    <hyperlink ref="A11" r:id="rId3" xr:uid="{B613807D-978E-4CA0-928A-B9CD9644C8F6}"/>
-    <hyperlink ref="D17" r:id="rId4" xr:uid="{6226ADC2-6F8E-4914-A1E9-DA822FBF2A00}"/>
-    <hyperlink ref="A19" r:id="rId5" xr:uid="{1C07BF01-9F0C-4351-A36A-823B3D1421E1}"/>
-    <hyperlink ref="D26" r:id="rId6" xr:uid="{DD2E06CD-E5AB-4B10-B597-A62BC91B4CE4}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId7"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E87A3A0-D815-41F9-954B-826D58641E2B}">
   <dimension ref="A1:D322"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9063,7 +9389,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{170CF2C0-E5DC-4FCA-8D73-E7E5C7297110}">
   <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9171,7 +9497,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10429FF1-7DBA-415E-968E-9D236B8DC32D}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9206,7 +9532,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0397D5EA-9127-4F39-A242-D8D4A93871ED}">
   <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9299,7 +9625,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC70315-55E0-46CA-8156-25A8AD92E211}">
   <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9442,7 +9768,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E9C6576-B939-40FE-9164-B9EF7525065D}">
   <dimension ref="A1:D28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9569,7 +9895,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76846435-1279-41EE-B6BA-33F004CE9CD2}">
   <dimension ref="A1:D305"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -10743,7 +11069,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36268CC4-0AC5-4653-846F-9B607EC203E4}">
   <dimension ref="A1:D153"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -11131,9 +11457,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BDF4E8D-D4E1-4180-9015-2E66B34CBB41}">
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -11282,13 +11608,39 @@
         <v>602</v>
       </c>
     </row>
-    <row r="49" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D49" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="50" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C50" s="5"/>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="12" t="s">
+        <v>701</v>
+      </c>
+      <c r="D51" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D52" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D53" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D62" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C63" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -11300,194 +11652,16 @@
     <hyperlink ref="D33" r:id="rId6" xr:uid="{20E93955-F6EE-4945-AF7A-5E21E68FD72A}"/>
     <hyperlink ref="A35" r:id="rId7" xr:uid="{EBEB57E2-D61C-429F-9ED4-13410C4795F5}"/>
     <hyperlink ref="D49" r:id="rId8" xr:uid="{E33833DE-847A-4DF8-93F7-4EAA9509A09E}"/>
+    <hyperlink ref="A51" r:id="rId9" xr:uid="{469541BF-F016-436B-8D3F-318C1F21C4BB}"/>
+    <hyperlink ref="D62" r:id="rId10" xr:uid="{A1E7AB8D-8141-4EC7-B5D4-34BB47C56BF0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId9"/>
-  <drawing r:id="rId10"/>
+  <pageSetup orientation="portrait" r:id="rId11"/>
+  <drawing r:id="rId12"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AAA3DB6-B181-432C-9183-F47857237DA8}">
-  <dimension ref="A1:D33"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="42.28515625" customWidth="1"/>
-    <col min="2" max="2" width="73.85546875" customWidth="1"/>
-    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="91.7109375" customWidth="1"/>
-    <col min="13" max="13" width="6.7109375" customWidth="1"/>
-    <col min="14" max="14" width="8.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C2" s="5"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
-        <v>117</v>
-      </c>
-      <c r="D3" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D4" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D5" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D9" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C10" s="5"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="17" t="s">
-        <v>122</v>
-      </c>
-      <c r="D11" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D12" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D13" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D14" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D15" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D16" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D18" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C19" s="5"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="12" t="s">
-        <v>141</v>
-      </c>
-      <c r="D20" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D21" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D22" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D23" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D25" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C26" s="5"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="13" t="s">
-        <v>546</v>
-      </c>
-      <c r="D27" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D28" t="s">
-        <v>548</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D29" t="s">
-        <v>549</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D30" t="s">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D32" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="33" spans="3:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C33" s="5"/>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" xr:uid="{A24F529E-D0E4-4D7C-8940-2EF8A048917C}"/>
-    <hyperlink ref="D9" r:id="rId2" xr:uid="{3733EA6B-CA32-4A95-A915-04BBA49179CD}"/>
-    <hyperlink ref="A11" r:id="rId3" xr:uid="{DF0AC1E1-3EA5-40DA-A2FC-0C7AB70D8D78}"/>
-    <hyperlink ref="D18" r:id="rId4" xr:uid="{305DB711-02E8-46A6-A4B2-FBE63ADC1454}"/>
-    <hyperlink ref="A20" r:id="rId5" xr:uid="{8CA448EC-D236-455D-8BAE-429EDAA19260}"/>
-    <hyperlink ref="D25" r:id="rId6" xr:uid="{E0D5FDE7-5097-47AC-89CC-3DD086203364}"/>
-    <hyperlink ref="A27" r:id="rId7" xr:uid="{062EB6D1-B6C8-4E86-BC47-6B515EB90A7C}"/>
-    <hyperlink ref="D32" r:id="rId8" xr:uid="{AADFAA3D-E8F3-4A0F-8516-9B9143A6E576}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId9"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5D8A62A-F83B-49C3-B94F-89CCE841A84E}">
   <dimension ref="A1:D70"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -11811,7 +11985,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E85A04F9-4C9C-43BD-8A69-EE24F451F616}">
   <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -11882,7 +12056,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51C4CDD9-9363-46B2-A2D8-BE11DE99714D}">
   <dimension ref="A1:D32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -12010,9 +12184,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDA924A8-9114-46BA-B39C-6743F04F80F3}">
-  <dimension ref="A1:D87"/>
+  <dimension ref="A1:D99"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50.85546875" customWidth="1"/>
@@ -12415,23 +12589,44 @@
         <v>689</v>
       </c>
     </row>
-    <row r="81" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D81" t="s">
         <v>690</v>
       </c>
     </row>
-    <row r="82" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D82" t="s">
         <v>691</v>
       </c>
     </row>
-    <row r="86" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D86" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="87" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C87" s="5"/>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88" s="12" t="s">
+        <v>712</v>
+      </c>
+      <c r="D88" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D89" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="98" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D98" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C99" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -12459,16 +12654,18 @@
     <hyperlink ref="D77" r:id="rId22" xr:uid="{31F07A9C-A9D1-4B48-B801-6FECB16DE579}"/>
     <hyperlink ref="A79" r:id="rId23" xr:uid="{3A9D7590-CAC7-4070-98C6-D190FF2D0A06}"/>
     <hyperlink ref="D86" r:id="rId24" xr:uid="{89FCF0CB-FB19-4DF1-9317-7405B8920DCD}"/>
+    <hyperlink ref="A88" r:id="rId25" xr:uid="{2F8DE2A5-C950-4C86-822F-3ADDFE77575A}"/>
+    <hyperlink ref="D98" r:id="rId26" xr:uid="{06803DC5-FCC5-49E2-9BD8-222808AB2171}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId25"/>
-  <drawing r:id="rId26"/>
+  <pageSetup orientation="portrait" r:id="rId27"/>
+  <drawing r:id="rId28"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83AD0EA2-442A-436B-AA00-D0DF9DB7227A}">
-  <dimension ref="A1:D113"/>
+  <dimension ref="A1:D179"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -12692,8 +12889,106 @@
         <v>9</v>
       </c>
     </row>
-    <row r="113" spans="3:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C113" s="5"/>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A114" s="12" t="s">
+        <v>692</v>
+      </c>
+      <c r="D114" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D115" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D128" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C129" s="5"/>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A130" s="12" t="s">
+        <v>695</v>
+      </c>
+      <c r="D130" t="s">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D131" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D132" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D133" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D134" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="159" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D159" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="160" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C160" s="5"/>
+    </row>
+    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A161" s="13" t="s">
+        <v>705</v>
+      </c>
+      <c r="D161" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D162" t="s">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D163" t="s">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D164" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D165" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D166" t="s">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="178" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D178" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="179" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C179" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -12709,14 +13004,20 @@
     <hyperlink ref="D98" r:id="rId10" xr:uid="{01BE9452-404A-4580-8C56-B003AE57914E}"/>
     <hyperlink ref="A100" r:id="rId11" xr:uid="{CECF130D-CC26-4D13-BA9A-5504D8EA8278}"/>
     <hyperlink ref="D112" r:id="rId12" xr:uid="{5BF85361-6BEF-4029-A6B4-31A2721F2F6D}"/>
+    <hyperlink ref="A114" r:id="rId13" xr:uid="{CDB2052A-A6D4-4128-B7DA-E1384C5E89E1}"/>
+    <hyperlink ref="D128" r:id="rId14" xr:uid="{205891C5-5617-4AA6-ABA6-169A50CB7595}"/>
+    <hyperlink ref="A130" r:id="rId15" xr:uid="{F7C57A2A-CDA7-458A-BB51-A3BD5AFAE78B}"/>
+    <hyperlink ref="D159" r:id="rId16" xr:uid="{428FB876-5055-4395-9A15-BD708B95F936}"/>
+    <hyperlink ref="A161" r:id="rId17" xr:uid="{D3BFCD62-E0EB-4F37-BC7A-16BE541C24E6}"/>
+    <hyperlink ref="D178" r:id="rId18" xr:uid="{F40B6475-1CC8-454A-A0AA-FA3B46403CB7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId13"/>
-  <drawing r:id="rId14"/>
+  <pageSetup orientation="portrait" r:id="rId19"/>
+  <drawing r:id="rId20"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56E27646-854C-4719-A92C-78F24A8C7C41}">
   <dimension ref="A1:D100"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13129,7 +13430,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CE8EF6C-9017-4EEF-A2CD-F2424B35AA25}">
   <dimension ref="A1:D68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13386,4 +13687,111 @@
   <pageSetup orientation="portrait" r:id="rId9"/>
   <drawing r:id="rId10"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7BE8B5F-B3C3-43A1-BD9C-D35CE748D483}">
+  <dimension ref="A1:D27"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="2" max="2" width="73.85546875" customWidth="1"/>
+    <col min="3" max="3" width="42.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.7109375" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="D3" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D9" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C10" s="5"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="D11" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D17" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C18" s="5"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="D19" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D20" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D21" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D22" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D26" s="2" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C27" s="5"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{976A6329-CE7B-45FA-9EC8-39B157036788}"/>
+    <hyperlink ref="D9" r:id="rId2" xr:uid="{60C7CCA8-6DFD-471B-BE7B-FBA6AA3D39EF}"/>
+    <hyperlink ref="A11" r:id="rId3" xr:uid="{B613807D-978E-4CA0-928A-B9CD9644C8F6}"/>
+    <hyperlink ref="D17" r:id="rId4" xr:uid="{6226ADC2-6F8E-4914-A1E9-DA822FBF2A00}"/>
+    <hyperlink ref="A19" r:id="rId5" xr:uid="{1C07BF01-9F0C-4351-A36A-823B3D1421E1}"/>
+    <hyperlink ref="D26" r:id="rId6" xr:uid="{DD2E06CD-E5AB-4B10-B597-A62BC91B4CE4}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId7"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
carPooling - June 22nd 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3BBA9B4-FB6E-4A37-B185-DCA3C2CBCB16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B44D4EB7-738B-4F42-BA20-D228571FB3A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="4" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="934" uniqueCount="715">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="938" uniqueCount="718">
   <si>
     <t>Statement</t>
   </si>
@@ -2280,6 +2280,15 @@
   </si>
   <si>
     <t>if map has sum - k then there is k possible</t>
+  </si>
+  <si>
+    <t>1094. Car Pooling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">keep an array of size 1000, add curr to arr[start], and subtract from arr[end] </t>
+  </si>
+  <si>
+    <t>iterate and find if at any point capacity is breached</t>
   </si>
 </sst>
 </file>
@@ -7055,6 +7064,50 @@
         <a:xfrm>
           <a:off x="4705350" y="16792575"/>
           <a:ext cx="2124371" cy="1848108"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>952500</xdr:colOff>
+      <xdr:row>100</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3953294</xdr:colOff>
+      <xdr:row>102</xdr:row>
+      <xdr:rowOff>171518</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Picture 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{706F69E1-C3AE-BABB-0CA8-C8EB9BB9639D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4343400" y="19116675"/>
+          <a:ext cx="3000794" cy="485843"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -12186,7 +12239,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDA924A8-9114-46BA-B39C-6743F04F80F3}">
-  <dimension ref="A1:D99"/>
+  <dimension ref="A1:D104"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50.85546875" customWidth="1"/>
@@ -12620,13 +12673,34 @@
         <v>714</v>
       </c>
     </row>
-    <row r="98" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D98" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="99" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C99" s="5"/>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A100" s="12" t="s">
+        <v>715</v>
+      </c>
+      <c r="D100" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D101" t="s">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D103" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C104" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -12656,10 +12730,12 @@
     <hyperlink ref="D86" r:id="rId24" xr:uid="{89FCF0CB-FB19-4DF1-9317-7405B8920DCD}"/>
     <hyperlink ref="A88" r:id="rId25" xr:uid="{2F8DE2A5-C950-4C86-822F-3ADDFE77575A}"/>
     <hyperlink ref="D98" r:id="rId26" xr:uid="{06803DC5-FCC5-49E2-9BD8-222808AB2171}"/>
+    <hyperlink ref="A100" r:id="rId27" xr:uid="{18A766A6-5CD3-4B46-84D5-8F39B78AA967}"/>
+    <hyperlink ref="D103" r:id="rId28" xr:uid="{E752EED3-858C-4BCB-9416-7073E040EB09}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId27"/>
-  <drawing r:id="rId28"/>
+  <pageSetup orientation="portrait" r:id="rId29"/>
+  <drawing r:id="rId30"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
MaxOfMinDifferenceOfSubsequenceOfSizeK - June 26th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B44D4EB7-738B-4F42-BA20-D228571FB3A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{913EF82E-FC52-45A3-B7BE-2F1BC4DC2A4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="4" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="938" uniqueCount="718">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="945" uniqueCount="724">
   <si>
     <t>Statement</t>
   </si>
@@ -2289,6 +2289,24 @@
   </si>
   <si>
     <t>iterate and find if at any point capacity is breached</t>
+  </si>
+  <si>
+    <t>2099. Find Subsequence of Length K With the Largest Sum</t>
+  </si>
+  <si>
+    <t>use minHeap to store k max elements indexes</t>
+  </si>
+  <si>
+    <t>sort index and return val</t>
+  </si>
+  <si>
+    <t>copy nums &amp; get kth largest from quick-select</t>
+  </si>
+  <si>
+    <t xml:space="preserve">use map to store k largest elements counts </t>
+  </si>
+  <si>
+    <t>iterate through nums and add them to result array</t>
   </si>
 </sst>
 </file>
@@ -7108,6 +7126,50 @@
         <a:xfrm>
           <a:off x="4343400" y="19116675"/>
           <a:ext cx="3000794" cy="485843"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>885825</xdr:colOff>
+      <xdr:row>107</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4153356</xdr:colOff>
+      <xdr:row>111</xdr:row>
+      <xdr:rowOff>162038</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Picture 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{850713AD-1033-32FD-748F-94581486049C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4276725" y="20497800"/>
+          <a:ext cx="3267531" cy="809738"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -12239,7 +12301,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDA924A8-9114-46BA-B39C-6743F04F80F3}">
-  <dimension ref="A1:D104"/>
+  <dimension ref="A1:D113"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50.85546875" customWidth="1"/>
@@ -12701,6 +12763,45 @@
     </row>
     <row r="104" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C104" s="5"/>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A105" s="14" t="s">
+        <v>718</v>
+      </c>
+      <c r="D105" t="s">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D106" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D107" s="4"/>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D108" t="s">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D109" t="s">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D110" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D112" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="3:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C113" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -12732,10 +12833,12 @@
     <hyperlink ref="D98" r:id="rId26" xr:uid="{06803DC5-FCC5-49E2-9BD8-222808AB2171}"/>
     <hyperlink ref="A100" r:id="rId27" xr:uid="{18A766A6-5CD3-4B46-84D5-8F39B78AA967}"/>
     <hyperlink ref="D103" r:id="rId28" xr:uid="{E752EED3-858C-4BCB-9416-7073E040EB09}"/>
+    <hyperlink ref="A105" r:id="rId29" xr:uid="{18C707F3-7727-4F9A-AF34-3F3BFFC6358B}"/>
+    <hyperlink ref="D112" r:id="rId30" xr:uid="{1BF05C36-80DD-46E4-8328-4E3524495B39}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId29"/>
-  <drawing r:id="rId30"/>
+  <pageSetup orientation="portrait" r:id="rId31"/>
+  <drawing r:id="rId32"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
StringMatchinginanArray - June 27th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{913EF82E-FC52-45A3-B7BE-2F1BC4DC2A4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88A5A1FC-820B-4EF9-AD0E-050C963A3E49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="4" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="17" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="Parenthesis" sheetId="7" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="945" uniqueCount="724">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="949" uniqueCount="727">
   <si>
     <t>Statement</t>
   </si>
@@ -2307,6 +2307,15 @@
   </si>
   <si>
     <t>iterate through nums and add them to result array</t>
+  </si>
+  <si>
+    <t>1408. String Matching in an Array</t>
+  </si>
+  <si>
+    <t>join words by " "</t>
+  </si>
+  <si>
+    <t>for each word if first index and last index are different then add to list</t>
   </si>
 </sst>
 </file>
@@ -5918,6 +5927,50 @@
         <a:xfrm>
           <a:off x="2867026" y="9763125"/>
           <a:ext cx="4819650" cy="2029108"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>19051</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4895851</xdr:colOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>123935</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A7087285-19EE-A565-8176-3008C2FCB993}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2838451" y="12668250"/>
+          <a:ext cx="4876800" cy="790685"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -11574,7 +11627,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BDF4E8D-D4E1-4180-9015-2E66B34CBB41}">
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -11757,6 +11810,30 @@
     <row r="63" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C63" s="5"/>
     </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="14" t="s">
+        <v>724</v>
+      </c>
+      <c r="D64" t="s">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="65" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D65" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="66" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D66" s="4"/>
+    </row>
+    <row r="71" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D71" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C72" s="5"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" xr:uid="{21D017E7-6C7E-4EA6-AE55-30155D149EEC}"/>
@@ -11769,10 +11846,12 @@
     <hyperlink ref="D49" r:id="rId8" xr:uid="{E33833DE-847A-4DF8-93F7-4EAA9509A09E}"/>
     <hyperlink ref="A51" r:id="rId9" xr:uid="{469541BF-F016-436B-8D3F-318C1F21C4BB}"/>
     <hyperlink ref="D62" r:id="rId10" xr:uid="{A1E7AB8D-8141-4EC7-B5D4-34BB47C56BF0}"/>
+    <hyperlink ref="A64" r:id="rId11" xr:uid="{1DB3F9A6-4972-4DC8-97D9-576F47BAC21F}"/>
+    <hyperlink ref="D71" r:id="rId12" xr:uid="{0DA3D38D-1453-4A98-8E78-652910101E3B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId11"/>
-  <drawing r:id="rId12"/>
+  <pageSetup orientation="portrait" r:id="rId13"/>
+  <drawing r:id="rId14"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
MaximumSumofTwoNon-OverlappingSubarrays - July 2nd 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88A5A1FC-820B-4EF9-AD0E-050C963A3E49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5DCFD94-D8D6-41EF-A610-410965B99575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="17" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" activeTab="4" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="Parenthesis" sheetId="7" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="949" uniqueCount="727">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="954" uniqueCount="731">
   <si>
     <t>Statement</t>
   </si>
@@ -2316,6 +2316,18 @@
   </si>
   <si>
     <t>for each word if first index and last index are different then add to list</t>
+  </si>
+  <si>
+    <t>1031. Maximum Sum of Two Non-Overlapping Subarrays</t>
+  </si>
+  <si>
+    <t>take firstLen sums starting for each element, same for secondLen</t>
+  </si>
+  <si>
+    <t>so, max is current sum1 + all combinations from i + firstLen in sum2, O(n^2)</t>
+  </si>
+  <si>
+    <t>thus keep max till end to both sum1 and sum2</t>
   </si>
 </sst>
 </file>
@@ -7223,6 +7235,50 @@
         <a:xfrm>
           <a:off x="4276725" y="20497800"/>
           <a:ext cx="3267531" cy="809738"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>66676</xdr:colOff>
+      <xdr:row>114</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4867276</xdr:colOff>
+      <xdr:row>117</xdr:row>
+      <xdr:rowOff>152482</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="Picture 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{65334BB3-DB41-E06A-8912-AFD1B54AF4F6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3457576" y="21850350"/>
+          <a:ext cx="4800600" cy="590632"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -12380,7 +12436,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDA924A8-9114-46BA-B39C-6743F04F80F3}">
-  <dimension ref="A1:D113"/>
+  <dimension ref="A1:D119"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50.85546875" customWidth="1"/>
@@ -12435,7 +12491,7 @@
       <c r="C8" s="5"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="13" t="s">
         <v>157</v>
       </c>
     </row>
@@ -12549,7 +12605,7 @@
       <c r="C29" s="5"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="4" t="s">
+      <c r="A30" s="14" t="s">
         <v>326</v>
       </c>
       <c r="D30" t="s">
@@ -12879,14 +12935,40 @@
         <v>9</v>
       </c>
     </row>
-    <row r="113" spans="3:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C113" s="5"/>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A114" s="12" t="s">
+        <v>727</v>
+      </c>
+      <c r="D114" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D115" t="s">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D116" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D118" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C119" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" xr:uid="{1078431E-90B5-490C-89E2-631EC2FC986D}"/>
     <hyperlink ref="D7" r:id="rId2" xr:uid="{A82BE56D-8664-44EF-9D97-3B9B32089A10}"/>
-    <hyperlink ref="A9" r:id="rId3" display="Median of Two Sorted Arrays" xr:uid="{E9DDCB05-35C4-411A-9E11-5D6F3CC3AF96}"/>
+    <hyperlink ref="A9" r:id="rId3" xr:uid="{E9DDCB05-35C4-411A-9E11-5D6F3CC3AF96}"/>
     <hyperlink ref="D21" r:id="rId4" xr:uid="{3402BAFA-50FF-4A91-9C05-9F6AEAC01303}"/>
     <hyperlink ref="A30" r:id="rId5" xr:uid="{F636B6F6-9869-4224-B82D-26113E394418}"/>
     <hyperlink ref="D28" r:id="rId6" xr:uid="{F7E2B43E-CE74-4C6C-BC40-1AF4C8945908}"/>
@@ -12914,10 +12996,12 @@
     <hyperlink ref="D103" r:id="rId28" xr:uid="{E752EED3-858C-4BCB-9416-7073E040EB09}"/>
     <hyperlink ref="A105" r:id="rId29" xr:uid="{18C707F3-7727-4F9A-AF34-3F3BFFC6358B}"/>
     <hyperlink ref="D112" r:id="rId30" xr:uid="{1BF05C36-80DD-46E4-8328-4E3524495B39}"/>
+    <hyperlink ref="A114" r:id="rId31" xr:uid="{08434F75-F556-4F20-83A8-DCF558870C39}"/>
+    <hyperlink ref="D118" r:id="rId32" xr:uid="{7D9FD892-78A8-4BAF-BA7C-A5AFE6CCD9A5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId31"/>
-  <drawing r:id="rId32"/>
+  <pageSetup orientation="portrait" r:id="rId33"/>
+  <drawing r:id="rId34"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Thek-thLexicographicalStringofAllHappyStringsofLengthn - July 3rd 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5DCFD94-D8D6-41EF-A610-410965B99575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C51E288A-CCAC-462E-A12B-1C564272E540}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" activeTab="4" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="17" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
   <sheets>
     <sheet name="Parenthesis" sheetId="7" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="954" uniqueCount="731">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="960" uniqueCount="736">
   <si>
     <t>Statement</t>
   </si>
@@ -2328,6 +2328,21 @@
   </si>
   <si>
     <t>thus keep max till end to both sum1 and sum2</t>
+  </si>
+  <si>
+    <t>1415. The k-th Lexicographical String of All Happy Strings of Length n</t>
+  </si>
+  <si>
+    <t>backtrack with prev and get all combinations, return k-1 index from list</t>
+  </si>
+  <si>
+    <t>since each char has 2^n-1 strings that start with</t>
+  </si>
+  <si>
+    <t>build such that if k is &lt;= first 2^n-1 then it's 'a' else b..</t>
+  </si>
+  <si>
+    <t>call recusively with k changing to k - (window - step)</t>
   </si>
 </sst>
 </file>
@@ -5983,6 +5998,50 @@
         <a:xfrm>
           <a:off x="2838451" y="12668250"/>
           <a:ext cx="4876800" cy="790685"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4867275</xdr:colOff>
+      <xdr:row>77</xdr:row>
+      <xdr:rowOff>181085</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30D053FD-9471-B76B-A078-C77C62C3E95B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2895600" y="14058900"/>
+          <a:ext cx="4791075" cy="790685"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -11683,7 +11742,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BDF4E8D-D4E1-4180-9015-2E66B34CBB41}">
-  <dimension ref="A1:D72"/>
+  <dimension ref="A1:D80"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -11874,21 +11933,55 @@
         <v>725</v>
       </c>
     </row>
-    <row r="65" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D65" t="s">
         <v>726</v>
       </c>
     </row>
-    <row r="66" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D66" s="4"/>
     </row>
-    <row r="71" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D71" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="72" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C72" s="5"/>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" s="12" t="s">
+        <v>731</v>
+      </c>
+      <c r="D73" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D74" s="4"/>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D75" t="s">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D76" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D77" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D79" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C80" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -11904,10 +11997,12 @@
     <hyperlink ref="D62" r:id="rId10" xr:uid="{A1E7AB8D-8141-4EC7-B5D4-34BB47C56BF0}"/>
     <hyperlink ref="A64" r:id="rId11" xr:uid="{1DB3F9A6-4972-4DC8-97D9-576F47BAC21F}"/>
     <hyperlink ref="D71" r:id="rId12" xr:uid="{0DA3D38D-1453-4A98-8E78-652910101E3B}"/>
+    <hyperlink ref="A73" r:id="rId13" xr:uid="{A59B1EBC-01F0-4866-9325-B974F1C2302E}"/>
+    <hyperlink ref="D79" r:id="rId14" xr:uid="{7A4200C7-EBB4-47CF-A52A-0EBFF8C5FDBA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId13"/>
-  <drawing r:id="rId14"/>
+  <pageSetup orientation="portrait" r:id="rId15"/>
+  <drawing r:id="rId16"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
java 8  && threads
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C51E288A-CCAC-462E-A12B-1C564272E540}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{544F5392-20C8-4861-B402-450148E5FDB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" firstSheet="1" activeTab="17" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="960" uniqueCount="736">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="965" uniqueCount="740">
   <si>
     <t>Statement</t>
   </si>
@@ -2343,6 +2343,18 @@
   </si>
   <si>
     <t>call recusively with k changing to k - (window - step)</t>
+  </si>
+  <si>
+    <t>443. String Compression</t>
+  </si>
+  <si>
+    <t>iterate from i=0</t>
+  </si>
+  <si>
+    <t>let j=i, till chars[i]==chars[j] i++</t>
+  </si>
+  <si>
+    <t>then process current i and j</t>
   </si>
 </sst>
 </file>
@@ -6042,6 +6054,50 @@
         <a:xfrm>
           <a:off x="2895600" y="14058900"/>
           <a:ext cx="4791075" cy="790685"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4895850</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>181059</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6543A363-D6AF-739D-3F05-E85F0FBB006B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2857500" y="15582900"/>
+          <a:ext cx="4857750" cy="600159"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -11742,7 +11798,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BDF4E8D-D4E1-4180-9015-2E66B34CBB41}">
-  <dimension ref="A1:D80"/>
+  <dimension ref="A1:D86"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -11982,6 +12038,32 @@
     </row>
     <row r="80" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C80" s="5"/>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" s="12" t="s">
+        <v>736</v>
+      </c>
+      <c r="D81" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D82" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D83" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D85" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C86" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -11999,10 +12081,12 @@
     <hyperlink ref="D71" r:id="rId12" xr:uid="{0DA3D38D-1453-4A98-8E78-652910101E3B}"/>
     <hyperlink ref="A73" r:id="rId13" xr:uid="{A59B1EBC-01F0-4866-9325-B974F1C2302E}"/>
     <hyperlink ref="D79" r:id="rId14" xr:uid="{7A4200C7-EBB4-47CF-A52A-0EBFF8C5FDBA}"/>
+    <hyperlink ref="A81" r:id="rId15" xr:uid="{8F1F0977-F68B-4AF3-857F-208D73825471}"/>
+    <hyperlink ref="D85" r:id="rId16" xr:uid="{08419843-609E-43B6-9275-01468D54A3E0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId15"/>
-  <drawing r:id="rId16"/>
+  <pageSetup orientation="portrait" r:id="rId17"/>
+  <drawing r:id="rId18"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
FlattenBinaryTreetoLinkedList - July 28th 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AAE46A5-1D14-4BF9-9AD1-6EFD29CF84C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8603E937-EC26-47D2-9AA4-8145D3180130}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" activeTab="4" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="965" uniqueCount="740">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="974" uniqueCount="748">
   <si>
     <t>Statement</t>
   </si>
@@ -2355,6 +2355,30 @@
   </si>
   <si>
     <t>check if size is full or empty before doing above operations</t>
+  </si>
+  <si>
+    <t>114. Flatten Binary Tree to Linked List</t>
+  </si>
+  <si>
+    <t>iterate and put all nodes in queue using pre-order traversal</t>
+  </si>
+  <si>
+    <t>remove one by one and set prev right to curr &amp; prev left to null</t>
+  </si>
+  <si>
+    <t>before recursively calling the flatten method, store left and right node references and assign left to null</t>
+  </si>
+  <si>
+    <t>after recursion</t>
+  </si>
+  <si>
+    <t>assign right to left</t>
+  </si>
+  <si>
+    <t>iterate till end from root towards right till null</t>
+  </si>
+  <si>
+    <t>assign right to right</t>
   </si>
 </sst>
 </file>
@@ -5604,6 +5628,50 @@
         <a:xfrm>
           <a:off x="2847975" y="27070051"/>
           <a:ext cx="4829175" cy="1847850"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>154</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4667870</xdr:colOff>
+      <xdr:row>167</xdr:row>
+      <xdr:rowOff>171801</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Picture 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5E26CC03-B383-A3EB-56C9-158D8BCD21F9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3048000" y="29470350"/>
+          <a:ext cx="4439270" cy="2514951"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -11372,7 +11440,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36268CC4-0AC5-4653-846F-9B607EC203E4}">
-  <dimension ref="A1:D153"/>
+  <dimension ref="A1:D169"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" customWidth="1"/>
@@ -11721,13 +11789,62 @@
         <v>675</v>
       </c>
     </row>
-    <row r="152" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D152" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="153" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C153" s="5"/>
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A154" s="11" t="s">
+        <v>740</v>
+      </c>
+      <c r="D154" t="s">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D155" t="s">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D156" s="4"/>
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D157" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D158" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D159" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D160" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="161" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D161" t="s">
+        <v>747</v>
+      </c>
+    </row>
+    <row r="168" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D168" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="169" spans="3:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C169" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -11752,9 +11869,11 @@
     <hyperlink ref="D140" r:id="rId19" xr:uid="{EAE54D37-109D-4231-B46E-AE213D8D5674}"/>
     <hyperlink ref="A142" r:id="rId20" xr:uid="{208DBEE3-DC36-4BCC-839D-302642CE3DB9}"/>
     <hyperlink ref="D152" r:id="rId21" xr:uid="{A293AB57-9F78-405F-830B-16419EF6197E}"/>
+    <hyperlink ref="A154" r:id="rId22" xr:uid="{66CBD261-BC7D-48C7-8EA3-19460CE47D7B}"/>
+    <hyperlink ref="D168" r:id="rId23" xr:uid="{3E61EFE4-B9E9-4247-9745-FB08E0B786EB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId22"/>
+  <drawing r:id="rId24"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
ObjectClone - July 31st 2022
</commit_message>
<xml_diff>
--- a/Leetcode_Solutions.xlsx
+++ b/Leetcode_Solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode-solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8603E937-EC26-47D2-9AA4-8145D3180130}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0722D81-9703-48E6-B5E9-9EE556DF1B6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" activeTab="4" xr2:uid="{A7CB0AC4-08E2-47A7-A436-D86FFC77E6E5}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="974" uniqueCount="748">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="975" uniqueCount="750">
   <si>
     <t>Statement</t>
   </si>
@@ -2379,6 +2379,12 @@
   </si>
   <si>
     <t>assign right to right</t>
+  </si>
+  <si>
+    <t>start from 0,isEven = true</t>
+  </si>
+  <si>
+    <t>121. Best Time to Buy and Sell Stock</t>
   </si>
 </sst>
 </file>
@@ -7556,15 +7562,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>600075</xdr:colOff>
-      <xdr:row>278</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:colOff>571500</xdr:colOff>
+      <xdr:row>280</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>4382028</xdr:colOff>
-      <xdr:row>281</xdr:row>
-      <xdr:rowOff>77</xdr:rowOff>
+      <xdr:colOff>4353453</xdr:colOff>
+      <xdr:row>283</xdr:row>
+      <xdr:rowOff>114377</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7587,7 +7593,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3638550" y="52978050"/>
+          <a:off x="3609975" y="53473350"/>
           <a:ext cx="3781953" cy="552527"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7600,15 +7606,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>914400</xdr:colOff>
-      <xdr:row>286</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:colOff>828675</xdr:colOff>
+      <xdr:row>285</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>3877088</xdr:colOff>
-      <xdr:row>297</xdr:row>
-      <xdr:rowOff>114603</xdr:rowOff>
+      <xdr:colOff>3791363</xdr:colOff>
+      <xdr:row>296</xdr:row>
+      <xdr:rowOff>152703</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7631,7 +7637,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3952875" y="54521100"/>
+          <a:off x="3867150" y="54368700"/>
           <a:ext cx="2962688" cy="2172003"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -13225,7 +13231,7 @@
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D172" t="s">
-        <v>379</v>
+        <v>748</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
@@ -13640,6 +13646,9 @@
       </c>
     </row>
     <row r="300" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A300" s="13" t="s">
+        <v>749</v>
+      </c>
       <c r="D300" t="s">
         <v>583</v>
       </c>
@@ -13716,10 +13725,11 @@
     <hyperlink ref="A299" r:id="rId60" xr:uid="{1FCAE6AE-0B3F-47E1-9767-971F723B2E83}"/>
     <hyperlink ref="D304" r:id="rId61" xr:uid="{4E6A4A67-63BB-4DA4-ACE0-DE299D79DF74}"/>
     <hyperlink ref="D7" r:id="rId62" xr:uid="{440ECE85-1159-4668-8AED-B2DAB74583B5}"/>
+    <hyperlink ref="A300" r:id="rId63" xr:uid="{5344B68E-1DF0-41D2-A3C9-4EC7FDF98CF6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId63"/>
-  <drawing r:id="rId64"/>
+  <pageSetup orientation="portrait" r:id="rId64"/>
+  <drawing r:id="rId65"/>
 </worksheet>
 </file>
 

</xml_diff>